<commit_message>
Actualización automática ERP - Pedidos Transmicion - 10/08/2026 19:06:47
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Sistema_Logistico_Peirano\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{851FEC6E-DDF9-4BD8-8A79-6D1A8DC6B5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14300C14-2A70-45F4-9399-A5B218D879C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{854DF19A-0C24-49C2-95F1-3828B168A7C8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F35A25CB-1CCD-4BDC-8526-8C916F45A488}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -4256,7 +4256,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2915D8BF-EE4A-485E-9370-060D7A960B73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{288ACFD6-C0B7-4E80-B429-B6C0F4CA9C3D}">
   <dimension ref="A1:H453"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 11/08/2026 14:28:52
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D02FDEB0-1335-4FED-AD23-E06A801D3F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3A058EB-AA6E-4184-822C-4D5A4A0A0049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E7BDC0C5-A6F9-4DEC-ABBD-E83A56431198}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A13A846E-569D-4C42-B442-80B4CE7712B4}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -4169,7 +4169,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3335470-EC2C-4671-A2FF-CB64DA8FE0D2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3789995-99B4-4516-AD4E-7C386CEEC013}">
   <dimension ref="A1:H441"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 12/08/2026 08:17:25
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1F559A7-F50D-4D24-9481-368263BBE645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1ED107C3-D8DA-41F8-9FE5-EA715B590F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{CBD33827-AADC-4FB9-914F-F1204A984410}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{2322D428-2DDC-494B-867A-A2B9B2D2D7F9}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -4388,7 +4388,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF3F844A-5B17-4C25-BFAD-7A3855511305}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD668B2E-7616-4EBD-9EA7-A62A586B40D1}">
   <dimension ref="A1:H469"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 21/08/2026 06:04:48
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4807645-4B7E-4130-A269-E87177540A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2A20913-C271-47CC-A699-8D2BECE761B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26505" yWindow="3765" windowWidth="15375" windowHeight="8325" xr2:uid="{40F9090B-8D9B-41B8-A15B-2B4B52674418}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3F966780-C724-4E90-A737-9EE2B961DE5B}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="554">
   <si>
     <t>0001</t>
   </si>
@@ -919,6 +919,9 @@
     <t xml:space="preserve">  213911</t>
   </si>
   <si>
+    <t xml:space="preserve">  213912</t>
+  </si>
+  <si>
     <t xml:space="preserve">  213914</t>
   </si>
   <si>
@@ -952,6 +955,9 @@
     <t xml:space="preserve">  213938</t>
   </si>
   <si>
+    <t xml:space="preserve">  213944</t>
+  </si>
+  <si>
     <t xml:space="preserve">  213946</t>
   </si>
   <si>
@@ -1321,12 +1327,129 @@
     <t>PIAZZA JOSE ALBERTO</t>
   </si>
   <si>
+    <t xml:space="preserve">  214087</t>
+  </si>
+  <si>
+    <t>SURVALMEDA CONSTRUCCIONES S. A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214089</t>
+  </si>
+  <si>
+    <t>PRIATEL PISOS S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214091</t>
+  </si>
+  <si>
+    <t>BELINDA S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214093</t>
+  </si>
+  <si>
+    <t>NICUESA E HIJOS S.R.L. -SANIT. NICUESA E HIJOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214095</t>
+  </si>
+  <si>
+    <t>BOLONDI JORGE A.-CORRALON MAILIN MADERAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214097</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214098</t>
+  </si>
+  <si>
+    <t>FICO HORACIO JAVIER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214099</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214101</t>
   </si>
   <si>
     <t>TRIPOLI CARLOS L.</t>
   </si>
   <si>
+    <t xml:space="preserve">  214105</t>
+  </si>
+  <si>
+    <t>GILLI FAUDIN LUIS V. -GILCOMAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214108</t>
+  </si>
+  <si>
+    <t>EDEN SANITARIOS S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214109</t>
+  </si>
+  <si>
+    <t>FANTINI FERNANDO ARIEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214113</t>
+  </si>
+  <si>
+    <t>RA S.H. DE ALFONSO RUBEN Y POZZUTO CARLOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214115</t>
+  </si>
+  <si>
+    <t>UCCELI GABRIEL A.-SANITARIOS GABRIEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214116</t>
+  </si>
+  <si>
+    <t>SCHEYER CARINA E,KOLB ESTEBAN H S.H.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214117</t>
+  </si>
+  <si>
+    <t>WELSH L Y HAUF E. -SANITARIOS DE LA COSTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214119</t>
+  </si>
+  <si>
+    <t>TUBOPLAST SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214121</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -1429,6 +1552,9 @@
     <t xml:space="preserve">    2826</t>
   </si>
   <si>
+    <t xml:space="preserve">    2829</t>
+  </si>
+  <si>
     <t>4444</t>
   </si>
   <si>
@@ -1498,7 +1624,7 @@
     <t xml:space="preserve">    2240</t>
   </si>
   <si>
-    <t xml:space="preserve">    2244</t>
+    <t xml:space="preserve">    2247</t>
   </si>
   <si>
     <t>9999</t>
@@ -2005,34 +2131,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{767F6232-E645-4A39-BF9A-057190255A70}">
-  <dimension ref="A1:H337"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E418CEC2-71E4-477F-B2C9-1ADD17A8D4DA}">
+  <dimension ref="A1:H365"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>504</v>
+        <v>546</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>505</v>
+        <v>547</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>506</v>
+        <v>548</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>507</v>
+        <v>549</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>508</v>
+        <v>550</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>509</v>
+        <v>551</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>510</v>
+        <v>552</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>511</v>
+        <v>553</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -6781,13 +6907,13 @@
         <v>56</v>
       </c>
       <c r="E184" t="s">
-        <v>72</v>
+        <v>297</v>
       </c>
       <c r="F184" s="1">
         <v>46252</v>
       </c>
       <c r="G184" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H184">
         <v>0</v>
@@ -6807,7 +6933,7 @@
         <v>56</v>
       </c>
       <c r="E185" t="s">
-        <v>249</v>
+        <v>72</v>
       </c>
       <c r="F185" s="1">
         <v>46252</v>
@@ -6833,7 +6959,7 @@
         <v>56</v>
       </c>
       <c r="E186" t="s">
-        <v>66</v>
+        <v>249</v>
       </c>
       <c r="F186" s="1">
         <v>46252</v>
@@ -6859,7 +6985,7 @@
         <v>56</v>
       </c>
       <c r="E187" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="F187" s="1">
         <v>46252</v>
@@ -6885,7 +7011,7 @@
         <v>56</v>
       </c>
       <c r="E188" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="F188" s="1">
         <v>46252</v>
@@ -6911,7 +7037,7 @@
         <v>56</v>
       </c>
       <c r="E189" t="s">
-        <v>305</v>
+        <v>70</v>
       </c>
       <c r="F189" s="1">
         <v>46252</v>
@@ -6928,22 +7054,22 @@
         <v>0</v>
       </c>
       <c r="B190" t="s">
+        <v>305</v>
+      </c>
+      <c r="C190">
+        <v>1</v>
+      </c>
+      <c r="D190" t="s">
+        <v>56</v>
+      </c>
+      <c r="E190" t="s">
         <v>306</v>
-      </c>
-      <c r="C190">
-        <v>1</v>
-      </c>
-      <c r="D190" t="s">
-        <v>56</v>
-      </c>
-      <c r="E190" t="s">
-        <v>83</v>
       </c>
       <c r="F190" s="1">
         <v>46252</v>
       </c>
       <c r="G190" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="H190">
         <v>0</v>
@@ -6963,7 +7089,7 @@
         <v>56</v>
       </c>
       <c r="E191" t="s">
-        <v>259</v>
+        <v>83</v>
       </c>
       <c r="F191" s="1">
         <v>46252</v>
@@ -6989,13 +7115,13 @@
         <v>56</v>
       </c>
       <c r="E192" t="s">
-        <v>159</v>
+        <v>259</v>
       </c>
       <c r="F192" s="1">
         <v>46252</v>
       </c>
       <c r="G192" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H192">
         <v>0</v>
@@ -7012,19 +7138,19 @@
         <v>1</v>
       </c>
       <c r="D193" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E193" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="F193" s="1">
         <v>46252</v>
       </c>
       <c r="G193" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H193">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.2">
@@ -7038,19 +7164,19 @@
         <v>1</v>
       </c>
       <c r="D194" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E194" t="s">
-        <v>311</v>
+        <v>172</v>
       </c>
       <c r="F194" s="1">
         <v>46252</v>
       </c>
       <c r="G194" s="1">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="H194">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.2">
@@ -7058,7 +7184,7 @@
         <v>0</v>
       </c>
       <c r="B195" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C195">
         <v>1</v>
@@ -7067,13 +7193,13 @@
         <v>56</v>
       </c>
       <c r="E195" t="s">
-        <v>132</v>
+        <v>174</v>
       </c>
       <c r="F195" s="1">
         <v>46252</v>
       </c>
       <c r="G195" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H195">
         <v>0</v>
@@ -7084,16 +7210,16 @@
         <v>0</v>
       </c>
       <c r="B196" t="s">
+        <v>312</v>
+      </c>
+      <c r="C196">
+        <v>1</v>
+      </c>
+      <c r="D196" t="s">
+        <v>56</v>
+      </c>
+      <c r="E196" t="s">
         <v>313</v>
-      </c>
-      <c r="C196">
-        <v>1</v>
-      </c>
-      <c r="D196" t="s">
-        <v>56</v>
-      </c>
-      <c r="E196" t="s">
-        <v>132</v>
       </c>
       <c r="F196" s="1">
         <v>46252</v>
@@ -7119,13 +7245,13 @@
         <v>56</v>
       </c>
       <c r="E197" t="s">
-        <v>315</v>
+        <v>132</v>
       </c>
       <c r="F197" s="1">
         <v>46252</v>
       </c>
       <c r="G197" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="H197">
         <v>0</v>
@@ -7136,25 +7262,25 @@
         <v>0</v>
       </c>
       <c r="B198" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C198">
         <v>1</v>
       </c>
       <c r="D198" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E198" t="s">
-        <v>317</v>
+        <v>132</v>
       </c>
       <c r="F198" s="1">
         <v>46252</v>
       </c>
       <c r="G198" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="H198">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.2">
@@ -7162,16 +7288,16 @@
         <v>0</v>
       </c>
       <c r="B199" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C199">
         <v>1</v>
       </c>
       <c r="D199" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E199" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F199" s="1">
         <v>46252</v>
@@ -7180,7 +7306,7 @@
         <v>46253</v>
       </c>
       <c r="H199">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.2">
@@ -7188,7 +7314,7 @@
         <v>0</v>
       </c>
       <c r="B200" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C200">
         <v>1</v>
@@ -7197,16 +7323,16 @@
         <v>2</v>
       </c>
       <c r="E200" t="s">
-        <v>236</v>
+        <v>319</v>
       </c>
       <c r="F200" s="1">
         <v>46252</v>
       </c>
       <c r="G200" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H200">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.2">
@@ -7214,16 +7340,16 @@
         <v>0</v>
       </c>
       <c r="B201" t="s">
+        <v>320</v>
+      </c>
+      <c r="C201">
+        <v>1</v>
+      </c>
+      <c r="D201" t="s">
+        <v>2</v>
+      </c>
+      <c r="E201" t="s">
         <v>321</v>
-      </c>
-      <c r="C201">
-        <v>1</v>
-      </c>
-      <c r="D201" t="s">
-        <v>56</v>
-      </c>
-      <c r="E201" t="s">
-        <v>322</v>
       </c>
       <c r="F201" s="1">
         <v>46252</v>
@@ -7232,7 +7358,7 @@
         <v>46253</v>
       </c>
       <c r="H201">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.2">
@@ -7240,25 +7366,25 @@
         <v>0</v>
       </c>
       <c r="B202" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C202">
         <v>1</v>
       </c>
       <c r="D202" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E202" t="s">
-        <v>324</v>
+        <v>236</v>
       </c>
       <c r="F202" s="1">
         <v>46252</v>
       </c>
       <c r="G202" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H202">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.2">
@@ -7266,7 +7392,7 @@
         <v>0</v>
       </c>
       <c r="B203" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C203">
         <v>1</v>
@@ -7292,22 +7418,22 @@
         <v>0</v>
       </c>
       <c r="B204" t="s">
+        <v>325</v>
+      </c>
+      <c r="C204">
+        <v>1</v>
+      </c>
+      <c r="D204" t="s">
+        <v>56</v>
+      </c>
+      <c r="E204" t="s">
         <v>326</v>
-      </c>
-      <c r="C204">
-        <v>1</v>
-      </c>
-      <c r="D204" t="s">
-        <v>56</v>
-      </c>
-      <c r="E204" t="s">
-        <v>204</v>
       </c>
       <c r="F204" s="1">
         <v>46252</v>
       </c>
       <c r="G204" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H204">
         <v>0</v>
@@ -7324,10 +7450,10 @@
         <v>1</v>
       </c>
       <c r="D205" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E205" t="s">
-        <v>204</v>
+        <v>326</v>
       </c>
       <c r="F205" s="1">
         <v>46252</v>
@@ -7336,7 +7462,7 @@
         <v>46253</v>
       </c>
       <c r="H205">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.2">
@@ -7353,7 +7479,7 @@
         <v>56</v>
       </c>
       <c r="E206" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="F206" s="1">
         <v>46252</v>
@@ -7379,13 +7505,13 @@
         <v>56</v>
       </c>
       <c r="E207" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="F207" s="1">
         <v>46252</v>
       </c>
       <c r="G207" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H207">
         <v>0</v>
@@ -7405,13 +7531,13 @@
         <v>56</v>
       </c>
       <c r="E208" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="F208" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G208" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H208">
         <v>0</v>
@@ -7431,13 +7557,13 @@
         <v>56</v>
       </c>
       <c r="E209" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="F209" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G209" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H209">
         <v>0</v>
@@ -7457,7 +7583,7 @@
         <v>56</v>
       </c>
       <c r="E210" t="s">
-        <v>333</v>
+        <v>163</v>
       </c>
       <c r="F210" s="1">
         <v>46253</v>
@@ -7474,25 +7600,25 @@
         <v>0</v>
       </c>
       <c r="B211" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C211">
         <v>1</v>
       </c>
       <c r="D211" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E211" t="s">
-        <v>335</v>
+        <v>163</v>
       </c>
       <c r="F211" s="1">
         <v>46253</v>
       </c>
       <c r="G211" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H211">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.2">
@@ -7500,7 +7626,7 @@
         <v>0</v>
       </c>
       <c r="B212" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C212">
         <v>1</v>
@@ -7509,7 +7635,7 @@
         <v>56</v>
       </c>
       <c r="E212" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F212" s="1">
         <v>46253</v>
@@ -7526,22 +7652,22 @@
         <v>0</v>
       </c>
       <c r="B213" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C213">
         <v>1</v>
       </c>
       <c r="D213" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E213" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F213" s="1">
         <v>46253</v>
       </c>
       <c r="G213" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H213">
         <v>0</v>
@@ -7552,16 +7678,16 @@
         <v>0</v>
       </c>
       <c r="B214" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C214">
         <v>1</v>
       </c>
       <c r="D214" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E214" t="s">
-        <v>26</v>
+        <v>339</v>
       </c>
       <c r="F214" s="1">
         <v>46253</v>
@@ -7570,7 +7696,7 @@
         <v>46253</v>
       </c>
       <c r="H214">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.2">
@@ -7578,16 +7704,16 @@
         <v>0</v>
       </c>
       <c r="B215" t="s">
+        <v>340</v>
+      </c>
+      <c r="C215">
+        <v>1</v>
+      </c>
+      <c r="D215" t="s">
+        <v>5</v>
+      </c>
+      <c r="E215" t="s">
         <v>341</v>
-      </c>
-      <c r="C215">
-        <v>1</v>
-      </c>
-      <c r="D215" t="s">
-        <v>2</v>
-      </c>
-      <c r="E215" t="s">
-        <v>26</v>
       </c>
       <c r="F215" s="1">
         <v>46253</v>
@@ -7596,7 +7722,7 @@
         <v>46253</v>
       </c>
       <c r="H215">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.2">
@@ -7610,7 +7736,7 @@
         <v>1</v>
       </c>
       <c r="D216" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E216" t="s">
         <v>26</v>
@@ -7622,7 +7748,7 @@
         <v>46253</v>
       </c>
       <c r="H216">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.2">
@@ -7639,7 +7765,7 @@
         <v>2</v>
       </c>
       <c r="E217" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
       <c r="F217" s="1">
         <v>46253</v>
@@ -7648,7 +7774,7 @@
         <v>46253</v>
       </c>
       <c r="H217">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.2">
@@ -7665,7 +7791,7 @@
         <v>2</v>
       </c>
       <c r="E218" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
       <c r="F218" s="1">
         <v>46253</v>
@@ -7691,7 +7817,7 @@
         <v>2</v>
       </c>
       <c r="E219" t="s">
-        <v>346</v>
+        <v>122</v>
       </c>
       <c r="F219" s="1">
         <v>46253</v>
@@ -7700,7 +7826,7 @@
         <v>46253</v>
       </c>
       <c r="H219">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.2">
@@ -7708,16 +7834,16 @@
         <v>0</v>
       </c>
       <c r="B220" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C220">
         <v>1</v>
       </c>
       <c r="D220" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E220" t="s">
-        <v>66</v>
+        <v>122</v>
       </c>
       <c r="F220" s="1">
         <v>46253</v>
@@ -7726,7 +7852,7 @@
         <v>46253</v>
       </c>
       <c r="H220">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.2">
@@ -7734,16 +7860,16 @@
         <v>0</v>
       </c>
       <c r="B221" t="s">
+        <v>347</v>
+      </c>
+      <c r="C221">
+        <v>1</v>
+      </c>
+      <c r="D221" t="s">
+        <v>2</v>
+      </c>
+      <c r="E221" t="s">
         <v>348</v>
-      </c>
-      <c r="C221">
-        <v>1</v>
-      </c>
-      <c r="D221" t="s">
-        <v>56</v>
-      </c>
-      <c r="E221" t="s">
-        <v>144</v>
       </c>
       <c r="F221" s="1">
         <v>46253</v>
@@ -7752,7 +7878,7 @@
         <v>46253</v>
       </c>
       <c r="H221">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.2">
@@ -7769,7 +7895,7 @@
         <v>56</v>
       </c>
       <c r="E222" t="s">
-        <v>350</v>
+        <v>66</v>
       </c>
       <c r="F222" s="1">
         <v>46253</v>
@@ -7786,7 +7912,7 @@
         <v>0</v>
       </c>
       <c r="B223" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C223">
         <v>1</v>
@@ -7795,7 +7921,7 @@
         <v>56</v>
       </c>
       <c r="E223" t="s">
-        <v>352</v>
+        <v>144</v>
       </c>
       <c r="F223" s="1">
         <v>46253</v>
@@ -7812,16 +7938,16 @@
         <v>0</v>
       </c>
       <c r="B224" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C224">
         <v>1</v>
       </c>
       <c r="D224" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E224" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F224" s="1">
         <v>46253</v>
@@ -7830,7 +7956,7 @@
         <v>46253</v>
       </c>
       <c r="H224">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.2">
@@ -7838,7 +7964,7 @@
         <v>0</v>
       </c>
       <c r="B225" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C225">
         <v>1</v>
@@ -7847,7 +7973,7 @@
         <v>56</v>
       </c>
       <c r="E225" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="F225" s="1">
         <v>46253</v>
@@ -7864,16 +7990,16 @@
         <v>0</v>
       </c>
       <c r="B226" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C226">
         <v>1</v>
       </c>
       <c r="D226" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E226" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="F226" s="1">
         <v>46253</v>
@@ -7882,7 +8008,7 @@
         <v>46253</v>
       </c>
       <c r="H226">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.2">
@@ -7890,7 +8016,7 @@
         <v>0</v>
       </c>
       <c r="B227" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C227">
         <v>1</v>
@@ -7899,7 +8025,7 @@
         <v>56</v>
       </c>
       <c r="E227" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="F227" s="1">
         <v>46253</v>
@@ -7916,7 +8042,7 @@
         <v>0</v>
       </c>
       <c r="B228" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C228">
         <v>1</v>
@@ -7925,7 +8051,7 @@
         <v>56</v>
       </c>
       <c r="E228" t="s">
-        <v>311</v>
+        <v>360</v>
       </c>
       <c r="F228" s="1">
         <v>46253</v>
@@ -7942,16 +8068,16 @@
         <v>0</v>
       </c>
       <c r="B229" t="s">
+        <v>361</v>
+      </c>
+      <c r="C229">
+        <v>1</v>
+      </c>
+      <c r="D229" t="s">
+        <v>56</v>
+      </c>
+      <c r="E229" t="s">
         <v>362</v>
-      </c>
-      <c r="C229">
-        <v>1</v>
-      </c>
-      <c r="D229" t="s">
-        <v>56</v>
-      </c>
-      <c r="E229" t="s">
-        <v>363</v>
       </c>
       <c r="F229" s="1">
         <v>46253</v>
@@ -7968,7 +8094,7 @@
         <v>0</v>
       </c>
       <c r="B230" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C230">
         <v>1</v>
@@ -7977,7 +8103,7 @@
         <v>56</v>
       </c>
       <c r="E230" t="s">
-        <v>365</v>
+        <v>313</v>
       </c>
       <c r="F230" s="1">
         <v>46253</v>
@@ -7994,7 +8120,7 @@
         <v>0</v>
       </c>
       <c r="B231" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C231">
         <v>1</v>
@@ -8003,13 +8129,13 @@
         <v>56</v>
       </c>
       <c r="E231" t="s">
-        <v>16</v>
+        <v>365</v>
       </c>
       <c r="F231" s="1">
         <v>46253</v>
       </c>
       <c r="G231" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H231">
         <v>0</v>
@@ -8020,16 +8146,16 @@
         <v>0</v>
       </c>
       <c r="B232" t="s">
+        <v>366</v>
+      </c>
+      <c r="C232">
+        <v>1</v>
+      </c>
+      <c r="D232" t="s">
+        <v>56</v>
+      </c>
+      <c r="E232" t="s">
         <v>367</v>
-      </c>
-      <c r="C232">
-        <v>1</v>
-      </c>
-      <c r="D232" t="s">
-        <v>56</v>
-      </c>
-      <c r="E232" t="s">
-        <v>368</v>
       </c>
       <c r="F232" s="1">
         <v>46253</v>
@@ -8046,7 +8172,7 @@
         <v>0</v>
       </c>
       <c r="B233" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C233">
         <v>1</v>
@@ -8055,13 +8181,13 @@
         <v>56</v>
       </c>
       <c r="E233" t="s">
-        <v>370</v>
+        <v>16</v>
       </c>
       <c r="F233" s="1">
         <v>46253</v>
       </c>
       <c r="G233" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H233">
         <v>0</v>
@@ -8072,7 +8198,7 @@
         <v>0</v>
       </c>
       <c r="B234" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C234">
         <v>1</v>
@@ -8081,7 +8207,7 @@
         <v>56</v>
       </c>
       <c r="E234" t="s">
-        <v>139</v>
+        <v>370</v>
       </c>
       <c r="F234" s="1">
         <v>46253</v>
@@ -8098,16 +8224,16 @@
         <v>0</v>
       </c>
       <c r="B235" t="s">
+        <v>371</v>
+      </c>
+      <c r="C235">
+        <v>1</v>
+      </c>
+      <c r="D235" t="s">
+        <v>56</v>
+      </c>
+      <c r="E235" t="s">
         <v>372</v>
-      </c>
-      <c r="C235">
-        <v>1</v>
-      </c>
-      <c r="D235" t="s">
-        <v>56</v>
-      </c>
-      <c r="E235" t="s">
-        <v>311</v>
       </c>
       <c r="F235" s="1">
         <v>46253</v>
@@ -8133,7 +8259,7 @@
         <v>56</v>
       </c>
       <c r="E236" t="s">
-        <v>26</v>
+        <v>139</v>
       </c>
       <c r="F236" s="1">
         <v>46253</v>
@@ -8159,7 +8285,7 @@
         <v>56</v>
       </c>
       <c r="E237" t="s">
-        <v>26</v>
+        <v>313</v>
       </c>
       <c r="F237" s="1">
         <v>46253</v>
@@ -8338,10 +8464,10 @@
         <v>1</v>
       </c>
       <c r="D244" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E244" t="s">
-        <v>382</v>
+        <v>26</v>
       </c>
       <c r="F244" s="1">
         <v>46253</v>
@@ -8350,7 +8476,7 @@
         <v>46253</v>
       </c>
       <c r="H244">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245" spans="1:8" x14ac:dyDescent="0.2">
@@ -8358,7 +8484,7 @@
         <v>0</v>
       </c>
       <c r="B245" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C245">
         <v>1</v>
@@ -8367,7 +8493,7 @@
         <v>56</v>
       </c>
       <c r="E245" t="s">
-        <v>384</v>
+        <v>26</v>
       </c>
       <c r="F245" s="1">
         <v>46253</v>
@@ -8384,16 +8510,16 @@
         <v>0</v>
       </c>
       <c r="B246" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C246">
         <v>1</v>
       </c>
       <c r="D246" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E246" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F246" s="1">
         <v>46253</v>
@@ -8402,7 +8528,7 @@
         <v>46253</v>
       </c>
       <c r="H246">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="247" spans="1:8" x14ac:dyDescent="0.2">
@@ -8410,16 +8536,16 @@
         <v>0</v>
       </c>
       <c r="B247" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C247">
         <v>1</v>
       </c>
       <c r="D247" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E247" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F247" s="1">
         <v>46253</v>
@@ -8428,7 +8554,7 @@
         <v>46253</v>
       </c>
       <c r="H247">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.2">
@@ -8436,16 +8562,16 @@
         <v>0</v>
       </c>
       <c r="B248" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C248">
         <v>1</v>
       </c>
       <c r="D248" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E248" t="s">
-        <v>335</v>
+        <v>388</v>
       </c>
       <c r="F248" s="1">
         <v>46253</v>
@@ -8454,7 +8580,7 @@
         <v>46253</v>
       </c>
       <c r="H248">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:8" x14ac:dyDescent="0.2">
@@ -8462,25 +8588,25 @@
         <v>0</v>
       </c>
       <c r="B249" t="s">
+        <v>389</v>
+      </c>
+      <c r="C249">
+        <v>1</v>
+      </c>
+      <c r="D249" t="s">
+        <v>2</v>
+      </c>
+      <c r="E249" t="s">
         <v>390</v>
-      </c>
-      <c r="C249">
-        <v>1</v>
-      </c>
-      <c r="D249" t="s">
-        <v>56</v>
-      </c>
-      <c r="E249" t="s">
-        <v>391</v>
       </c>
       <c r="F249" s="1">
         <v>46253</v>
       </c>
       <c r="G249" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H249">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="250" spans="1:8" x14ac:dyDescent="0.2">
@@ -8488,25 +8614,25 @@
         <v>0</v>
       </c>
       <c r="B250" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C250">
         <v>1</v>
       </c>
       <c r="D250" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E250" t="s">
-        <v>20</v>
+        <v>337</v>
       </c>
       <c r="F250" s="1">
         <v>46253</v>
       </c>
       <c r="G250" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H250">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="251" spans="1:8" x14ac:dyDescent="0.2">
@@ -8514,16 +8640,16 @@
         <v>0</v>
       </c>
       <c r="B251" t="s">
+        <v>392</v>
+      </c>
+      <c r="C251">
+        <v>1</v>
+      </c>
+      <c r="D251" t="s">
+        <v>56</v>
+      </c>
+      <c r="E251" t="s">
         <v>393</v>
-      </c>
-      <c r="C251">
-        <v>1</v>
-      </c>
-      <c r="D251" t="s">
-        <v>56</v>
-      </c>
-      <c r="E251" t="s">
-        <v>394</v>
       </c>
       <c r="F251" s="1">
         <v>46253</v>
@@ -8540,7 +8666,7 @@
         <v>0</v>
       </c>
       <c r="B252" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C252">
         <v>1</v>
@@ -8549,7 +8675,7 @@
         <v>56</v>
       </c>
       <c r="E252" t="s">
-        <v>394</v>
+        <v>20</v>
       </c>
       <c r="F252" s="1">
         <v>46253</v>
@@ -8566,16 +8692,16 @@
         <v>0</v>
       </c>
       <c r="B253" t="s">
+        <v>395</v>
+      </c>
+      <c r="C253">
+        <v>1</v>
+      </c>
+      <c r="D253" t="s">
+        <v>56</v>
+      </c>
+      <c r="E253" t="s">
         <v>396</v>
-      </c>
-      <c r="C253">
-        <v>1</v>
-      </c>
-      <c r="D253" t="s">
-        <v>56</v>
-      </c>
-      <c r="E253" t="s">
-        <v>397</v>
       </c>
       <c r="F253" s="1">
         <v>46253</v>
@@ -8592,7 +8718,7 @@
         <v>0</v>
       </c>
       <c r="B254" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C254">
         <v>1</v>
@@ -8601,7 +8727,7 @@
         <v>56</v>
       </c>
       <c r="E254" t="s">
-        <v>52</v>
+        <v>396</v>
       </c>
       <c r="F254" s="1">
         <v>46253</v>
@@ -8618,16 +8744,16 @@
         <v>0</v>
       </c>
       <c r="B255" t="s">
+        <v>398</v>
+      </c>
+      <c r="C255">
+        <v>1</v>
+      </c>
+      <c r="D255" t="s">
+        <v>56</v>
+      </c>
+      <c r="E255" t="s">
         <v>399</v>
-      </c>
-      <c r="C255">
-        <v>1</v>
-      </c>
-      <c r="D255" t="s">
-        <v>56</v>
-      </c>
-      <c r="E255" t="s">
-        <v>52</v>
       </c>
       <c r="F255" s="1">
         <v>46253</v>
@@ -8679,7 +8805,7 @@
         <v>56</v>
       </c>
       <c r="E257" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="F257" s="1">
         <v>46253</v>
@@ -8705,7 +8831,7 @@
         <v>56</v>
       </c>
       <c r="E258" t="s">
-        <v>403</v>
+        <v>52</v>
       </c>
       <c r="F258" s="1">
         <v>46253</v>
@@ -8722,16 +8848,16 @@
         <v>0</v>
       </c>
       <c r="B259" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C259">
         <v>1</v>
       </c>
       <c r="D259" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E259" t="s">
-        <v>405</v>
+        <v>18</v>
       </c>
       <c r="F259" s="1">
         <v>46253</v>
@@ -8748,7 +8874,7 @@
         <v>0</v>
       </c>
       <c r="B260" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C260">
         <v>1</v>
@@ -8757,7 +8883,7 @@
         <v>56</v>
       </c>
       <c r="E260" t="s">
-        <v>281</v>
+        <v>405</v>
       </c>
       <c r="F260" s="1">
         <v>46253</v>
@@ -8774,19 +8900,19 @@
         <v>0</v>
       </c>
       <c r="B261" t="s">
+        <v>406</v>
+      </c>
+      <c r="C261">
+        <v>2</v>
+      </c>
+      <c r="D261" t="s">
+        <v>56</v>
+      </c>
+      <c r="E261" t="s">
         <v>407</v>
       </c>
-      <c r="C261">
-        <v>1</v>
-      </c>
-      <c r="D261" t="s">
-        <v>56</v>
-      </c>
-      <c r="E261" t="s">
-        <v>132</v>
-      </c>
       <c r="F261" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G261" s="1">
         <v>46254</v>
@@ -8809,10 +8935,10 @@
         <v>56</v>
       </c>
       <c r="E262" t="s">
-        <v>70</v>
+        <v>281</v>
       </c>
       <c r="F262" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G262" s="1">
         <v>46254</v>
@@ -8835,7 +8961,7 @@
         <v>56</v>
       </c>
       <c r="E263" t="s">
-        <v>410</v>
+        <v>132</v>
       </c>
       <c r="F263" s="1">
         <v>46254</v>
@@ -8852,16 +8978,16 @@
         <v>0</v>
       </c>
       <c r="B264" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C264">
         <v>1</v>
       </c>
       <c r="D264" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E264" t="s">
-        <v>412</v>
+        <v>70</v>
       </c>
       <c r="F264" s="1">
         <v>46254</v>
@@ -8870,7 +8996,7 @@
         <v>46254</v>
       </c>
       <c r="H264">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265" spans="1:8" x14ac:dyDescent="0.2">
@@ -8878,7 +9004,7 @@
         <v>0</v>
       </c>
       <c r="B265" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C265">
         <v>1</v>
@@ -8887,7 +9013,7 @@
         <v>56</v>
       </c>
       <c r="E265" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="F265" s="1">
         <v>46254</v>
@@ -8904,16 +9030,16 @@
         <v>0</v>
       </c>
       <c r="B266" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C266">
         <v>1</v>
       </c>
       <c r="D266" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E266" t="s">
-        <v>122</v>
+        <v>414</v>
       </c>
       <c r="F266" s="1">
         <v>46254</v>
@@ -8922,7 +9048,7 @@
         <v>46254</v>
       </c>
       <c r="H266">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="267" spans="1:8" x14ac:dyDescent="0.2">
@@ -8930,16 +9056,16 @@
         <v>0</v>
       </c>
       <c r="B267" t="s">
+        <v>415</v>
+      </c>
+      <c r="C267">
+        <v>1</v>
+      </c>
+      <c r="D267" t="s">
+        <v>56</v>
+      </c>
+      <c r="E267" t="s">
         <v>416</v>
-      </c>
-      <c r="C267">
-        <v>1</v>
-      </c>
-      <c r="D267" t="s">
-        <v>56</v>
-      </c>
-      <c r="E267" t="s">
-        <v>26</v>
       </c>
       <c r="F267" s="1">
         <v>46254</v>
@@ -8965,7 +9091,7 @@
         <v>56</v>
       </c>
       <c r="E268" t="s">
-        <v>26</v>
+        <v>122</v>
       </c>
       <c r="F268" s="1">
         <v>46254</v>
@@ -9017,7 +9143,7 @@
         <v>56</v>
       </c>
       <c r="E270" t="s">
-        <v>420</v>
+        <v>26</v>
       </c>
       <c r="F270" s="1">
         <v>46254</v>
@@ -9034,7 +9160,7 @@
         <v>0</v>
       </c>
       <c r="B271" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C271">
         <v>1</v>
@@ -9043,7 +9169,7 @@
         <v>56</v>
       </c>
       <c r="E271" t="s">
-        <v>420</v>
+        <v>26</v>
       </c>
       <c r="F271" s="1">
         <v>46254</v>
@@ -9060,16 +9186,16 @@
         <v>0</v>
       </c>
       <c r="B272" t="s">
+        <v>421</v>
+      </c>
+      <c r="C272">
+        <v>1</v>
+      </c>
+      <c r="D272" t="s">
+        <v>56</v>
+      </c>
+      <c r="E272" t="s">
         <v>422</v>
-      </c>
-      <c r="C272">
-        <v>1</v>
-      </c>
-      <c r="D272" t="s">
-        <v>56</v>
-      </c>
-      <c r="E272" t="s">
-        <v>14</v>
       </c>
       <c r="F272" s="1">
         <v>46254</v>
@@ -9095,7 +9221,7 @@
         <v>56</v>
       </c>
       <c r="E273" t="s">
-        <v>34</v>
+        <v>422</v>
       </c>
       <c r="F273" s="1">
         <v>46254</v>
@@ -9121,7 +9247,7 @@
         <v>56</v>
       </c>
       <c r="E274" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F274" s="1">
         <v>46254</v>
@@ -9147,7 +9273,7 @@
         <v>56</v>
       </c>
       <c r="E275" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F275" s="1">
         <v>46254</v>
@@ -9173,7 +9299,7 @@
         <v>56</v>
       </c>
       <c r="E276" t="s">
-        <v>427</v>
+        <v>12</v>
       </c>
       <c r="F276" s="1">
         <v>46254</v>
@@ -9190,7 +9316,7 @@
         <v>0</v>
       </c>
       <c r="B277" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C277">
         <v>1</v>
@@ -9199,7 +9325,7 @@
         <v>56</v>
       </c>
       <c r="E277" t="s">
-        <v>94</v>
+        <v>12</v>
       </c>
       <c r="F277" s="1">
         <v>46254</v>
@@ -9216,16 +9342,16 @@
         <v>0</v>
       </c>
       <c r="B278" t="s">
+        <v>428</v>
+      </c>
+      <c r="C278">
+        <v>1</v>
+      </c>
+      <c r="D278" t="s">
+        <v>56</v>
+      </c>
+      <c r="E278" t="s">
         <v>429</v>
-      </c>
-      <c r="C278">
-        <v>1</v>
-      </c>
-      <c r="D278" t="s">
-        <v>56</v>
-      </c>
-      <c r="E278" t="s">
-        <v>430</v>
       </c>
       <c r="F278" s="1">
         <v>46254</v>
@@ -9242,16 +9368,16 @@
         <v>0</v>
       </c>
       <c r="B279" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C279">
         <v>1</v>
       </c>
       <c r="D279" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E279" t="s">
-        <v>432</v>
+        <v>94</v>
       </c>
       <c r="F279" s="1">
         <v>46254</v>
@@ -9268,7 +9394,7 @@
         <v>0</v>
       </c>
       <c r="B280" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C280">
         <v>1</v>
@@ -9277,7 +9403,7 @@
         <v>56</v>
       </c>
       <c r="E280" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="F280" s="1">
         <v>46254</v>
@@ -9291,51 +9417,51 @@
     </row>
     <row r="281" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
-        <v>435</v>
+        <v>0</v>
       </c>
       <c r="B281" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C281">
         <v>1</v>
       </c>
       <c r="D281" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E281" t="s">
-        <v>275</v>
+        <v>434</v>
       </c>
       <c r="F281" s="1">
-        <v>46148</v>
+        <v>46254</v>
       </c>
       <c r="G281" s="1">
-        <v>46149</v>
+        <v>46254</v>
       </c>
       <c r="H281">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B282" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C282">
         <v>1</v>
       </c>
       <c r="D282" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E282" t="s">
-        <v>29</v>
+        <v>436</v>
       </c>
       <c r="F282" s="1">
-        <v>46133</v>
+        <v>46254</v>
       </c>
       <c r="G282" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="H282">
         <v>0</v>
@@ -9343,25 +9469,25 @@
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
+        <v>0</v>
+      </c>
+      <c r="B283" t="s">
         <v>437</v>
       </c>
-      <c r="B283" t="s">
-        <v>439</v>
-      </c>
       <c r="C283">
         <v>1</v>
       </c>
       <c r="D283" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E283" t="s">
-        <v>29</v>
+        <v>438</v>
       </c>
       <c r="F283" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="G283" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="H283">
         <v>0</v>
@@ -9369,25 +9495,25 @@
     </row>
     <row r="284" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B284" t="s">
+        <v>439</v>
+      </c>
+      <c r="C284">
+        <v>1</v>
+      </c>
+      <c r="D284" t="s">
+        <v>56</v>
+      </c>
+      <c r="E284" t="s">
         <v>440</v>
       </c>
-      <c r="C284">
-        <v>1</v>
-      </c>
-      <c r="D284" t="s">
-        <v>5</v>
-      </c>
-      <c r="E284" t="s">
-        <v>14</v>
-      </c>
       <c r="F284" s="1">
-        <v>46156</v>
+        <v>46254</v>
       </c>
       <c r="G284" s="1">
-        <v>46156</v>
+        <v>46254</v>
       </c>
       <c r="H284">
         <v>0</v>
@@ -9395,7 +9521,7 @@
     </row>
     <row r="285" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B285" t="s">
         <v>441</v>
@@ -9404,30 +9530,30 @@
         <v>1</v>
       </c>
       <c r="D285" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E285" t="s">
-        <v>434</v>
+        <v>54</v>
       </c>
       <c r="F285" s="1">
-        <v>46195</v>
+        <v>46254</v>
       </c>
       <c r="G285" s="1">
-        <v>46195</v>
+        <v>46254</v>
       </c>
       <c r="H285">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B286" t="s">
         <v>442</v>
       </c>
       <c r="C286">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D286" t="s">
         <v>56</v>
@@ -9436,10 +9562,10 @@
         <v>443</v>
       </c>
       <c r="F286" s="1">
-        <v>46206</v>
+        <v>46254</v>
       </c>
       <c r="G286" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H286">
         <v>0</v>
@@ -9447,51 +9573,51 @@
     </row>
     <row r="287" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B287" t="s">
         <v>444</v>
       </c>
       <c r="C287">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D287" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E287" t="s">
-        <v>445</v>
+        <v>12</v>
       </c>
       <c r="F287" s="1">
-        <v>46209</v>
+        <v>46254</v>
       </c>
       <c r="G287" s="1">
-        <v>46218</v>
+        <v>46254</v>
       </c>
       <c r="H287">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B288" t="s">
+        <v>445</v>
+      </c>
+      <c r="C288">
+        <v>1</v>
+      </c>
+      <c r="D288" t="s">
+        <v>56</v>
+      </c>
+      <c r="E288" t="s">
         <v>446</v>
       </c>
-      <c r="C288">
-        <v>1</v>
-      </c>
-      <c r="D288" t="s">
-        <v>5</v>
-      </c>
-      <c r="E288" t="s">
-        <v>447</v>
-      </c>
       <c r="F288" s="1">
-        <v>46213</v>
+        <v>46254</v>
       </c>
       <c r="G288" s="1">
-        <v>46213</v>
+        <v>46254</v>
       </c>
       <c r="H288">
         <v>0</v>
@@ -9499,85 +9625,85 @@
     </row>
     <row r="289" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B289" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C289">
         <v>1</v>
       </c>
       <c r="D289" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E289" t="s">
-        <v>208</v>
+        <v>3</v>
       </c>
       <c r="F289" s="1">
-        <v>46213</v>
+        <v>46254</v>
       </c>
       <c r="G289" s="1">
-        <v>46216</v>
+        <v>46254</v>
       </c>
       <c r="H289">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="290" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B290" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C290">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D290" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E290" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="F290" s="1">
-        <v>46220</v>
+        <v>46254</v>
       </c>
       <c r="G290" s="1">
-        <v>46231</v>
+        <v>46254</v>
       </c>
       <c r="H290">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="291" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B291" t="s">
+        <v>449</v>
+      </c>
+      <c r="C291">
+        <v>1</v>
+      </c>
+      <c r="D291" t="s">
+        <v>56</v>
+      </c>
+      <c r="E291" t="s">
         <v>450</v>
       </c>
-      <c r="C291">
-        <v>1</v>
-      </c>
-      <c r="D291" t="s">
-        <v>2</v>
-      </c>
-      <c r="E291" t="s">
-        <v>434</v>
-      </c>
       <c r="F291" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G291" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H291">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B292" t="s">
         <v>451</v>
@@ -9586,24 +9712,24 @@
         <v>1</v>
       </c>
       <c r="D292" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E292" t="s">
-        <v>208</v>
+        <v>132</v>
       </c>
       <c r="F292" s="1">
-        <v>46224</v>
+        <v>46254</v>
       </c>
       <c r="G292" s="1">
-        <v>46224</v>
+        <v>46254</v>
       </c>
       <c r="H292">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="293" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B293" t="s">
         <v>452</v>
@@ -9612,120 +9738,120 @@
         <v>1</v>
       </c>
       <c r="D293" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E293" t="s">
-        <v>434</v>
+        <v>453</v>
       </c>
       <c r="F293" s="1">
-        <v>46230</v>
+        <v>46254</v>
       </c>
       <c r="G293" s="1">
-        <v>46231</v>
+        <v>46254</v>
       </c>
       <c r="H293">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="294" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B294" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C294">
         <v>1</v>
       </c>
       <c r="D294" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E294" t="s">
-        <v>94</v>
+        <v>455</v>
       </c>
       <c r="F294" s="1">
-        <v>46232</v>
+        <v>46254</v>
       </c>
       <c r="G294" s="1">
-        <v>46233</v>
+        <v>46254</v>
       </c>
       <c r="H294">
-        <v>126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B295" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C295">
         <v>1</v>
       </c>
       <c r="D295" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E295" t="s">
-        <v>94</v>
+        <v>283</v>
       </c>
       <c r="F295" s="1">
-        <v>46232</v>
+        <v>46254</v>
       </c>
       <c r="G295" s="1">
-        <v>46233</v>
+        <v>46254</v>
       </c>
       <c r="H295">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="296" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B296" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="C296">
         <v>1</v>
       </c>
       <c r="D296" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E296" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F296" s="1">
-        <v>46238</v>
+        <v>46254</v>
       </c>
       <c r="G296" s="1">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="H296">
-        <v>117</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B297" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C297">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D297" t="s">
         <v>56</v>
       </c>
       <c r="E297" t="s">
-        <v>443</v>
+        <v>459</v>
       </c>
       <c r="F297" s="1">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="G297" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H297">
         <v>0</v>
@@ -9733,25 +9859,25 @@
     </row>
     <row r="298" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B298" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="C298">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D298" t="s">
         <v>56</v>
       </c>
       <c r="E298" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="F298" s="1">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="G298" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H298">
         <v>0</v>
@@ -9759,36 +9885,36 @@
     </row>
     <row r="299" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B299" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="C299">
         <v>1</v>
       </c>
       <c r="D299" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E299" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F299" s="1">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="G299" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H299">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="300" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B300" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="C300">
         <v>1</v>
@@ -9797,13 +9923,13 @@
         <v>56</v>
       </c>
       <c r="E300" t="s">
-        <v>293</v>
+        <v>464</v>
       </c>
       <c r="F300" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="G300" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H300">
         <v>0</v>
@@ -9811,10 +9937,10 @@
     </row>
     <row r="301" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B301" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="C301">
         <v>1</v>
@@ -9823,13 +9949,13 @@
         <v>56</v>
       </c>
       <c r="E301" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="F301" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="G301" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="H301">
         <v>0</v>
@@ -9837,25 +9963,25 @@
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B302" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="C302">
         <v>1</v>
       </c>
       <c r="D302" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E302" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="F302" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="G302" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H302">
         <v>0</v>
@@ -9863,36 +9989,36 @@
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B303" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="C303">
         <v>1</v>
       </c>
       <c r="D303" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E303" t="s">
-        <v>208</v>
+        <v>469</v>
       </c>
       <c r="F303" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="G303" s="1">
         <v>46254</v>
       </c>
       <c r="H303">
-        <v>105</v>
+        <v>0</v>
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B304" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="C304">
         <v>1</v>
@@ -9901,13 +10027,13 @@
         <v>56</v>
       </c>
       <c r="E304" t="s">
-        <v>139</v>
+        <v>471</v>
       </c>
       <c r="F304" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="G304" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H304">
         <v>0</v>
@@ -9915,10 +10041,10 @@
     </row>
     <row r="305" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B305" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="C305">
         <v>1</v>
@@ -9927,10 +10053,10 @@
         <v>56</v>
       </c>
       <c r="E305" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
       <c r="F305" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="G305" s="1">
         <v>46254</v>
@@ -9941,10 +10067,10 @@
     </row>
     <row r="306" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B306" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C306">
         <v>1</v>
@@ -9953,7 +10079,7 @@
         <v>56</v>
       </c>
       <c r="E306" t="s">
-        <v>420</v>
+        <v>474</v>
       </c>
       <c r="F306" s="1">
         <v>46254</v>
@@ -9967,10 +10093,10 @@
     </row>
     <row r="307" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
-        <v>437</v>
+        <v>0</v>
       </c>
       <c r="B307" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="C307">
         <v>1</v>
@@ -9979,7 +10105,7 @@
         <v>56</v>
       </c>
       <c r="E307" t="s">
-        <v>14</v>
+        <v>388</v>
       </c>
       <c r="F307" s="1">
         <v>46254</v>
@@ -9993,62 +10119,62 @@
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
-        <v>437</v>
+        <v>476</v>
       </c>
       <c r="B308" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="C308">
         <v>1</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E308" t="s">
-        <v>94</v>
+        <v>275</v>
       </c>
       <c r="F308" s="1">
-        <v>46254</v>
+        <v>46148</v>
       </c>
       <c r="G308" s="1">
-        <v>46254</v>
+        <v>46149</v>
       </c>
       <c r="H308">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B309" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
       <c r="C309">
         <v>1</v>
       </c>
       <c r="D309" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="E309" t="s">
-        <v>471</v>
+        <v>29</v>
       </c>
       <c r="F309" s="1">
-        <v>46063</v>
+        <v>46133</v>
       </c>
       <c r="G309" s="1">
-        <v>46064</v>
+        <v>46134</v>
       </c>
       <c r="H309">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B310" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="C310">
         <v>1</v>
@@ -10057,13 +10183,13 @@
         <v>5</v>
       </c>
       <c r="E310" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F310" s="1">
-        <v>46113</v>
+        <v>46134</v>
       </c>
       <c r="G310" s="1">
-        <v>46125</v>
+        <v>46134</v>
       </c>
       <c r="H310">
         <v>0</v>
@@ -10071,36 +10197,36 @@
     </row>
     <row r="311" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B311" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="C311">
         <v>1</v>
       </c>
       <c r="D311" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E311" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="F311" s="1">
-        <v>46125</v>
+        <v>46156</v>
       </c>
       <c r="G311" s="1">
-        <v>46125</v>
+        <v>46156</v>
       </c>
       <c r="H311">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B312" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="C312">
         <v>1</v>
@@ -10109,65 +10235,65 @@
         <v>2</v>
       </c>
       <c r="E312" t="s">
-        <v>40</v>
+        <v>453</v>
       </c>
       <c r="F312" s="1">
-        <v>46126</v>
+        <v>46195</v>
       </c>
       <c r="G312" s="1">
-        <v>46126</v>
+        <v>46195</v>
       </c>
       <c r="H312">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B313" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="C313">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D313" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E313" t="s">
-        <v>40</v>
+        <v>484</v>
       </c>
       <c r="F313" s="1">
-        <v>46126</v>
+        <v>46206</v>
       </c>
       <c r="G313" s="1">
-        <v>46126</v>
+        <v>46252</v>
       </c>
       <c r="H313">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B314" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="C314">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D314" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E314" t="s">
-        <v>40</v>
+        <v>486</v>
       </c>
       <c r="F314" s="1">
-        <v>46128</v>
+        <v>46209</v>
       </c>
       <c r="G314" s="1">
-        <v>46128</v>
+        <v>46218</v>
       </c>
       <c r="H314">
         <v>1</v>
@@ -10175,10 +10301,10 @@
     </row>
     <row r="315" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B315" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="C315">
         <v>1</v>
@@ -10187,13 +10313,13 @@
         <v>5</v>
       </c>
       <c r="E315" t="s">
-        <v>40</v>
+        <v>488</v>
       </c>
       <c r="F315" s="1">
-        <v>46132</v>
+        <v>46213</v>
       </c>
       <c r="G315" s="1">
-        <v>46132</v>
+        <v>46213</v>
       </c>
       <c r="H315">
         <v>0</v>
@@ -10201,62 +10327,62 @@
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B316" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="C316">
         <v>1</v>
       </c>
       <c r="D316" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E316" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F316" s="1">
-        <v>46161</v>
+        <v>46213</v>
       </c>
       <c r="G316" s="1">
-        <v>46161</v>
+        <v>46216</v>
       </c>
       <c r="H316">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B317" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="C317">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D317" t="s">
         <v>2</v>
       </c>
       <c r="E317" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F317" s="1">
-        <v>46174</v>
+        <v>46220</v>
       </c>
       <c r="G317" s="1">
-        <v>46174</v>
+        <v>46231</v>
       </c>
       <c r="H317">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B318" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
       <c r="C318">
         <v>1</v>
@@ -10265,76 +10391,76 @@
         <v>2</v>
       </c>
       <c r="E318" t="s">
-        <v>40</v>
+        <v>453</v>
       </c>
       <c r="F318" s="1">
-        <v>46174</v>
+        <v>46223</v>
       </c>
       <c r="G318" s="1">
-        <v>46174</v>
+        <v>46223</v>
       </c>
       <c r="H318">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B319" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
       <c r="C319">
         <v>1</v>
       </c>
       <c r="D319" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E319" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F319" s="1">
-        <v>46195</v>
+        <v>46224</v>
       </c>
       <c r="G319" s="1">
-        <v>46252</v>
+        <v>46224</v>
       </c>
       <c r="H319">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B320" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="C320">
         <v>1</v>
       </c>
       <c r="D320" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E320" t="s">
-        <v>40</v>
+        <v>453</v>
       </c>
       <c r="F320" s="1">
-        <v>46210</v>
+        <v>46230</v>
       </c>
       <c r="G320" s="1">
-        <v>46210</v>
+        <v>46231</v>
       </c>
       <c r="H320">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B321" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="C321">
         <v>1</v>
@@ -10343,88 +10469,88 @@
         <v>2</v>
       </c>
       <c r="E321" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F321" s="1">
-        <v>46213</v>
+        <v>46232</v>
       </c>
       <c r="G321" s="1">
-        <v>46213</v>
+        <v>46233</v>
       </c>
       <c r="H321">
-        <v>1</v>
+        <v>126</v>
       </c>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B322" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
       <c r="C322">
         <v>1</v>
       </c>
       <c r="D322" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E322" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F322" s="1">
-        <v>46218</v>
+        <v>46232</v>
       </c>
       <c r="G322" s="1">
-        <v>46252</v>
+        <v>46233</v>
       </c>
       <c r="H322">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="323" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B323" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="C323">
         <v>1</v>
       </c>
       <c r="D323" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E323" t="s">
-        <v>54</v>
+        <v>208</v>
       </c>
       <c r="F323" s="1">
-        <v>46226</v>
+        <v>46238</v>
       </c>
       <c r="G323" s="1">
-        <v>46226</v>
+        <v>46239</v>
       </c>
       <c r="H323">
-        <v>0</v>
+        <v>117</v>
       </c>
     </row>
     <row r="324" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B324" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="C324">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D324" t="s">
         <v>56</v>
       </c>
       <c r="E324" t="s">
-        <v>40</v>
+        <v>484</v>
       </c>
       <c r="F324" s="1">
-        <v>46227</v>
+        <v>46239</v>
       </c>
       <c r="G324" s="1">
         <v>46252</v>
@@ -10435,22 +10561,22 @@
     </row>
     <row r="325" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B325" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="C325">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D325" t="s">
         <v>56</v>
       </c>
       <c r="E325" t="s">
-        <v>40</v>
+        <v>484</v>
       </c>
       <c r="F325" s="1">
-        <v>46227</v>
+        <v>46239</v>
       </c>
       <c r="G325" s="1">
         <v>46252</v>
@@ -10461,36 +10587,36 @@
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B326" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
       <c r="C326">
         <v>1</v>
       </c>
       <c r="D326" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E326" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F326" s="1">
-        <v>46227</v>
+        <v>46247</v>
       </c>
       <c r="G326" s="1">
-        <v>46228</v>
+        <v>46252</v>
       </c>
       <c r="H326">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B327" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="C327">
         <v>1</v>
@@ -10499,10 +10625,10 @@
         <v>56</v>
       </c>
       <c r="E327" t="s">
-        <v>54</v>
+        <v>293</v>
       </c>
       <c r="F327" s="1">
-        <v>46230</v>
+        <v>46252</v>
       </c>
       <c r="G327" s="1">
         <v>46252</v>
@@ -10513,25 +10639,25 @@
     </row>
     <row r="328" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B328" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="C328">
         <v>1</v>
       </c>
       <c r="D328" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E328" t="s">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="F328" s="1">
-        <v>46231</v>
+        <v>46252</v>
       </c>
       <c r="G328" s="1">
-        <v>46231</v>
+        <v>46252</v>
       </c>
       <c r="H328">
         <v>0</v>
@@ -10539,25 +10665,25 @@
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B329" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="C329">
         <v>1</v>
       </c>
       <c r="D329" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E329" t="s">
-        <v>40</v>
+        <v>503</v>
       </c>
       <c r="F329" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G329" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H329">
         <v>0</v>
@@ -10565,209 +10691,937 @@
     </row>
     <row r="330" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B330" t="s">
-        <v>492</v>
+        <v>504</v>
       </c>
       <c r="C330">
         <v>1</v>
       </c>
       <c r="D330" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E330" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F330" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G330" s="1">
         <v>46254</v>
       </c>
       <c r="H330">
-        <v>0</v>
+        <v>105</v>
       </c>
     </row>
     <row r="331" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B331" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="C331">
         <v>1</v>
       </c>
       <c r="D331" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E331" t="s">
-        <v>495</v>
+        <v>139</v>
       </c>
       <c r="F331" s="1">
-        <v>46083</v>
+        <v>46253</v>
       </c>
       <c r="G331" s="1">
-        <v>46084</v>
+        <v>46253</v>
       </c>
       <c r="H331">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="332" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B332" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="C332">
         <v>1</v>
       </c>
       <c r="D332" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E332" t="s">
-        <v>495</v>
+        <v>399</v>
       </c>
       <c r="F332" s="1">
-        <v>46132</v>
+        <v>46253</v>
       </c>
       <c r="G332" s="1">
-        <v>46133</v>
+        <v>46254</v>
       </c>
       <c r="H332">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="333" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B333" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="C333">
         <v>1</v>
       </c>
       <c r="D333" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E333" t="s">
-        <v>498</v>
+        <v>422</v>
       </c>
       <c r="F333" s="1">
-        <v>46157</v>
+        <v>46254</v>
       </c>
       <c r="G333" s="1">
-        <v>46157</v>
+        <v>46254</v>
       </c>
       <c r="H333">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="334" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B334" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="C334">
         <v>1</v>
       </c>
       <c r="D334" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E334" t="s">
-        <v>500</v>
+        <v>14</v>
       </c>
       <c r="F334" s="1">
-        <v>46168</v>
+        <v>46254</v>
       </c>
       <c r="G334" s="1">
-        <v>46170</v>
+        <v>46254</v>
       </c>
       <c r="H334">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="335" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B335" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
       <c r="C335">
         <v>1</v>
       </c>
       <c r="D335" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E335" t="s">
-        <v>498</v>
+        <v>94</v>
       </c>
       <c r="F335" s="1">
-        <v>46244</v>
+        <v>46254</v>
       </c>
       <c r="G335" s="1">
-        <v>46244</v>
+        <v>46254</v>
       </c>
       <c r="H335">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="336" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="B336" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="C336">
         <v>1</v>
       </c>
       <c r="D336" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E336" t="s">
-        <v>498</v>
+        <v>461</v>
       </c>
       <c r="F336" s="1">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="G336" s="1">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="H336">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
-        <v>493</v>
+        <v>511</v>
       </c>
       <c r="B337" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="C337">
         <v>1</v>
       </c>
       <c r="D337" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E337" t="s">
-        <v>495</v>
+        <v>513</v>
       </c>
       <c r="F337" s="1">
+        <v>46063</v>
+      </c>
+      <c r="G337" s="1">
+        <v>46064</v>
+      </c>
+      <c r="H337">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A338" t="s">
+        <v>511</v>
+      </c>
+      <c r="B338" t="s">
+        <v>514</v>
+      </c>
+      <c r="C338">
+        <v>1</v>
+      </c>
+      <c r="D338" t="s">
+        <v>5</v>
+      </c>
+      <c r="E338" t="s">
+        <v>40</v>
+      </c>
+      <c r="F338" s="1">
+        <v>46113</v>
+      </c>
+      <c r="G338" s="1">
+        <v>46125</v>
+      </c>
+      <c r="H338">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A339" t="s">
+        <v>511</v>
+      </c>
+      <c r="B339" t="s">
+        <v>515</v>
+      </c>
+      <c r="C339">
+        <v>1</v>
+      </c>
+      <c r="D339" t="s">
+        <v>2</v>
+      </c>
+      <c r="E339" t="s">
+        <v>40</v>
+      </c>
+      <c r="F339" s="1">
+        <v>46125</v>
+      </c>
+      <c r="G339" s="1">
+        <v>46125</v>
+      </c>
+      <c r="H339">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="340" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A340" t="s">
+        <v>511</v>
+      </c>
+      <c r="B340" t="s">
+        <v>516</v>
+      </c>
+      <c r="C340">
+        <v>1</v>
+      </c>
+      <c r="D340" t="s">
+        <v>2</v>
+      </c>
+      <c r="E340" t="s">
+        <v>40</v>
+      </c>
+      <c r="F340" s="1">
+        <v>46126</v>
+      </c>
+      <c r="G340" s="1">
+        <v>46126</v>
+      </c>
+      <c r="H340">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A341" t="s">
+        <v>511</v>
+      </c>
+      <c r="B341" t="s">
+        <v>517</v>
+      </c>
+      <c r="C341">
+        <v>1</v>
+      </c>
+      <c r="D341" t="s">
+        <v>2</v>
+      </c>
+      <c r="E341" t="s">
+        <v>40</v>
+      </c>
+      <c r="F341" s="1">
+        <v>46126</v>
+      </c>
+      <c r="G341" s="1">
+        <v>46126</v>
+      </c>
+      <c r="H341">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A342" t="s">
+        <v>511</v>
+      </c>
+      <c r="B342" t="s">
+        <v>518</v>
+      </c>
+      <c r="C342">
+        <v>1</v>
+      </c>
+      <c r="D342" t="s">
+        <v>2</v>
+      </c>
+      <c r="E342" t="s">
+        <v>40</v>
+      </c>
+      <c r="F342" s="1">
+        <v>46128</v>
+      </c>
+      <c r="G342" s="1">
+        <v>46128</v>
+      </c>
+      <c r="H342">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A343" t="s">
+        <v>511</v>
+      </c>
+      <c r="B343" t="s">
+        <v>519</v>
+      </c>
+      <c r="C343">
+        <v>1</v>
+      </c>
+      <c r="D343" t="s">
+        <v>5</v>
+      </c>
+      <c r="E343" t="s">
+        <v>40</v>
+      </c>
+      <c r="F343" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G343" s="1">
+        <v>46132</v>
+      </c>
+      <c r="H343">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A344" t="s">
+        <v>511</v>
+      </c>
+      <c r="B344" t="s">
+        <v>520</v>
+      </c>
+      <c r="C344">
+        <v>1</v>
+      </c>
+      <c r="D344" t="s">
+        <v>2</v>
+      </c>
+      <c r="E344" t="s">
+        <v>40</v>
+      </c>
+      <c r="F344" s="1">
+        <v>46161</v>
+      </c>
+      <c r="G344" s="1">
+        <v>46161</v>
+      </c>
+      <c r="H344">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="345" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A345" t="s">
+        <v>511</v>
+      </c>
+      <c r="B345" t="s">
+        <v>521</v>
+      </c>
+      <c r="C345">
+        <v>1</v>
+      </c>
+      <c r="D345" t="s">
+        <v>2</v>
+      </c>
+      <c r="E345" t="s">
+        <v>40</v>
+      </c>
+      <c r="F345" s="1">
+        <v>46174</v>
+      </c>
+      <c r="G345" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H345">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="346" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A346" t="s">
+        <v>511</v>
+      </c>
+      <c r="B346" t="s">
+        <v>522</v>
+      </c>
+      <c r="C346">
+        <v>1</v>
+      </c>
+      <c r="D346" t="s">
+        <v>2</v>
+      </c>
+      <c r="E346" t="s">
+        <v>40</v>
+      </c>
+      <c r="F346" s="1">
+        <v>46174</v>
+      </c>
+      <c r="G346" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H346">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="347" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A347" t="s">
+        <v>511</v>
+      </c>
+      <c r="B347" t="s">
+        <v>523</v>
+      </c>
+      <c r="C347">
+        <v>1</v>
+      </c>
+      <c r="D347" t="s">
+        <v>56</v>
+      </c>
+      <c r="E347" t="s">
+        <v>40</v>
+      </c>
+      <c r="F347" s="1">
+        <v>46195</v>
+      </c>
+      <c r="G347" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H347">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A348" t="s">
+        <v>511</v>
+      </c>
+      <c r="B348" t="s">
+        <v>524</v>
+      </c>
+      <c r="C348">
+        <v>1</v>
+      </c>
+      <c r="D348" t="s">
+        <v>5</v>
+      </c>
+      <c r="E348" t="s">
+        <v>40</v>
+      </c>
+      <c r="F348" s="1">
+        <v>46210</v>
+      </c>
+      <c r="G348" s="1">
+        <v>46210</v>
+      </c>
+      <c r="H348">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A349" t="s">
+        <v>511</v>
+      </c>
+      <c r="B349" t="s">
+        <v>525</v>
+      </c>
+      <c r="C349">
+        <v>1</v>
+      </c>
+      <c r="D349" t="s">
+        <v>2</v>
+      </c>
+      <c r="E349" t="s">
+        <v>40</v>
+      </c>
+      <c r="F349" s="1">
+        <v>46213</v>
+      </c>
+      <c r="G349" s="1">
+        <v>46213</v>
+      </c>
+      <c r="H349">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="350" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A350" t="s">
+        <v>511</v>
+      </c>
+      <c r="B350" t="s">
+        <v>526</v>
+      </c>
+      <c r="C350">
+        <v>1</v>
+      </c>
+      <c r="D350" t="s">
+        <v>56</v>
+      </c>
+      <c r="E350" t="s">
+        <v>40</v>
+      </c>
+      <c r="F350" s="1">
+        <v>46218</v>
+      </c>
+      <c r="G350" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H350">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A351" t="s">
+        <v>511</v>
+      </c>
+      <c r="B351" t="s">
+        <v>527</v>
+      </c>
+      <c r="C351">
+        <v>1</v>
+      </c>
+      <c r="D351" t="s">
+        <v>5</v>
+      </c>
+      <c r="E351" t="s">
+        <v>54</v>
+      </c>
+      <c r="F351" s="1">
+        <v>46226</v>
+      </c>
+      <c r="G351" s="1">
+        <v>46226</v>
+      </c>
+      <c r="H351">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A352" t="s">
+        <v>511</v>
+      </c>
+      <c r="B352" t="s">
+        <v>528</v>
+      </c>
+      <c r="C352">
+        <v>1</v>
+      </c>
+      <c r="D352" t="s">
+        <v>56</v>
+      </c>
+      <c r="E352" t="s">
+        <v>40</v>
+      </c>
+      <c r="F352" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G352" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H352">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A353" t="s">
+        <v>511</v>
+      </c>
+      <c r="B353" t="s">
+        <v>529</v>
+      </c>
+      <c r="C353">
+        <v>1</v>
+      </c>
+      <c r="D353" t="s">
+        <v>56</v>
+      </c>
+      <c r="E353" t="s">
+        <v>40</v>
+      </c>
+      <c r="F353" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G353" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H353">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A354" t="s">
+        <v>511</v>
+      </c>
+      <c r="B354" t="s">
+        <v>530</v>
+      </c>
+      <c r="C354">
+        <v>1</v>
+      </c>
+      <c r="D354" t="s">
+        <v>5</v>
+      </c>
+      <c r="E354" t="s">
+        <v>40</v>
+      </c>
+      <c r="F354" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G354" s="1">
+        <v>46228</v>
+      </c>
+      <c r="H354">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A355" t="s">
+        <v>511</v>
+      </c>
+      <c r="B355" t="s">
+        <v>531</v>
+      </c>
+      <c r="C355">
+        <v>1</v>
+      </c>
+      <c r="D355" t="s">
+        <v>56</v>
+      </c>
+      <c r="E355" t="s">
+        <v>54</v>
+      </c>
+      <c r="F355" s="1">
+        <v>46230</v>
+      </c>
+      <c r="G355" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H355">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A356" t="s">
+        <v>511</v>
+      </c>
+      <c r="B356" t="s">
+        <v>532</v>
+      </c>
+      <c r="C356">
+        <v>1</v>
+      </c>
+      <c r="D356" t="s">
+        <v>5</v>
+      </c>
+      <c r="E356" t="s">
+        <v>40</v>
+      </c>
+      <c r="F356" s="1">
+        <v>46231</v>
+      </c>
+      <c r="G356" s="1">
+        <v>46231</v>
+      </c>
+      <c r="H356">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A357" t="s">
+        <v>511</v>
+      </c>
+      <c r="B357" t="s">
+        <v>533</v>
+      </c>
+      <c r="C357">
+        <v>1</v>
+      </c>
+      <c r="D357" t="s">
+        <v>56</v>
+      </c>
+      <c r="E357" t="s">
+        <v>40</v>
+      </c>
+      <c r="F357" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G357" s="1">
+        <v>46254</v>
+      </c>
+      <c r="H357">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A358" t="s">
+        <v>511</v>
+      </c>
+      <c r="B358" t="s">
+        <v>534</v>
+      </c>
+      <c r="C358">
+        <v>1</v>
+      </c>
+      <c r="D358" t="s">
+        <v>56</v>
+      </c>
+      <c r="E358" t="s">
+        <v>40</v>
+      </c>
+      <c r="F358" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G358" s="1">
+        <v>46254</v>
+      </c>
+      <c r="H358">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A359" t="s">
+        <v>535</v>
+      </c>
+      <c r="B359" t="s">
+        <v>536</v>
+      </c>
+      <c r="C359">
+        <v>1</v>
+      </c>
+      <c r="D359" t="s">
+        <v>2</v>
+      </c>
+      <c r="E359" t="s">
+        <v>537</v>
+      </c>
+      <c r="F359" s="1">
+        <v>46083</v>
+      </c>
+      <c r="G359" s="1">
+        <v>46084</v>
+      </c>
+      <c r="H359">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="360" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A360" t="s">
+        <v>535</v>
+      </c>
+      <c r="B360" t="s">
+        <v>538</v>
+      </c>
+      <c r="C360">
+        <v>1</v>
+      </c>
+      <c r="D360" t="s">
+        <v>2</v>
+      </c>
+      <c r="E360" t="s">
+        <v>537</v>
+      </c>
+      <c r="F360" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G360" s="1">
+        <v>46133</v>
+      </c>
+      <c r="H360">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="361" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A361" t="s">
+        <v>535</v>
+      </c>
+      <c r="B361" t="s">
+        <v>539</v>
+      </c>
+      <c r="C361">
+        <v>1</v>
+      </c>
+      <c r="D361" t="s">
+        <v>2</v>
+      </c>
+      <c r="E361" t="s">
+        <v>540</v>
+      </c>
+      <c r="F361" s="1">
+        <v>46157</v>
+      </c>
+      <c r="G361" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H361">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="362" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A362" t="s">
+        <v>535</v>
+      </c>
+      <c r="B362" t="s">
+        <v>541</v>
+      </c>
+      <c r="C362">
+        <v>1</v>
+      </c>
+      <c r="D362" t="s">
+        <v>2</v>
+      </c>
+      <c r="E362" t="s">
+        <v>542</v>
+      </c>
+      <c r="F362" s="1">
+        <v>46168</v>
+      </c>
+      <c r="G362" s="1">
+        <v>46170</v>
+      </c>
+      <c r="H362">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="363" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A363" t="s">
+        <v>535</v>
+      </c>
+      <c r="B363" t="s">
+        <v>543</v>
+      </c>
+      <c r="C363">
+        <v>1</v>
+      </c>
+      <c r="D363" t="s">
+        <v>2</v>
+      </c>
+      <c r="E363" t="s">
+        <v>540</v>
+      </c>
+      <c r="F363" s="1">
+        <v>46244</v>
+      </c>
+      <c r="G363" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H363">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A364" t="s">
+        <v>535</v>
+      </c>
+      <c r="B364" t="s">
+        <v>544</v>
+      </c>
+      <c r="C364">
+        <v>1</v>
+      </c>
+      <c r="D364" t="s">
+        <v>2</v>
+      </c>
+      <c r="E364" t="s">
+        <v>540</v>
+      </c>
+      <c r="F364" s="1">
         <v>46247</v>
       </c>
-      <c r="G337" s="1">
+      <c r="G364" s="1">
         <v>46247</v>
       </c>
-      <c r="H337">
+      <c r="H364">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="365" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A365" t="s">
+        <v>535</v>
+      </c>
+      <c r="B365" t="s">
+        <v>545</v>
+      </c>
+      <c r="C365">
+        <v>1</v>
+      </c>
+      <c r="D365" t="s">
+        <v>2</v>
+      </c>
+      <c r="E365" t="s">
+        <v>537</v>
+      </c>
+      <c r="F365" s="1">
+        <v>46247</v>
+      </c>
+      <c r="G365" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H365">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 21/08/2026 09:30:52
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2A20913-C271-47CC-A699-8D2BECE761B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AB404C2-F1AE-49EA-BD41-CC52B66ACD6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3F966780-C724-4E90-A737-9EE2B961DE5B}"/>
+    <workbookView xWindow="26505" yWindow="3765" windowWidth="15375" windowHeight="8325" xr2:uid="{190D1A81-71E9-4756-9E1B-E75968853F8B}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="597">
   <si>
     <t>0001</t>
   </si>
@@ -1069,6 +1069,9 @@
     <t>CMM ARGENTINA SA</t>
   </si>
   <si>
+    <t xml:space="preserve">  213999</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214000</t>
   </si>
   <si>
@@ -1378,6 +1381,9 @@
     <t xml:space="preserve">  214099</t>
   </si>
   <si>
+    <t xml:space="preserve">  214100</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214101</t>
   </si>
   <si>
@@ -1447,9 +1453,117 @@
     <t>TUBOPLAST SRL</t>
   </si>
   <si>
+    <t xml:space="preserve">  214120</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214121</t>
   </si>
   <si>
+    <t xml:space="preserve">  214122</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214123</t>
+  </si>
+  <si>
+    <t>PERALTA DANIEL -SANIT. DAPER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214126</t>
+  </si>
+  <si>
+    <t>VALDEZ HUGO A -DEL SUR MATERIALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214127</t>
+  </si>
+  <si>
+    <t>SANITARIOS SANJUAN S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214128</t>
+  </si>
+  <si>
+    <t>LOSAMIL CONSTRUCCIONES S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214129</t>
+  </si>
+  <si>
+    <t>DE GIORGIO V,DE GIORGIO G,DE GIORGIO S,DE GIORGIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214136</t>
+  </si>
+  <si>
+    <t>NESGAMET S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214137</t>
+  </si>
+  <si>
+    <t>SANITARIOS YERBAL DE LUIS TALAMONA Y OSCAR TALAMON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214138</t>
+  </si>
+  <si>
+    <t>INTERMARBLE S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214142</t>
+  </si>
+  <si>
+    <t>DECORMAT S.R.L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214144</t>
+  </si>
+  <si>
+    <t>CASA CASMMA SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214148</t>
+  </si>
+  <si>
+    <t>PARDO MATERIALES SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214149</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  214151</t>
+  </si>
+  <si>
+    <t>VILLALBA MARIANO</t>
+  </si>
+  <si>
     <t>0004</t>
   </si>
   <si>
@@ -1540,21 +1654,36 @@
     <t xml:space="preserve">    2822</t>
   </si>
   <si>
-    <t xml:space="preserve">    2823</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2824</t>
   </si>
   <si>
-    <t xml:space="preserve">    2825</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2826</t>
   </si>
   <si>
+    <t xml:space="preserve">    2828</t>
+  </si>
+  <si>
     <t xml:space="preserve">    2829</t>
   </si>
   <si>
+    <t xml:space="preserve">    2830</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2831</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2832</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2834</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2835</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    2836</t>
+  </si>
+  <si>
     <t>4444</t>
   </si>
   <si>
@@ -1624,7 +1753,7 @@
     <t xml:space="preserve">    2240</t>
   </si>
   <si>
-    <t xml:space="preserve">    2247</t>
+    <t xml:space="preserve">    2254</t>
   </si>
   <si>
     <t>9999</t>
@@ -2131,34 +2260,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E418CEC2-71E4-477F-B2C9-1ADD17A8D4DA}">
-  <dimension ref="A1:H365"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C9B5CD1-D75A-4780-8000-E5B6EBE21ABB}">
+  <dimension ref="A1:H396"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>546</v>
+        <v>589</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>547</v>
+        <v>590</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>548</v>
+        <v>591</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>549</v>
+        <v>592</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>550</v>
+        <v>593</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>551</v>
+        <v>594</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>552</v>
+        <v>595</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>553</v>
+        <v>596</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -6644,7 +6773,7 @@
         <v>1</v>
       </c>
       <c r="D174" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E174" t="s">
         <v>281</v>
@@ -6656,7 +6785,7 @@
         <v>46252</v>
       </c>
       <c r="H174">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.2">
@@ -6904,7 +7033,7 @@
         <v>1</v>
       </c>
       <c r="D184" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E184" t="s">
         <v>297</v>
@@ -6916,7 +7045,7 @@
         <v>46254</v>
       </c>
       <c r="H184">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.2">
@@ -7398,7 +7527,7 @@
         <v>1</v>
       </c>
       <c r="D203" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E203" t="s">
         <v>324</v>
@@ -7410,7 +7539,7 @@
         <v>46253</v>
       </c>
       <c r="H203">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.2">
@@ -7424,7 +7553,7 @@
         <v>1</v>
       </c>
       <c r="D204" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E204" t="s">
         <v>326</v>
@@ -7436,7 +7565,7 @@
         <v>46253</v>
       </c>
       <c r="H204">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.2">
@@ -7528,7 +7657,7 @@
         <v>1</v>
       </c>
       <c r="D208" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E208" t="s">
         <v>134</v>
@@ -7540,7 +7669,7 @@
         <v>46254</v>
       </c>
       <c r="H208">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.2">
@@ -7554,7 +7683,7 @@
         <v>1</v>
       </c>
       <c r="D209" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E209" t="s">
         <v>134</v>
@@ -7566,7 +7695,7 @@
         <v>46254</v>
       </c>
       <c r="H209">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.2">
@@ -7580,7 +7709,7 @@
         <v>1</v>
       </c>
       <c r="D210" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E210" t="s">
         <v>163</v>
@@ -7592,7 +7721,7 @@
         <v>46253</v>
       </c>
       <c r="H210">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.2">
@@ -7895,13 +8024,13 @@
         <v>56</v>
       </c>
       <c r="E222" t="s">
-        <v>66</v>
+        <v>34</v>
       </c>
       <c r="F222" s="1">
         <v>46253</v>
       </c>
       <c r="G222" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H222">
         <v>0</v>
@@ -7918,10 +8047,10 @@
         <v>1</v>
       </c>
       <c r="D223" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E223" t="s">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="F223" s="1">
         <v>46253</v>
@@ -7930,7 +8059,7 @@
         <v>46253</v>
       </c>
       <c r="H223">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.2">
@@ -7944,10 +8073,10 @@
         <v>1</v>
       </c>
       <c r="D224" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E224" t="s">
-        <v>352</v>
+        <v>144</v>
       </c>
       <c r="F224" s="1">
         <v>46253</v>
@@ -7956,7 +8085,7 @@
         <v>46253</v>
       </c>
       <c r="H224">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.2">
@@ -7964,16 +8093,16 @@
         <v>0</v>
       </c>
       <c r="B225" t="s">
+        <v>352</v>
+      </c>
+      <c r="C225">
+        <v>1</v>
+      </c>
+      <c r="D225" t="s">
+        <v>56</v>
+      </c>
+      <c r="E225" t="s">
         <v>353</v>
-      </c>
-      <c r="C225">
-        <v>1</v>
-      </c>
-      <c r="D225" t="s">
-        <v>56</v>
-      </c>
-      <c r="E225" t="s">
-        <v>354</v>
       </c>
       <c r="F225" s="1">
         <v>46253</v>
@@ -7990,16 +8119,16 @@
         <v>0</v>
       </c>
       <c r="B226" t="s">
+        <v>354</v>
+      </c>
+      <c r="C226">
+        <v>1</v>
+      </c>
+      <c r="D226" t="s">
+        <v>56</v>
+      </c>
+      <c r="E226" t="s">
         <v>355</v>
-      </c>
-      <c r="C226">
-        <v>1</v>
-      </c>
-      <c r="D226" t="s">
-        <v>2</v>
-      </c>
-      <c r="E226" t="s">
-        <v>356</v>
       </c>
       <c r="F226" s="1">
         <v>46253</v>
@@ -8008,7 +8137,7 @@
         <v>46253</v>
       </c>
       <c r="H226">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.2">
@@ -8016,16 +8145,16 @@
         <v>0</v>
       </c>
       <c r="B227" t="s">
+        <v>356</v>
+      </c>
+      <c r="C227">
+        <v>1</v>
+      </c>
+      <c r="D227" t="s">
+        <v>2</v>
+      </c>
+      <c r="E227" t="s">
         <v>357</v>
-      </c>
-      <c r="C227">
-        <v>1</v>
-      </c>
-      <c r="D227" t="s">
-        <v>56</v>
-      </c>
-      <c r="E227" t="s">
-        <v>358</v>
       </c>
       <c r="F227" s="1">
         <v>46253</v>
@@ -8034,7 +8163,7 @@
         <v>46253</v>
       </c>
       <c r="H227">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="228" spans="1:8" x14ac:dyDescent="0.2">
@@ -8042,16 +8171,16 @@
         <v>0</v>
       </c>
       <c r="B228" t="s">
+        <v>358</v>
+      </c>
+      <c r="C228">
+        <v>1</v>
+      </c>
+      <c r="D228" t="s">
+        <v>56</v>
+      </c>
+      <c r="E228" t="s">
         <v>359</v>
-      </c>
-      <c r="C228">
-        <v>1</v>
-      </c>
-      <c r="D228" t="s">
-        <v>56</v>
-      </c>
-      <c r="E228" t="s">
-        <v>360</v>
       </c>
       <c r="F228" s="1">
         <v>46253</v>
@@ -8068,16 +8197,16 @@
         <v>0</v>
       </c>
       <c r="B229" t="s">
+        <v>360</v>
+      </c>
+      <c r="C229">
+        <v>1</v>
+      </c>
+      <c r="D229" t="s">
+        <v>56</v>
+      </c>
+      <c r="E229" t="s">
         <v>361</v>
-      </c>
-      <c r="C229">
-        <v>1</v>
-      </c>
-      <c r="D229" t="s">
-        <v>56</v>
-      </c>
-      <c r="E229" t="s">
-        <v>362</v>
       </c>
       <c r="F229" s="1">
         <v>46253</v>
@@ -8094,16 +8223,16 @@
         <v>0</v>
       </c>
       <c r="B230" t="s">
+        <v>362</v>
+      </c>
+      <c r="C230">
+        <v>1</v>
+      </c>
+      <c r="D230" t="s">
+        <v>56</v>
+      </c>
+      <c r="E230" t="s">
         <v>363</v>
-      </c>
-      <c r="C230">
-        <v>1</v>
-      </c>
-      <c r="D230" t="s">
-        <v>56</v>
-      </c>
-      <c r="E230" t="s">
-        <v>313</v>
       </c>
       <c r="F230" s="1">
         <v>46253</v>
@@ -8129,7 +8258,7 @@
         <v>56</v>
       </c>
       <c r="E231" t="s">
-        <v>365</v>
+        <v>313</v>
       </c>
       <c r="F231" s="1">
         <v>46253</v>
@@ -8146,16 +8275,16 @@
         <v>0</v>
       </c>
       <c r="B232" t="s">
+        <v>365</v>
+      </c>
+      <c r="C232">
+        <v>1</v>
+      </c>
+      <c r="D232" t="s">
+        <v>56</v>
+      </c>
+      <c r="E232" t="s">
         <v>366</v>
-      </c>
-      <c r="C232">
-        <v>1</v>
-      </c>
-      <c r="D232" t="s">
-        <v>56</v>
-      </c>
-      <c r="E232" t="s">
-        <v>367</v>
       </c>
       <c r="F232" s="1">
         <v>46253</v>
@@ -8172,22 +8301,22 @@
         <v>0</v>
       </c>
       <c r="B233" t="s">
+        <v>367</v>
+      </c>
+      <c r="C233">
+        <v>1</v>
+      </c>
+      <c r="D233" t="s">
+        <v>56</v>
+      </c>
+      <c r="E233" t="s">
         <v>368</v>
-      </c>
-      <c r="C233">
-        <v>1</v>
-      </c>
-      <c r="D233" t="s">
-        <v>56</v>
-      </c>
-      <c r="E233" t="s">
-        <v>16</v>
       </c>
       <c r="F233" s="1">
         <v>46253</v>
       </c>
       <c r="G233" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H233">
         <v>0</v>
@@ -8207,13 +8336,13 @@
         <v>56</v>
       </c>
       <c r="E234" t="s">
-        <v>370</v>
+        <v>16</v>
       </c>
       <c r="F234" s="1">
         <v>46253</v>
       </c>
       <c r="G234" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="H234">
         <v>0</v>
@@ -8224,16 +8353,16 @@
         <v>0</v>
       </c>
       <c r="B235" t="s">
+        <v>370</v>
+      </c>
+      <c r="C235">
+        <v>1</v>
+      </c>
+      <c r="D235" t="s">
+        <v>2</v>
+      </c>
+      <c r="E235" t="s">
         <v>371</v>
-      </c>
-      <c r="C235">
-        <v>1</v>
-      </c>
-      <c r="D235" t="s">
-        <v>56</v>
-      </c>
-      <c r="E235" t="s">
-        <v>372</v>
       </c>
       <c r="F235" s="1">
         <v>46253</v>
@@ -8242,7 +8371,7 @@
         <v>46253</v>
       </c>
       <c r="H235">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.2">
@@ -8250,16 +8379,16 @@
         <v>0</v>
       </c>
       <c r="B236" t="s">
+        <v>372</v>
+      </c>
+      <c r="C236">
+        <v>1</v>
+      </c>
+      <c r="D236" t="s">
+        <v>56</v>
+      </c>
+      <c r="E236" t="s">
         <v>373</v>
-      </c>
-      <c r="C236">
-        <v>1</v>
-      </c>
-      <c r="D236" t="s">
-        <v>56</v>
-      </c>
-      <c r="E236" t="s">
-        <v>139</v>
       </c>
       <c r="F236" s="1">
         <v>46253</v>
@@ -8285,7 +8414,7 @@
         <v>56</v>
       </c>
       <c r="E237" t="s">
-        <v>313</v>
+        <v>139</v>
       </c>
       <c r="F237" s="1">
         <v>46253</v>
@@ -8311,7 +8440,7 @@
         <v>56</v>
       </c>
       <c r="E238" t="s">
-        <v>26</v>
+        <v>313</v>
       </c>
       <c r="F238" s="1">
         <v>46253</v>
@@ -8516,10 +8645,10 @@
         <v>1</v>
       </c>
       <c r="D246" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E246" t="s">
-        <v>384</v>
+        <v>26</v>
       </c>
       <c r="F246" s="1">
         <v>46253</v>
@@ -8528,7 +8657,7 @@
         <v>46253</v>
       </c>
       <c r="H246">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:8" x14ac:dyDescent="0.2">
@@ -8536,16 +8665,16 @@
         <v>0</v>
       </c>
       <c r="B247" t="s">
+        <v>384</v>
+      </c>
+      <c r="C247">
+        <v>1</v>
+      </c>
+      <c r="D247" t="s">
+        <v>2</v>
+      </c>
+      <c r="E247" t="s">
         <v>385</v>
-      </c>
-      <c r="C247">
-        <v>1</v>
-      </c>
-      <c r="D247" t="s">
-        <v>56</v>
-      </c>
-      <c r="E247" t="s">
-        <v>386</v>
       </c>
       <c r="F247" s="1">
         <v>46253</v>
@@ -8554,7 +8683,7 @@
         <v>46253</v>
       </c>
       <c r="H247">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.2">
@@ -8562,16 +8691,16 @@
         <v>0</v>
       </c>
       <c r="B248" t="s">
+        <v>386</v>
+      </c>
+      <c r="C248">
+        <v>1</v>
+      </c>
+      <c r="D248" t="s">
+        <v>56</v>
+      </c>
+      <c r="E248" t="s">
         <v>387</v>
-      </c>
-      <c r="C248">
-        <v>1</v>
-      </c>
-      <c r="D248" t="s">
-        <v>56</v>
-      </c>
-      <c r="E248" t="s">
-        <v>388</v>
       </c>
       <c r="F248" s="1">
         <v>46253</v>
@@ -8588,16 +8717,16 @@
         <v>0</v>
       </c>
       <c r="B249" t="s">
+        <v>388</v>
+      </c>
+      <c r="C249">
+        <v>1</v>
+      </c>
+      <c r="D249" t="s">
+        <v>56</v>
+      </c>
+      <c r="E249" t="s">
         <v>389</v>
-      </c>
-      <c r="C249">
-        <v>1</v>
-      </c>
-      <c r="D249" t="s">
-        <v>2</v>
-      </c>
-      <c r="E249" t="s">
-        <v>390</v>
       </c>
       <c r="F249" s="1">
         <v>46253</v>
@@ -8606,7 +8735,7 @@
         <v>46253</v>
       </c>
       <c r="H249">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:8" x14ac:dyDescent="0.2">
@@ -8614,16 +8743,16 @@
         <v>0</v>
       </c>
       <c r="B250" t="s">
+        <v>390</v>
+      </c>
+      <c r="C250">
+        <v>1</v>
+      </c>
+      <c r="D250" t="s">
+        <v>2</v>
+      </c>
+      <c r="E250" t="s">
         <v>391</v>
-      </c>
-      <c r="C250">
-        <v>1</v>
-      </c>
-      <c r="D250" t="s">
-        <v>2</v>
-      </c>
-      <c r="E250" t="s">
-        <v>337</v>
       </c>
       <c r="F250" s="1">
         <v>46253</v>
@@ -8632,7 +8761,7 @@
         <v>46253</v>
       </c>
       <c r="H250">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="251" spans="1:8" x14ac:dyDescent="0.2">
@@ -8646,19 +8775,19 @@
         <v>1</v>
       </c>
       <c r="D251" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E251" t="s">
-        <v>393</v>
+        <v>337</v>
       </c>
       <c r="F251" s="1">
         <v>46253</v>
       </c>
       <c r="G251" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H251">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="252" spans="1:8" x14ac:dyDescent="0.2">
@@ -8666,16 +8795,16 @@
         <v>0</v>
       </c>
       <c r="B252" t="s">
+        <v>393</v>
+      </c>
+      <c r="C252">
+        <v>1</v>
+      </c>
+      <c r="D252" t="s">
+        <v>68</v>
+      </c>
+      <c r="E252" t="s">
         <v>394</v>
-      </c>
-      <c r="C252">
-        <v>1</v>
-      </c>
-      <c r="D252" t="s">
-        <v>56</v>
-      </c>
-      <c r="E252" t="s">
-        <v>20</v>
       </c>
       <c r="F252" s="1">
         <v>46253</v>
@@ -8684,7 +8813,7 @@
         <v>46254</v>
       </c>
       <c r="H252">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.2">
@@ -8701,7 +8830,7 @@
         <v>56</v>
       </c>
       <c r="E253" t="s">
-        <v>396</v>
+        <v>20</v>
       </c>
       <c r="F253" s="1">
         <v>46253</v>
@@ -8718,16 +8847,16 @@
         <v>0</v>
       </c>
       <c r="B254" t="s">
+        <v>396</v>
+      </c>
+      <c r="C254">
+        <v>1</v>
+      </c>
+      <c r="D254" t="s">
+        <v>2</v>
+      </c>
+      <c r="E254" t="s">
         <v>397</v>
-      </c>
-      <c r="C254">
-        <v>1</v>
-      </c>
-      <c r="D254" t="s">
-        <v>56</v>
-      </c>
-      <c r="E254" t="s">
-        <v>396</v>
       </c>
       <c r="F254" s="1">
         <v>46253</v>
@@ -8736,7 +8865,7 @@
         <v>46254</v>
       </c>
       <c r="H254">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="255" spans="1:8" x14ac:dyDescent="0.2">
@@ -8750,10 +8879,10 @@
         <v>1</v>
       </c>
       <c r="D255" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E255" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="F255" s="1">
         <v>46253</v>
@@ -8762,7 +8891,7 @@
         <v>46254</v>
       </c>
       <c r="H255">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.2">
@@ -8770,16 +8899,16 @@
         <v>0</v>
       </c>
       <c r="B256" t="s">
+        <v>399</v>
+      </c>
+      <c r="C256">
+        <v>1</v>
+      </c>
+      <c r="D256" t="s">
+        <v>2</v>
+      </c>
+      <c r="E256" t="s">
         <v>400</v>
-      </c>
-      <c r="C256">
-        <v>1</v>
-      </c>
-      <c r="D256" t="s">
-        <v>56</v>
-      </c>
-      <c r="E256" t="s">
-        <v>52</v>
       </c>
       <c r="F256" s="1">
         <v>46253</v>
@@ -8788,7 +8917,7 @@
         <v>46254</v>
       </c>
       <c r="H256">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="257" spans="1:8" x14ac:dyDescent="0.2">
@@ -8802,7 +8931,7 @@
         <v>1</v>
       </c>
       <c r="D257" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E257" t="s">
         <v>52</v>
@@ -8814,7 +8943,7 @@
         <v>46254</v>
       </c>
       <c r="H257">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="258" spans="1:8" x14ac:dyDescent="0.2">
@@ -8828,7 +8957,7 @@
         <v>1</v>
       </c>
       <c r="D258" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E258" t="s">
         <v>52</v>
@@ -8840,7 +8969,7 @@
         <v>46254</v>
       </c>
       <c r="H258">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="259" spans="1:8" x14ac:dyDescent="0.2">
@@ -8857,7 +8986,7 @@
         <v>56</v>
       </c>
       <c r="E259" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="F259" s="1">
         <v>46253</v>
@@ -8880,10 +9009,10 @@
         <v>1</v>
       </c>
       <c r="D260" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E260" t="s">
-        <v>405</v>
+        <v>18</v>
       </c>
       <c r="F260" s="1">
         <v>46253</v>
@@ -8892,7 +9021,7 @@
         <v>46254</v>
       </c>
       <c r="H260">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="261" spans="1:8" x14ac:dyDescent="0.2">
@@ -8900,16 +9029,16 @@
         <v>0</v>
       </c>
       <c r="B261" t="s">
+        <v>405</v>
+      </c>
+      <c r="C261">
+        <v>1</v>
+      </c>
+      <c r="D261" t="s">
+        <v>56</v>
+      </c>
+      <c r="E261" t="s">
         <v>406</v>
-      </c>
-      <c r="C261">
-        <v>2</v>
-      </c>
-      <c r="D261" t="s">
-        <v>56</v>
-      </c>
-      <c r="E261" t="s">
-        <v>407</v>
       </c>
       <c r="F261" s="1">
         <v>46253</v>
@@ -8926,16 +9055,16 @@
         <v>0</v>
       </c>
       <c r="B262" t="s">
+        <v>407</v>
+      </c>
+      <c r="C262">
+        <v>2</v>
+      </c>
+      <c r="D262" t="s">
+        <v>56</v>
+      </c>
+      <c r="E262" t="s">
         <v>408</v>
-      </c>
-      <c r="C262">
-        <v>1</v>
-      </c>
-      <c r="D262" t="s">
-        <v>56</v>
-      </c>
-      <c r="E262" t="s">
-        <v>281</v>
       </c>
       <c r="F262" s="1">
         <v>46253</v>
@@ -8958,19 +9087,19 @@
         <v>1</v>
       </c>
       <c r="D263" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="E263" t="s">
-        <v>132</v>
+        <v>281</v>
       </c>
       <c r="F263" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G263" s="1">
         <v>46254</v>
       </c>
       <c r="H263">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="264" spans="1:8" x14ac:dyDescent="0.2">
@@ -8987,7 +9116,7 @@
         <v>56</v>
       </c>
       <c r="E264" t="s">
-        <v>70</v>
+        <v>132</v>
       </c>
       <c r="F264" s="1">
         <v>46254</v>
@@ -9013,7 +9142,7 @@
         <v>56</v>
       </c>
       <c r="E265" t="s">
-        <v>412</v>
+        <v>70</v>
       </c>
       <c r="F265" s="1">
         <v>46254</v>
@@ -9030,17 +9159,17 @@
         <v>0</v>
       </c>
       <c r="B266" t="s">
+        <v>412</v>
+      </c>
+      <c r="C266">
+        <v>1</v>
+      </c>
+      <c r="D266" t="s">
+        <v>56</v>
+      </c>
+      <c r="E266" t="s">
         <v>413</v>
       </c>
-      <c r="C266">
-        <v>1</v>
-      </c>
-      <c r="D266" t="s">
-        <v>2</v>
-      </c>
-      <c r="E266" t="s">
-        <v>414</v>
-      </c>
       <c r="F266" s="1">
         <v>46254</v>
       </c>
@@ -9048,7 +9177,7 @@
         <v>46254</v>
       </c>
       <c r="H266">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="267" spans="1:8" x14ac:dyDescent="0.2">
@@ -9056,17 +9185,17 @@
         <v>0</v>
       </c>
       <c r="B267" t="s">
+        <v>414</v>
+      </c>
+      <c r="C267">
+        <v>1</v>
+      </c>
+      <c r="D267" t="s">
+        <v>2</v>
+      </c>
+      <c r="E267" t="s">
         <v>415</v>
       </c>
-      <c r="C267">
-        <v>1</v>
-      </c>
-      <c r="D267" t="s">
-        <v>56</v>
-      </c>
-      <c r="E267" t="s">
-        <v>416</v>
-      </c>
       <c r="F267" s="1">
         <v>46254</v>
       </c>
@@ -9074,7 +9203,7 @@
         <v>46254</v>
       </c>
       <c r="H267">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="268" spans="1:8" x14ac:dyDescent="0.2">
@@ -9082,16 +9211,16 @@
         <v>0</v>
       </c>
       <c r="B268" t="s">
+        <v>416</v>
+      </c>
+      <c r="C268">
+        <v>1</v>
+      </c>
+      <c r="D268" t="s">
+        <v>56</v>
+      </c>
+      <c r="E268" t="s">
         <v>417</v>
-      </c>
-      <c r="C268">
-        <v>1</v>
-      </c>
-      <c r="D268" t="s">
-        <v>56</v>
-      </c>
-      <c r="E268" t="s">
-        <v>122</v>
       </c>
       <c r="F268" s="1">
         <v>46254</v>
@@ -9117,7 +9246,7 @@
         <v>56</v>
       </c>
       <c r="E269" t="s">
-        <v>26</v>
+        <v>122</v>
       </c>
       <c r="F269" s="1">
         <v>46254</v>
@@ -9195,7 +9324,7 @@
         <v>56</v>
       </c>
       <c r="E272" t="s">
-        <v>422</v>
+        <v>26</v>
       </c>
       <c r="F272" s="1">
         <v>46254</v>
@@ -9212,16 +9341,16 @@
         <v>0</v>
       </c>
       <c r="B273" t="s">
+        <v>422</v>
+      </c>
+      <c r="C273">
+        <v>1</v>
+      </c>
+      <c r="D273" t="s">
+        <v>56</v>
+      </c>
+      <c r="E273" t="s">
         <v>423</v>
-      </c>
-      <c r="C273">
-        <v>1</v>
-      </c>
-      <c r="D273" t="s">
-        <v>56</v>
-      </c>
-      <c r="E273" t="s">
-        <v>422</v>
       </c>
       <c r="F273" s="1">
         <v>46254</v>
@@ -9247,7 +9376,7 @@
         <v>56</v>
       </c>
       <c r="E274" t="s">
-        <v>14</v>
+        <v>423</v>
       </c>
       <c r="F274" s="1">
         <v>46254</v>
@@ -9270,10 +9399,10 @@
         <v>1</v>
       </c>
       <c r="D275" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E275" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="F275" s="1">
         <v>46254</v>
@@ -9282,7 +9411,7 @@
         <v>46254</v>
       </c>
       <c r="H275">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="276" spans="1:8" x14ac:dyDescent="0.2">
@@ -9299,7 +9428,7 @@
         <v>56</v>
       </c>
       <c r="E276" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F276" s="1">
         <v>46254</v>
@@ -9351,7 +9480,7 @@
         <v>56</v>
       </c>
       <c r="E278" t="s">
-        <v>429</v>
+        <v>12</v>
       </c>
       <c r="F278" s="1">
         <v>46254</v>
@@ -9368,16 +9497,16 @@
         <v>0</v>
       </c>
       <c r="B279" t="s">
+        <v>429</v>
+      </c>
+      <c r="C279">
+        <v>1</v>
+      </c>
+      <c r="D279" t="s">
+        <v>56</v>
+      </c>
+      <c r="E279" t="s">
         <v>430</v>
-      </c>
-      <c r="C279">
-        <v>1</v>
-      </c>
-      <c r="D279" t="s">
-        <v>56</v>
-      </c>
-      <c r="E279" t="s">
-        <v>94</v>
       </c>
       <c r="F279" s="1">
         <v>46254</v>
@@ -9403,7 +9532,7 @@
         <v>56</v>
       </c>
       <c r="E280" t="s">
-        <v>432</v>
+        <v>94</v>
       </c>
       <c r="F280" s="1">
         <v>46254</v>
@@ -9420,16 +9549,16 @@
         <v>0</v>
       </c>
       <c r="B281" t="s">
+        <v>432</v>
+      </c>
+      <c r="C281">
+        <v>1</v>
+      </c>
+      <c r="D281" t="s">
+        <v>56</v>
+      </c>
+      <c r="E281" t="s">
         <v>433</v>
-      </c>
-      <c r="C281">
-        <v>1</v>
-      </c>
-      <c r="D281" t="s">
-        <v>5</v>
-      </c>
-      <c r="E281" t="s">
-        <v>434</v>
       </c>
       <c r="F281" s="1">
         <v>46254</v>
@@ -9446,16 +9575,16 @@
         <v>0</v>
       </c>
       <c r="B282" t="s">
+        <v>434</v>
+      </c>
+      <c r="C282">
+        <v>1</v>
+      </c>
+      <c r="D282" t="s">
+        <v>5</v>
+      </c>
+      <c r="E282" t="s">
         <v>435</v>
-      </c>
-      <c r="C282">
-        <v>1</v>
-      </c>
-      <c r="D282" t="s">
-        <v>56</v>
-      </c>
-      <c r="E282" t="s">
-        <v>436</v>
       </c>
       <c r="F282" s="1">
         <v>46254</v>
@@ -9472,16 +9601,16 @@
         <v>0</v>
       </c>
       <c r="B283" t="s">
+        <v>436</v>
+      </c>
+      <c r="C283">
+        <v>1</v>
+      </c>
+      <c r="D283" t="s">
+        <v>56</v>
+      </c>
+      <c r="E283" t="s">
         <v>437</v>
-      </c>
-      <c r="C283">
-        <v>1</v>
-      </c>
-      <c r="D283" t="s">
-        <v>56</v>
-      </c>
-      <c r="E283" t="s">
-        <v>438</v>
       </c>
       <c r="F283" s="1">
         <v>46254</v>
@@ -9498,16 +9627,16 @@
         <v>0</v>
       </c>
       <c r="B284" t="s">
+        <v>438</v>
+      </c>
+      <c r="C284">
+        <v>1</v>
+      </c>
+      <c r="D284" t="s">
+        <v>56</v>
+      </c>
+      <c r="E284" t="s">
         <v>439</v>
-      </c>
-      <c r="C284">
-        <v>1</v>
-      </c>
-      <c r="D284" t="s">
-        <v>56</v>
-      </c>
-      <c r="E284" t="s">
-        <v>440</v>
       </c>
       <c r="F284" s="1">
         <v>46254</v>
@@ -9524,16 +9653,16 @@
         <v>0</v>
       </c>
       <c r="B285" t="s">
+        <v>440</v>
+      </c>
+      <c r="C285">
+        <v>1</v>
+      </c>
+      <c r="D285" t="s">
+        <v>56</v>
+      </c>
+      <c r="E285" t="s">
         <v>441</v>
-      </c>
-      <c r="C285">
-        <v>1</v>
-      </c>
-      <c r="D285" t="s">
-        <v>56</v>
-      </c>
-      <c r="E285" t="s">
-        <v>54</v>
       </c>
       <c r="F285" s="1">
         <v>46254</v>
@@ -9559,7 +9688,7 @@
         <v>56</v>
       </c>
       <c r="E286" t="s">
-        <v>443</v>
+        <v>54</v>
       </c>
       <c r="F286" s="1">
         <v>46254</v>
@@ -9576,16 +9705,16 @@
         <v>0</v>
       </c>
       <c r="B287" t="s">
+        <v>443</v>
+      </c>
+      <c r="C287">
+        <v>1</v>
+      </c>
+      <c r="D287" t="s">
+        <v>56</v>
+      </c>
+      <c r="E287" t="s">
         <v>444</v>
-      </c>
-      <c r="C287">
-        <v>1</v>
-      </c>
-      <c r="D287" t="s">
-        <v>56</v>
-      </c>
-      <c r="E287" t="s">
-        <v>12</v>
       </c>
       <c r="F287" s="1">
         <v>46254</v>
@@ -9611,7 +9740,7 @@
         <v>56</v>
       </c>
       <c r="E288" t="s">
-        <v>446</v>
+        <v>12</v>
       </c>
       <c r="F288" s="1">
         <v>46254</v>
@@ -9628,16 +9757,16 @@
         <v>0</v>
       </c>
       <c r="B289" t="s">
+        <v>446</v>
+      </c>
+      <c r="C289">
+        <v>1</v>
+      </c>
+      <c r="D289" t="s">
+        <v>56</v>
+      </c>
+      <c r="E289" t="s">
         <v>447</v>
-      </c>
-      <c r="C289">
-        <v>1</v>
-      </c>
-      <c r="D289" t="s">
-        <v>56</v>
-      </c>
-      <c r="E289" t="s">
-        <v>3</v>
       </c>
       <c r="F289" s="1">
         <v>46254</v>
@@ -9663,7 +9792,7 @@
         <v>56</v>
       </c>
       <c r="E290" t="s">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="F290" s="1">
         <v>46254</v>
@@ -9689,7 +9818,7 @@
         <v>56</v>
       </c>
       <c r="E291" t="s">
-        <v>450</v>
+        <v>57</v>
       </c>
       <c r="F291" s="1">
         <v>46254</v>
@@ -9706,16 +9835,16 @@
         <v>0</v>
       </c>
       <c r="B292" t="s">
+        <v>450</v>
+      </c>
+      <c r="C292">
+        <v>1</v>
+      </c>
+      <c r="D292" t="s">
+        <v>56</v>
+      </c>
+      <c r="E292" t="s">
         <v>451</v>
-      </c>
-      <c r="C292">
-        <v>1</v>
-      </c>
-      <c r="D292" t="s">
-        <v>56</v>
-      </c>
-      <c r="E292" t="s">
-        <v>132</v>
       </c>
       <c r="F292" s="1">
         <v>46254</v>
@@ -9741,7 +9870,7 @@
         <v>56</v>
       </c>
       <c r="E293" t="s">
-        <v>453</v>
+        <v>132</v>
       </c>
       <c r="F293" s="1">
         <v>46254</v>
@@ -9758,7 +9887,7 @@
         <v>0</v>
       </c>
       <c r="B294" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C294">
         <v>1</v>
@@ -9767,13 +9896,13 @@
         <v>56</v>
       </c>
       <c r="E294" t="s">
-        <v>455</v>
+        <v>281</v>
       </c>
       <c r="F294" s="1">
         <v>46254</v>
       </c>
       <c r="G294" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H294">
         <v>0</v>
@@ -9784,16 +9913,16 @@
         <v>0</v>
       </c>
       <c r="B295" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C295">
         <v>1</v>
       </c>
       <c r="D295" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E295" t="s">
-        <v>283</v>
+        <v>455</v>
       </c>
       <c r="F295" s="1">
         <v>46254</v>
@@ -9802,7 +9931,7 @@
         <v>46254</v>
       </c>
       <c r="H295">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="296" spans="1:8" x14ac:dyDescent="0.2">
@@ -9810,16 +9939,16 @@
         <v>0</v>
       </c>
       <c r="B296" t="s">
+        <v>456</v>
+      </c>
+      <c r="C296">
+        <v>1</v>
+      </c>
+      <c r="D296" t="s">
+        <v>56</v>
+      </c>
+      <c r="E296" t="s">
         <v>457</v>
-      </c>
-      <c r="C296">
-        <v>1</v>
-      </c>
-      <c r="D296" t="s">
-        <v>56</v>
-      </c>
-      <c r="E296" t="s">
-        <v>217</v>
       </c>
       <c r="F296" s="1">
         <v>46254</v>
@@ -9845,7 +9974,7 @@
         <v>56</v>
       </c>
       <c r="E297" t="s">
-        <v>459</v>
+        <v>283</v>
       </c>
       <c r="F297" s="1">
         <v>46254</v>
@@ -9862,7 +9991,7 @@
         <v>0</v>
       </c>
       <c r="B298" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C298">
         <v>1</v>
@@ -9871,7 +10000,7 @@
         <v>56</v>
       </c>
       <c r="E298" t="s">
-        <v>461</v>
+        <v>217</v>
       </c>
       <c r="F298" s="1">
         <v>46254</v>
@@ -9888,7 +10017,7 @@
         <v>0</v>
       </c>
       <c r="B299" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C299">
         <v>1</v>
@@ -9897,7 +10026,7 @@
         <v>56</v>
       </c>
       <c r="E299" t="s">
-        <v>12</v>
+        <v>461</v>
       </c>
       <c r="F299" s="1">
         <v>46254</v>
@@ -9914,16 +10043,16 @@
         <v>0</v>
       </c>
       <c r="B300" t="s">
+        <v>462</v>
+      </c>
+      <c r="C300">
+        <v>1</v>
+      </c>
+      <c r="D300" t="s">
+        <v>56</v>
+      </c>
+      <c r="E300" t="s">
         <v>463</v>
-      </c>
-      <c r="C300">
-        <v>1</v>
-      </c>
-      <c r="D300" t="s">
-        <v>56</v>
-      </c>
-      <c r="E300" t="s">
-        <v>464</v>
       </c>
       <c r="F300" s="1">
         <v>46254</v>
@@ -9940,7 +10069,7 @@
         <v>0</v>
       </c>
       <c r="B301" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C301">
         <v>1</v>
@@ -9949,7 +10078,7 @@
         <v>56</v>
       </c>
       <c r="E301" t="s">
-        <v>161</v>
+        <v>12</v>
       </c>
       <c r="F301" s="1">
         <v>46254</v>
@@ -9966,16 +10095,16 @@
         <v>0</v>
       </c>
       <c r="B302" t="s">
+        <v>465</v>
+      </c>
+      <c r="C302">
+        <v>1</v>
+      </c>
+      <c r="D302" t="s">
+        <v>56</v>
+      </c>
+      <c r="E302" t="s">
         <v>466</v>
-      </c>
-      <c r="C302">
-        <v>1</v>
-      </c>
-      <c r="D302" t="s">
-        <v>56</v>
-      </c>
-      <c r="E302" t="s">
-        <v>467</v>
       </c>
       <c r="F302" s="1">
         <v>46254</v>
@@ -9992,7 +10121,7 @@
         <v>0</v>
       </c>
       <c r="B303" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C303">
         <v>1</v>
@@ -10001,7 +10130,7 @@
         <v>56</v>
       </c>
       <c r="E303" t="s">
-        <v>469</v>
+        <v>161</v>
       </c>
       <c r="F303" s="1">
         <v>46254</v>
@@ -10018,7 +10147,7 @@
         <v>0</v>
       </c>
       <c r="B304" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C304">
         <v>1</v>
@@ -10027,7 +10156,7 @@
         <v>56</v>
       </c>
       <c r="E304" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="F304" s="1">
         <v>46254</v>
@@ -10044,7 +10173,7 @@
         <v>0</v>
       </c>
       <c r="B305" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C305">
         <v>1</v>
@@ -10053,7 +10182,7 @@
         <v>56</v>
       </c>
       <c r="E305" t="s">
-        <v>384</v>
+        <v>471</v>
       </c>
       <c r="F305" s="1">
         <v>46254</v>
@@ -10070,16 +10199,16 @@
         <v>0</v>
       </c>
       <c r="B306" t="s">
+        <v>472</v>
+      </c>
+      <c r="C306">
+        <v>1</v>
+      </c>
+      <c r="D306" t="s">
+        <v>56</v>
+      </c>
+      <c r="E306" t="s">
         <v>473</v>
-      </c>
-      <c r="C306">
-        <v>1</v>
-      </c>
-      <c r="D306" t="s">
-        <v>56</v>
-      </c>
-      <c r="E306" t="s">
-        <v>474</v>
       </c>
       <c r="F306" s="1">
         <v>46254</v>
@@ -10096,7 +10225,7 @@
         <v>0</v>
       </c>
       <c r="B307" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C307">
         <v>1</v>
@@ -10105,7 +10234,7 @@
         <v>56</v>
       </c>
       <c r="E307" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F307" s="1">
         <v>46254</v>
@@ -10119,51 +10248,51 @@
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
+        <v>0</v>
+      </c>
+      <c r="B308" t="s">
+        <v>475</v>
+      </c>
+      <c r="C308">
+        <v>1</v>
+      </c>
+      <c r="D308" t="s">
+        <v>56</v>
+      </c>
+      <c r="E308" t="s">
         <v>476</v>
       </c>
-      <c r="B308" t="s">
-        <v>477</v>
-      </c>
-      <c r="C308">
-        <v>1</v>
-      </c>
-      <c r="D308" t="s">
-        <v>2</v>
-      </c>
-      <c r="E308" t="s">
-        <v>275</v>
-      </c>
       <c r="F308" s="1">
-        <v>46148</v>
+        <v>46254</v>
       </c>
       <c r="G308" s="1">
-        <v>46149</v>
+        <v>46254</v>
       </c>
       <c r="H308">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B309" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C309">
         <v>1</v>
       </c>
       <c r="D309" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E309" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="F309" s="1">
-        <v>46133</v>
+        <v>46254</v>
       </c>
       <c r="G309" s="1">
-        <v>46134</v>
+        <v>46255</v>
       </c>
       <c r="H309">
         <v>0</v>
@@ -10171,25 +10300,25 @@
     </row>
     <row r="310" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
+        <v>0</v>
+      </c>
+      <c r="B310" t="s">
         <v>478</v>
       </c>
-      <c r="B310" t="s">
-        <v>480</v>
-      </c>
       <c r="C310">
         <v>1</v>
       </c>
       <c r="D310" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E310" t="s">
-        <v>29</v>
+        <v>389</v>
       </c>
       <c r="F310" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="G310" s="1">
-        <v>46134</v>
+        <v>46254</v>
       </c>
       <c r="H310">
         <v>0</v>
@@ -10197,25 +10326,25 @@
     </row>
     <row r="311" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B311" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C311">
         <v>1</v>
       </c>
       <c r="D311" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E311" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="F311" s="1">
-        <v>46156</v>
+        <v>46254</v>
       </c>
       <c r="G311" s="1">
-        <v>46156</v>
+        <v>46255</v>
       </c>
       <c r="H311">
         <v>0</v>
@@ -10223,51 +10352,51 @@
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B312" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C312">
         <v>1</v>
       </c>
       <c r="D312" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E312" t="s">
-        <v>453</v>
+        <v>481</v>
       </c>
       <c r="F312" s="1">
-        <v>46195</v>
+        <v>46254</v>
       </c>
       <c r="G312" s="1">
-        <v>46195</v>
+        <v>46255</v>
       </c>
       <c r="H312">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B313" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C313">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D313" t="s">
         <v>56</v>
       </c>
       <c r="E313" t="s">
-        <v>484</v>
+        <v>249</v>
       </c>
       <c r="F313" s="1">
-        <v>46206</v>
+        <v>46254</v>
       </c>
       <c r="G313" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H313">
         <v>0</v>
@@ -10275,51 +10404,51 @@
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B314" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C314">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D314" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E314" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F314" s="1">
-        <v>46209</v>
+        <v>46254</v>
       </c>
       <c r="G314" s="1">
-        <v>46218</v>
+        <v>46255</v>
       </c>
       <c r="H314">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="315" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B315" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C315">
         <v>1</v>
       </c>
       <c r="D315" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E315" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="F315" s="1">
-        <v>46213</v>
+        <v>46254</v>
       </c>
       <c r="G315" s="1">
-        <v>46213</v>
+        <v>46255</v>
       </c>
       <c r="H315">
         <v>0</v>
@@ -10327,59 +10456,59 @@
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B316" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="C316">
         <v>1</v>
       </c>
       <c r="D316" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E316" t="s">
-        <v>208</v>
+        <v>488</v>
       </c>
       <c r="F316" s="1">
-        <v>46213</v>
+        <v>46254</v>
       </c>
       <c r="G316" s="1">
-        <v>46216</v>
+        <v>46255</v>
       </c>
       <c r="H316">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B317" t="s">
+        <v>489</v>
+      </c>
+      <c r="C317">
+        <v>1</v>
+      </c>
+      <c r="D317" t="s">
+        <v>56</v>
+      </c>
+      <c r="E317" t="s">
         <v>490</v>
       </c>
-      <c r="C317">
-        <v>3</v>
-      </c>
-      <c r="D317" t="s">
-        <v>2</v>
-      </c>
-      <c r="E317" t="s">
-        <v>94</v>
-      </c>
       <c r="F317" s="1">
-        <v>46220</v>
+        <v>46254</v>
       </c>
       <c r="G317" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
       <c r="H317">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B318" t="s">
         <v>491</v>
@@ -10388,24 +10517,24 @@
         <v>1</v>
       </c>
       <c r="D318" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E318" t="s">
-        <v>453</v>
+        <v>490</v>
       </c>
       <c r="F318" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G318" s="1">
-        <v>46223</v>
+        <v>46255</v>
       </c>
       <c r="H318">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B319" t="s">
         <v>492</v>
@@ -10414,24 +10543,24 @@
         <v>1</v>
       </c>
       <c r="D319" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E319" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="F319" s="1">
-        <v>46224</v>
+        <v>46254</v>
       </c>
       <c r="G319" s="1">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="H319">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B320" t="s">
         <v>493</v>
@@ -10440,24 +10569,24 @@
         <v>1</v>
       </c>
       <c r="D320" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E320" t="s">
-        <v>453</v>
+        <v>490</v>
       </c>
       <c r="F320" s="1">
-        <v>46230</v>
+        <v>46254</v>
       </c>
       <c r="G320" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
       <c r="H320">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B321" t="s">
         <v>494</v>
@@ -10466,94 +10595,94 @@
         <v>1</v>
       </c>
       <c r="D321" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E321" t="s">
-        <v>94</v>
+        <v>495</v>
       </c>
       <c r="F321" s="1">
-        <v>46232</v>
+        <v>46254</v>
       </c>
       <c r="G321" s="1">
-        <v>46233</v>
+        <v>46255</v>
       </c>
       <c r="H321">
-        <v>126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B322" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C322">
         <v>1</v>
       </c>
       <c r="D322" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E322" t="s">
-        <v>94</v>
+        <v>497</v>
       </c>
       <c r="F322" s="1">
-        <v>46232</v>
+        <v>46254</v>
       </c>
       <c r="G322" s="1">
-        <v>46233</v>
+        <v>46255</v>
       </c>
       <c r="H322">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="323" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B323" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C323">
         <v>1</v>
       </c>
       <c r="D323" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E323" t="s">
-        <v>208</v>
+        <v>499</v>
       </c>
       <c r="F323" s="1">
-        <v>46238</v>
+        <v>46254</v>
       </c>
       <c r="G323" s="1">
-        <v>46239</v>
+        <v>46255</v>
       </c>
       <c r="H323">
-        <v>117</v>
+        <v>0</v>
       </c>
     </row>
     <row r="324" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B324" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C324">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D324" t="s">
         <v>56</v>
       </c>
       <c r="E324" t="s">
-        <v>484</v>
+        <v>261</v>
       </c>
       <c r="F324" s="1">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="G324" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H324">
         <v>0</v>
@@ -10561,25 +10690,25 @@
     </row>
     <row r="325" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B325" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C325">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D325" t="s">
         <v>56</v>
       </c>
       <c r="E325" t="s">
-        <v>484</v>
+        <v>257</v>
       </c>
       <c r="F325" s="1">
-        <v>46239</v>
+        <v>46254</v>
       </c>
       <c r="G325" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H325">
         <v>0</v>
@@ -10587,36 +10716,36 @@
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B326" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="C326">
         <v>1</v>
       </c>
       <c r="D326" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E326" t="s">
-        <v>29</v>
+        <v>503</v>
       </c>
       <c r="F326" s="1">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="G326" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H326">
-        <v>29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B327" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="C327">
         <v>1</v>
@@ -10625,13 +10754,13 @@
         <v>56</v>
       </c>
       <c r="E327" t="s">
-        <v>293</v>
+        <v>505</v>
       </c>
       <c r="F327" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="G327" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H327">
         <v>0</v>
@@ -10639,10 +10768,10 @@
     </row>
     <row r="328" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B328" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="C328">
         <v>1</v>
@@ -10651,13 +10780,13 @@
         <v>56</v>
       </c>
       <c r="E328" t="s">
-        <v>132</v>
+        <v>503</v>
       </c>
       <c r="F328" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
       <c r="G328" s="1">
-        <v>46252</v>
+        <v>46255</v>
       </c>
       <c r="H328">
         <v>0</v>
@@ -10665,25 +10794,25 @@
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B329" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="C329">
         <v>1</v>
       </c>
       <c r="D329" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E329" t="s">
-        <v>503</v>
+        <v>293</v>
       </c>
       <c r="F329" s="1">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="G329" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H329">
         <v>0</v>
@@ -10691,36 +10820,36 @@
     </row>
     <row r="330" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B330" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C330">
         <v>1</v>
       </c>
       <c r="D330" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E330" t="s">
-        <v>208</v>
+        <v>509</v>
       </c>
       <c r="F330" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="G330" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H330">
-        <v>105</v>
+        <v>0</v>
       </c>
     </row>
     <row r="331" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B331" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="C331">
         <v>1</v>
@@ -10729,13 +10858,13 @@
         <v>56</v>
       </c>
       <c r="E331" t="s">
-        <v>139</v>
+        <v>12</v>
       </c>
       <c r="F331" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="G331" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H331">
         <v>0</v>
@@ -10743,10 +10872,10 @@
     </row>
     <row r="332" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B332" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="C332">
         <v>1</v>
@@ -10755,13 +10884,13 @@
         <v>56</v>
       </c>
       <c r="E332" t="s">
-        <v>399</v>
+        <v>26</v>
       </c>
       <c r="F332" s="1">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="G332" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H332">
         <v>0</v>
@@ -10769,10 +10898,10 @@
     </row>
     <row r="333" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="B333" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="C333">
         <v>1</v>
@@ -10781,13 +10910,13 @@
         <v>56</v>
       </c>
       <c r="E333" t="s">
-        <v>422</v>
+        <v>513</v>
       </c>
       <c r="F333" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="G333" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="H333">
         <v>0</v>
@@ -10795,51 +10924,51 @@
     </row>
     <row r="334" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
-        <v>478</v>
+        <v>514</v>
       </c>
       <c r="B334" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="C334">
         <v>1</v>
       </c>
       <c r="D334" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E334" t="s">
-        <v>14</v>
+        <v>275</v>
       </c>
       <c r="F334" s="1">
-        <v>46254</v>
+        <v>46148</v>
       </c>
       <c r="G334" s="1">
-        <v>46254</v>
+        <v>46149</v>
       </c>
       <c r="H334">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="335" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
-        <v>478</v>
+        <v>516</v>
       </c>
       <c r="B335" t="s">
-        <v>509</v>
+        <v>517</v>
       </c>
       <c r="C335">
         <v>1</v>
       </c>
       <c r="D335" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E335" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="F335" s="1">
-        <v>46254</v>
+        <v>46133</v>
       </c>
       <c r="G335" s="1">
-        <v>46254</v>
+        <v>46134</v>
       </c>
       <c r="H335">
         <v>0</v>
@@ -10847,25 +10976,25 @@
     </row>
     <row r="336" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
-        <v>478</v>
+        <v>516</v>
       </c>
       <c r="B336" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="C336">
         <v>1</v>
       </c>
       <c r="D336" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E336" t="s">
-        <v>461</v>
+        <v>29</v>
       </c>
       <c r="F336" s="1">
-        <v>46254</v>
+        <v>46134</v>
       </c>
       <c r="G336" s="1">
-        <v>46254</v>
+        <v>46134</v>
       </c>
       <c r="H336">
         <v>0</v>
@@ -10873,103 +11002,103 @@
     </row>
     <row r="337" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B337" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="C337">
         <v>1</v>
       </c>
       <c r="D337" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="E337" t="s">
-        <v>513</v>
+        <v>14</v>
       </c>
       <c r="F337" s="1">
-        <v>46063</v>
+        <v>46156</v>
       </c>
       <c r="G337" s="1">
-        <v>46064</v>
+        <v>46156</v>
       </c>
       <c r="H337">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="338" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B338" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="C338">
         <v>1</v>
       </c>
       <c r="D338" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E338" t="s">
-        <v>40</v>
+        <v>455</v>
       </c>
       <c r="F338" s="1">
-        <v>46113</v>
+        <v>46195</v>
       </c>
       <c r="G338" s="1">
-        <v>46125</v>
+        <v>46195</v>
       </c>
       <c r="H338">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="339" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B339" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="C339">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D339" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E339" t="s">
-        <v>40</v>
+        <v>522</v>
       </c>
       <c r="F339" s="1">
-        <v>46125</v>
+        <v>46206</v>
       </c>
       <c r="G339" s="1">
-        <v>46125</v>
+        <v>46252</v>
       </c>
       <c r="H339">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="340" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B340" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="C340">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D340" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E340" t="s">
-        <v>40</v>
+        <v>524</v>
       </c>
       <c r="F340" s="1">
-        <v>46126</v>
+        <v>46209</v>
       </c>
       <c r="G340" s="1">
-        <v>46126</v>
+        <v>46218</v>
       </c>
       <c r="H340">
         <v>1</v>
@@ -10977,88 +11106,88 @@
     </row>
     <row r="341" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B341" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="C341">
         <v>1</v>
       </c>
       <c r="D341" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E341" t="s">
-        <v>40</v>
+        <v>526</v>
       </c>
       <c r="F341" s="1">
-        <v>46126</v>
+        <v>46213</v>
       </c>
       <c r="G341" s="1">
-        <v>46126</v>
+        <v>46213</v>
       </c>
       <c r="H341">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B342" t="s">
-        <v>518</v>
+        <v>527</v>
       </c>
       <c r="C342">
         <v>1</v>
       </c>
       <c r="D342" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E342" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F342" s="1">
-        <v>46128</v>
+        <v>46213</v>
       </c>
       <c r="G342" s="1">
-        <v>46128</v>
+        <v>46216</v>
       </c>
       <c r="H342">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="343" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B343" t="s">
-        <v>519</v>
+        <v>528</v>
       </c>
       <c r="C343">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D343" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E343" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F343" s="1">
-        <v>46132</v>
+        <v>46220</v>
       </c>
       <c r="G343" s="1">
-        <v>46132</v>
+        <v>46231</v>
       </c>
       <c r="H343">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="344" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B344" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="C344">
         <v>1</v>
@@ -11067,50 +11196,50 @@
         <v>2</v>
       </c>
       <c r="E344" t="s">
-        <v>40</v>
+        <v>455</v>
       </c>
       <c r="F344" s="1">
-        <v>46161</v>
+        <v>46223</v>
       </c>
       <c r="G344" s="1">
-        <v>46161</v>
+        <v>46223</v>
       </c>
       <c r="H344">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="345" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B345" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="C345">
         <v>1</v>
       </c>
       <c r="D345" t="s">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E345" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F345" s="1">
-        <v>46174</v>
+        <v>46224</v>
       </c>
       <c r="G345" s="1">
-        <v>46174</v>
+        <v>46224</v>
       </c>
       <c r="H345">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="346" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B346" t="s">
-        <v>522</v>
+        <v>531</v>
       </c>
       <c r="C346">
         <v>1</v>
@@ -11119,76 +11248,76 @@
         <v>2</v>
       </c>
       <c r="E346" t="s">
-        <v>40</v>
+        <v>455</v>
       </c>
       <c r="F346" s="1">
-        <v>46174</v>
+        <v>46230</v>
       </c>
       <c r="G346" s="1">
-        <v>46174</v>
+        <v>46231</v>
       </c>
       <c r="H346">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="347" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B347" t="s">
-        <v>523</v>
+        <v>532</v>
       </c>
       <c r="C347">
         <v>1</v>
       </c>
       <c r="D347" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E347" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F347" s="1">
-        <v>46195</v>
+        <v>46232</v>
       </c>
       <c r="G347" s="1">
-        <v>46252</v>
+        <v>46233</v>
       </c>
       <c r="H347">
-        <v>0</v>
+        <v>126</v>
       </c>
     </row>
     <row r="348" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B348" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="C348">
         <v>1</v>
       </c>
       <c r="D348" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E348" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="F348" s="1">
-        <v>46210</v>
+        <v>46232</v>
       </c>
       <c r="G348" s="1">
-        <v>46210</v>
+        <v>46233</v>
       </c>
       <c r="H348">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="349" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B349" t="s">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="C349">
         <v>1</v>
@@ -11197,36 +11326,36 @@
         <v>2</v>
       </c>
       <c r="E349" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F349" s="1">
-        <v>46213</v>
+        <v>46238</v>
       </c>
       <c r="G349" s="1">
-        <v>46213</v>
+        <v>46239</v>
       </c>
       <c r="H349">
-        <v>1</v>
+        <v>117</v>
       </c>
     </row>
     <row r="350" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B350" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="C350">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D350" t="s">
         <v>56</v>
       </c>
       <c r="E350" t="s">
-        <v>40</v>
+        <v>522</v>
       </c>
       <c r="F350" s="1">
-        <v>46218</v>
+        <v>46239</v>
       </c>
       <c r="G350" s="1">
         <v>46252</v>
@@ -11237,25 +11366,25 @@
     </row>
     <row r="351" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B351" t="s">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="C351">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D351" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E351" t="s">
-        <v>54</v>
+        <v>522</v>
       </c>
       <c r="F351" s="1">
-        <v>46226</v>
+        <v>46239</v>
       </c>
       <c r="G351" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
       <c r="H351">
         <v>0</v>
@@ -11263,36 +11392,36 @@
     </row>
     <row r="352" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B352" t="s">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="C352">
         <v>1</v>
       </c>
       <c r="D352" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E352" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F352" s="1">
-        <v>46227</v>
+        <v>46247</v>
       </c>
       <c r="G352" s="1">
         <v>46252</v>
       </c>
       <c r="H352">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="353" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B353" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="C353">
         <v>1</v>
@@ -11301,10 +11430,10 @@
         <v>56</v>
       </c>
       <c r="E353" t="s">
-        <v>40</v>
+        <v>293</v>
       </c>
       <c r="F353" s="1">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="G353" s="1">
         <v>46252</v>
@@ -11315,25 +11444,25 @@
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B354" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="C354">
         <v>1</v>
       </c>
       <c r="D354" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E354" t="s">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="F354" s="1">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="G354" s="1">
-        <v>46228</v>
+        <v>46252</v>
       </c>
       <c r="H354">
         <v>0</v>
@@ -11341,25 +11470,25 @@
     </row>
     <row r="355" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B355" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="C355">
         <v>1</v>
       </c>
       <c r="D355" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E355" t="s">
-        <v>54</v>
+        <v>541</v>
       </c>
       <c r="F355" s="1">
-        <v>46230</v>
+        <v>46253</v>
       </c>
       <c r="G355" s="1">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="H355">
         <v>0</v>
@@ -11367,36 +11496,36 @@
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B356" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="C356">
         <v>1</v>
       </c>
       <c r="D356" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E356" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="F356" s="1">
-        <v>46231</v>
+        <v>46253</v>
       </c>
       <c r="G356" s="1">
-        <v>46231</v>
+        <v>46254</v>
       </c>
       <c r="H356">
-        <v>0</v>
+        <v>105</v>
       </c>
     </row>
     <row r="357" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B357" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="C357">
         <v>1</v>
@@ -11405,13 +11534,13 @@
         <v>56</v>
       </c>
       <c r="E357" t="s">
-        <v>40</v>
+        <v>139</v>
       </c>
       <c r="F357" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G357" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="H357">
         <v>0</v>
@@ -11419,10 +11548,10 @@
     </row>
     <row r="358" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B358" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="C358">
         <v>1</v>
@@ -11431,7 +11560,7 @@
         <v>56</v>
       </c>
       <c r="E358" t="s">
-        <v>40</v>
+        <v>423</v>
       </c>
       <c r="F358" s="1">
         <v>46254</v>
@@ -11445,183 +11574,989 @@
     </row>
     <row r="359" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B359" t="s">
-        <v>536</v>
+        <v>545</v>
       </c>
       <c r="C359">
         <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E359" t="s">
-        <v>537</v>
+        <v>94</v>
       </c>
       <c r="F359" s="1">
-        <v>46083</v>
+        <v>46254</v>
       </c>
       <c r="G359" s="1">
-        <v>46084</v>
+        <v>46254</v>
       </c>
       <c r="H359">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="360" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B360" t="s">
-        <v>538</v>
+        <v>546</v>
       </c>
       <c r="C360">
         <v>1</v>
       </c>
       <c r="D360" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E360" t="s">
-        <v>537</v>
+        <v>98</v>
       </c>
       <c r="F360" s="1">
-        <v>46132</v>
+        <v>46254</v>
       </c>
       <c r="G360" s="1">
-        <v>46133</v>
+        <v>46255</v>
       </c>
       <c r="H360">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="361" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B361" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="C361">
         <v>1</v>
       </c>
       <c r="D361" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E361" t="s">
-        <v>540</v>
+        <v>463</v>
       </c>
       <c r="F361" s="1">
-        <v>46157</v>
+        <v>46254</v>
       </c>
       <c r="G361" s="1">
-        <v>46157</v>
+        <v>46254</v>
       </c>
       <c r="H361">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="362" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B362" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="C362">
         <v>1</v>
       </c>
       <c r="D362" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E362" t="s">
-        <v>542</v>
+        <v>98</v>
       </c>
       <c r="F362" s="1">
-        <v>46168</v>
+        <v>46254</v>
       </c>
       <c r="G362" s="1">
-        <v>46170</v>
+        <v>46255</v>
       </c>
       <c r="H362">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B363" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="C363">
         <v>1</v>
       </c>
       <c r="D363" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E363" t="s">
-        <v>540</v>
+        <v>100</v>
       </c>
       <c r="F363" s="1">
-        <v>46244</v>
+        <v>46254</v>
       </c>
       <c r="G363" s="1">
-        <v>46244</v>
+        <v>46255</v>
       </c>
       <c r="H363">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="364" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B364" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="C364">
         <v>1</v>
       </c>
       <c r="D364" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E364" t="s">
-        <v>540</v>
+        <v>110</v>
       </c>
       <c r="F364" s="1">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="G364" s="1">
-        <v>46247</v>
+        <v>46255</v>
       </c>
       <c r="H364">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="B365" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C365">
         <v>1</v>
       </c>
       <c r="D365" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E365" t="s">
-        <v>537</v>
+        <v>110</v>
       </c>
       <c r="F365" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G365" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H365">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A366" t="s">
+        <v>516</v>
+      </c>
+      <c r="B366" t="s">
+        <v>552</v>
+      </c>
+      <c r="C366">
+        <v>1</v>
+      </c>
+      <c r="D366" t="s">
+        <v>56</v>
+      </c>
+      <c r="E366" t="s">
+        <v>503</v>
+      </c>
+      <c r="F366" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G366" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H366">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A367" t="s">
+        <v>516</v>
+      </c>
+      <c r="B367" t="s">
+        <v>553</v>
+      </c>
+      <c r="C367">
+        <v>1</v>
+      </c>
+      <c r="D367" t="s">
+        <v>56</v>
+      </c>
+      <c r="E367" t="s">
+        <v>503</v>
+      </c>
+      <c r="F367" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G367" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H367">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A368" t="s">
+        <v>554</v>
+      </c>
+      <c r="B368" t="s">
+        <v>555</v>
+      </c>
+      <c r="C368">
+        <v>1</v>
+      </c>
+      <c r="D368" t="s">
+        <v>68</v>
+      </c>
+      <c r="E368" t="s">
+        <v>556</v>
+      </c>
+      <c r="F368" s="1">
+        <v>46063</v>
+      </c>
+      <c r="G368" s="1">
+        <v>46064</v>
+      </c>
+      <c r="H368">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A369" t="s">
+        <v>554</v>
+      </c>
+      <c r="B369" t="s">
+        <v>557</v>
+      </c>
+      <c r="C369">
+        <v>1</v>
+      </c>
+      <c r="D369" t="s">
+        <v>5</v>
+      </c>
+      <c r="E369" t="s">
+        <v>40</v>
+      </c>
+      <c r="F369" s="1">
+        <v>46113</v>
+      </c>
+      <c r="G369" s="1">
+        <v>46125</v>
+      </c>
+      <c r="H369">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A370" t="s">
+        <v>554</v>
+      </c>
+      <c r="B370" t="s">
+        <v>558</v>
+      </c>
+      <c r="C370">
+        <v>1</v>
+      </c>
+      <c r="D370" t="s">
+        <v>2</v>
+      </c>
+      <c r="E370" t="s">
+        <v>40</v>
+      </c>
+      <c r="F370" s="1">
+        <v>46125</v>
+      </c>
+      <c r="G370" s="1">
+        <v>46125</v>
+      </c>
+      <c r="H370">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="371" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A371" t="s">
+        <v>554</v>
+      </c>
+      <c r="B371" t="s">
+        <v>559</v>
+      </c>
+      <c r="C371">
+        <v>1</v>
+      </c>
+      <c r="D371" t="s">
+        <v>2</v>
+      </c>
+      <c r="E371" t="s">
+        <v>40</v>
+      </c>
+      <c r="F371" s="1">
+        <v>46126</v>
+      </c>
+      <c r="G371" s="1">
+        <v>46126</v>
+      </c>
+      <c r="H371">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A372" t="s">
+        <v>554</v>
+      </c>
+      <c r="B372" t="s">
+        <v>560</v>
+      </c>
+      <c r="C372">
+        <v>1</v>
+      </c>
+      <c r="D372" t="s">
+        <v>2</v>
+      </c>
+      <c r="E372" t="s">
+        <v>40</v>
+      </c>
+      <c r="F372" s="1">
+        <v>46126</v>
+      </c>
+      <c r="G372" s="1">
+        <v>46126</v>
+      </c>
+      <c r="H372">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A373" t="s">
+        <v>554</v>
+      </c>
+      <c r="B373" t="s">
+        <v>561</v>
+      </c>
+      <c r="C373">
+        <v>1</v>
+      </c>
+      <c r="D373" t="s">
+        <v>2</v>
+      </c>
+      <c r="E373" t="s">
+        <v>40</v>
+      </c>
+      <c r="F373" s="1">
+        <v>46128</v>
+      </c>
+      <c r="G373" s="1">
+        <v>46128</v>
+      </c>
+      <c r="H373">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="374" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A374" t="s">
+        <v>554</v>
+      </c>
+      <c r="B374" t="s">
+        <v>562</v>
+      </c>
+      <c r="C374">
+        <v>1</v>
+      </c>
+      <c r="D374" t="s">
+        <v>5</v>
+      </c>
+      <c r="E374" t="s">
+        <v>40</v>
+      </c>
+      <c r="F374" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G374" s="1">
+        <v>46132</v>
+      </c>
+      <c r="H374">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A375" t="s">
+        <v>554</v>
+      </c>
+      <c r="B375" t="s">
+        <v>563</v>
+      </c>
+      <c r="C375">
+        <v>1</v>
+      </c>
+      <c r="D375" t="s">
+        <v>2</v>
+      </c>
+      <c r="E375" t="s">
+        <v>40</v>
+      </c>
+      <c r="F375" s="1">
+        <v>46161</v>
+      </c>
+      <c r="G375" s="1">
+        <v>46161</v>
+      </c>
+      <c r="H375">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A376" t="s">
+        <v>554</v>
+      </c>
+      <c r="B376" t="s">
+        <v>564</v>
+      </c>
+      <c r="C376">
+        <v>1</v>
+      </c>
+      <c r="D376" t="s">
+        <v>2</v>
+      </c>
+      <c r="E376" t="s">
+        <v>40</v>
+      </c>
+      <c r="F376" s="1">
+        <v>46174</v>
+      </c>
+      <c r="G376" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H376">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A377" t="s">
+        <v>554</v>
+      </c>
+      <c r="B377" t="s">
+        <v>565</v>
+      </c>
+      <c r="C377">
+        <v>1</v>
+      </c>
+      <c r="D377" t="s">
+        <v>2</v>
+      </c>
+      <c r="E377" t="s">
+        <v>40</v>
+      </c>
+      <c r="F377" s="1">
+        <v>46174</v>
+      </c>
+      <c r="G377" s="1">
+        <v>46174</v>
+      </c>
+      <c r="H377">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A378" t="s">
+        <v>554</v>
+      </c>
+      <c r="B378" t="s">
+        <v>566</v>
+      </c>
+      <c r="C378">
+        <v>1</v>
+      </c>
+      <c r="D378" t="s">
+        <v>56</v>
+      </c>
+      <c r="E378" t="s">
+        <v>40</v>
+      </c>
+      <c r="F378" s="1">
+        <v>46195</v>
+      </c>
+      <c r="G378" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H378">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A379" t="s">
+        <v>554</v>
+      </c>
+      <c r="B379" t="s">
+        <v>567</v>
+      </c>
+      <c r="C379">
+        <v>1</v>
+      </c>
+      <c r="D379" t="s">
+        <v>5</v>
+      </c>
+      <c r="E379" t="s">
+        <v>40</v>
+      </c>
+      <c r="F379" s="1">
+        <v>46210</v>
+      </c>
+      <c r="G379" s="1">
+        <v>46210</v>
+      </c>
+      <c r="H379">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A380" t="s">
+        <v>554</v>
+      </c>
+      <c r="B380" t="s">
+        <v>568</v>
+      </c>
+      <c r="C380">
+        <v>1</v>
+      </c>
+      <c r="D380" t="s">
+        <v>2</v>
+      </c>
+      <c r="E380" t="s">
+        <v>40</v>
+      </c>
+      <c r="F380" s="1">
+        <v>46213</v>
+      </c>
+      <c r="G380" s="1">
+        <v>46213</v>
+      </c>
+      <c r="H380">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="381" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A381" t="s">
+        <v>554</v>
+      </c>
+      <c r="B381" t="s">
+        <v>569</v>
+      </c>
+      <c r="C381">
+        <v>1</v>
+      </c>
+      <c r="D381" t="s">
+        <v>56</v>
+      </c>
+      <c r="E381" t="s">
+        <v>40</v>
+      </c>
+      <c r="F381" s="1">
+        <v>46218</v>
+      </c>
+      <c r="G381" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H381">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A382" t="s">
+        <v>554</v>
+      </c>
+      <c r="B382" t="s">
+        <v>570</v>
+      </c>
+      <c r="C382">
+        <v>1</v>
+      </c>
+      <c r="D382" t="s">
+        <v>5</v>
+      </c>
+      <c r="E382" t="s">
+        <v>54</v>
+      </c>
+      <c r="F382" s="1">
+        <v>46226</v>
+      </c>
+      <c r="G382" s="1">
+        <v>46226</v>
+      </c>
+      <c r="H382">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A383" t="s">
+        <v>554</v>
+      </c>
+      <c r="B383" t="s">
+        <v>571</v>
+      </c>
+      <c r="C383">
+        <v>1</v>
+      </c>
+      <c r="D383" t="s">
+        <v>56</v>
+      </c>
+      <c r="E383" t="s">
+        <v>40</v>
+      </c>
+      <c r="F383" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G383" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H383">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A384" t="s">
+        <v>554</v>
+      </c>
+      <c r="B384" t="s">
+        <v>572</v>
+      </c>
+      <c r="C384">
+        <v>1</v>
+      </c>
+      <c r="D384" t="s">
+        <v>56</v>
+      </c>
+      <c r="E384" t="s">
+        <v>40</v>
+      </c>
+      <c r="F384" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G384" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H384">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A385" t="s">
+        <v>554</v>
+      </c>
+      <c r="B385" t="s">
+        <v>573</v>
+      </c>
+      <c r="C385">
+        <v>1</v>
+      </c>
+      <c r="D385" t="s">
+        <v>5</v>
+      </c>
+      <c r="E385" t="s">
+        <v>40</v>
+      </c>
+      <c r="F385" s="1">
+        <v>46227</v>
+      </c>
+      <c r="G385" s="1">
+        <v>46228</v>
+      </c>
+      <c r="H385">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A386" t="s">
+        <v>554</v>
+      </c>
+      <c r="B386" t="s">
+        <v>574</v>
+      </c>
+      <c r="C386">
+        <v>1</v>
+      </c>
+      <c r="D386" t="s">
+        <v>56</v>
+      </c>
+      <c r="E386" t="s">
+        <v>54</v>
+      </c>
+      <c r="F386" s="1">
+        <v>46230</v>
+      </c>
+      <c r="G386" s="1">
+        <v>46252</v>
+      </c>
+      <c r="H386">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A387" t="s">
+        <v>554</v>
+      </c>
+      <c r="B387" t="s">
+        <v>575</v>
+      </c>
+      <c r="C387">
+        <v>1</v>
+      </c>
+      <c r="D387" t="s">
+        <v>5</v>
+      </c>
+      <c r="E387" t="s">
+        <v>40</v>
+      </c>
+      <c r="F387" s="1">
+        <v>46231</v>
+      </c>
+      <c r="G387" s="1">
+        <v>46231</v>
+      </c>
+      <c r="H387">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A388" t="s">
+        <v>554</v>
+      </c>
+      <c r="B388" t="s">
+        <v>576</v>
+      </c>
+      <c r="C388">
+        <v>1</v>
+      </c>
+      <c r="D388" t="s">
+        <v>5</v>
+      </c>
+      <c r="E388" t="s">
+        <v>40</v>
+      </c>
+      <c r="F388" s="1">
+        <v>46254</v>
+      </c>
+      <c r="G388" s="1">
+        <v>46254</v>
+      </c>
+      <c r="H388">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A389" t="s">
+        <v>554</v>
+      </c>
+      <c r="B389" t="s">
+        <v>577</v>
+      </c>
+      <c r="C389">
+        <v>1</v>
+      </c>
+      <c r="D389" t="s">
+        <v>56</v>
+      </c>
+      <c r="E389" t="s">
+        <v>40</v>
+      </c>
+      <c r="F389" s="1">
+        <v>46255</v>
+      </c>
+      <c r="G389" s="1">
+        <v>46255</v>
+      </c>
+      <c r="H389">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A390" t="s">
+        <v>578</v>
+      </c>
+      <c r="B390" t="s">
+        <v>579</v>
+      </c>
+      <c r="C390">
+        <v>1</v>
+      </c>
+      <c r="D390" t="s">
+        <v>2</v>
+      </c>
+      <c r="E390" t="s">
+        <v>580</v>
+      </c>
+      <c r="F390" s="1">
+        <v>46083</v>
+      </c>
+      <c r="G390" s="1">
+        <v>46084</v>
+      </c>
+      <c r="H390">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="391" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A391" t="s">
+        <v>578</v>
+      </c>
+      <c r="B391" t="s">
+        <v>581</v>
+      </c>
+      <c r="C391">
+        <v>1</v>
+      </c>
+      <c r="D391" t="s">
+        <v>2</v>
+      </c>
+      <c r="E391" t="s">
+        <v>580</v>
+      </c>
+      <c r="F391" s="1">
+        <v>46132</v>
+      </c>
+      <c r="G391" s="1">
+        <v>46133</v>
+      </c>
+      <c r="H391">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A392" t="s">
+        <v>578</v>
+      </c>
+      <c r="B392" t="s">
+        <v>582</v>
+      </c>
+      <c r="C392">
+        <v>1</v>
+      </c>
+      <c r="D392" t="s">
+        <v>2</v>
+      </c>
+      <c r="E392" t="s">
+        <v>583</v>
+      </c>
+      <c r="F392" s="1">
+        <v>46157</v>
+      </c>
+      <c r="G392" s="1">
+        <v>46157</v>
+      </c>
+      <c r="H392">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="393" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A393" t="s">
+        <v>578</v>
+      </c>
+      <c r="B393" t="s">
+        <v>584</v>
+      </c>
+      <c r="C393">
+        <v>1</v>
+      </c>
+      <c r="D393" t="s">
+        <v>2</v>
+      </c>
+      <c r="E393" t="s">
+        <v>585</v>
+      </c>
+      <c r="F393" s="1">
+        <v>46168</v>
+      </c>
+      <c r="G393" s="1">
+        <v>46170</v>
+      </c>
+      <c r="H393">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="394" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A394" t="s">
+        <v>578</v>
+      </c>
+      <c r="B394" t="s">
+        <v>586</v>
+      </c>
+      <c r="C394">
+        <v>1</v>
+      </c>
+      <c r="D394" t="s">
+        <v>2</v>
+      </c>
+      <c r="E394" t="s">
+        <v>583</v>
+      </c>
+      <c r="F394" s="1">
+        <v>46244</v>
+      </c>
+      <c r="G394" s="1">
+        <v>46244</v>
+      </c>
+      <c r="H394">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="395" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A395" t="s">
+        <v>578</v>
+      </c>
+      <c r="B395" t="s">
+        <v>587</v>
+      </c>
+      <c r="C395">
+        <v>1</v>
+      </c>
+      <c r="D395" t="s">
+        <v>2</v>
+      </c>
+      <c r="E395" t="s">
+        <v>583</v>
+      </c>
+      <c r="F395" s="1">
         <v>46247</v>
       </c>
-      <c r="G365" s="1">
+      <c r="G395" s="1">
         <v>46247</v>
       </c>
-      <c r="H365">
+      <c r="H395">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="396" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A396" t="s">
+        <v>578</v>
+      </c>
+      <c r="B396" t="s">
+        <v>588</v>
+      </c>
+      <c r="C396">
+        <v>1</v>
+      </c>
+      <c r="D396" t="s">
+        <v>2</v>
+      </c>
+      <c r="E396" t="s">
+        <v>580</v>
+      </c>
+      <c r="F396" s="1">
+        <v>46247</v>
+      </c>
+      <c r="G396" s="1">
+        <v>46247</v>
+      </c>
+      <c r="H396">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 22/08/2026 09:52:03
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E55C8A46-0CD1-4E8F-AA00-A330D50EA55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BE52C57-FF3A-43EE-AD9F-B2B8F15C1584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27195" yWindow="4455" windowWidth="15375" windowHeight="8325" xr2:uid="{CE17D439-2207-4B04-856E-C2DA8F3F9AB0}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F3EF298B-41C7-4855-832E-4E769876D2B9}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2062" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2042" uniqueCount="811">
   <si>
     <t>0001</t>
   </si>
@@ -1741,6 +1741,9 @@
     <t>DECORMAT S.R.L.</t>
   </si>
   <si>
+    <t xml:space="preserve">  214143</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214144</t>
   </si>
   <si>
@@ -2014,15 +2017,18 @@
     <t xml:space="preserve">  214203</t>
   </si>
   <si>
+    <t xml:space="preserve">  214204</t>
+  </si>
+  <si>
+    <t>TB02</t>
+  </si>
+  <si>
+    <t>IT BROKERS S.A.</t>
+  </si>
+  <si>
     <t xml:space="preserve">  214205</t>
   </si>
   <si>
-    <t>TB02</t>
-  </si>
-  <si>
-    <t>IT BROKERS S.A.</t>
-  </si>
-  <si>
     <t xml:space="preserve">  214206</t>
   </si>
   <si>
@@ -2110,9 +2116,6 @@
     <t xml:space="preserve">  214222</t>
   </si>
   <si>
-    <t xml:space="preserve">  214223</t>
-  </si>
-  <si>
     <t xml:space="preserve">  214224</t>
   </si>
   <si>
@@ -2275,15 +2278,9 @@
     <t xml:space="preserve">    2827</t>
   </si>
   <si>
-    <t xml:space="preserve">    2828</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2829</t>
   </si>
   <si>
-    <t xml:space="preserve">    2830</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2831</t>
   </si>
   <si>
@@ -2317,9 +2314,6 @@
     <t>VARIOS</t>
   </si>
   <si>
-    <t xml:space="preserve">    2841</t>
-  </si>
-  <si>
     <t>4444</t>
   </si>
   <si>
@@ -2393,12 +2387,6 @@
   </si>
   <si>
     <t xml:space="preserve">    2258</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2261</t>
   </si>
   <si>
     <t>9999</t>
@@ -2914,31 +2902,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BA96046-D851-4BB7-B8CA-2F6FDF561BF7}">
-  <dimension ref="A1:G412"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE68528F-9967-494B-98A8-1493F02C3C69}">
+  <dimension ref="A1:G408"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>808</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>809</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>810</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>811</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>812</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>813</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -6537,7 +6525,7 @@
         <v>363</v>
       </c>
       <c r="C158" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D158" t="s">
         <v>364</v>
@@ -7664,7 +7652,7 @@
         <v>454</v>
       </c>
       <c r="C207" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D207" t="s">
         <v>455</v>
@@ -7917,7 +7905,7 @@
         <v>475</v>
       </c>
       <c r="C218" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D218" t="s">
         <v>16</v>
@@ -8124,7 +8112,7 @@
         <v>492</v>
       </c>
       <c r="C227" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D227" t="s">
         <v>493</v>
@@ -8193,7 +8181,7 @@
         <v>499</v>
       </c>
       <c r="C230" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D230" t="s">
         <v>138</v>
@@ -8699,7 +8687,7 @@
         <v>545</v>
       </c>
       <c r="C252" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D252" t="s">
         <v>546</v>
@@ -8722,7 +8710,7 @@
         <v>548</v>
       </c>
       <c r="C253" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D253" t="s">
         <v>546</v>
@@ -8768,7 +8756,7 @@
         <v>550</v>
       </c>
       <c r="C255" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D255" t="s">
         <v>546</v>
@@ -9024,16 +9012,16 @@
         <v>80</v>
       </c>
       <c r="D266" t="s">
-        <v>574</v>
+        <v>337</v>
       </c>
       <c r="E266" t="s">
-        <v>575</v>
+        <v>338</v>
       </c>
       <c r="F266" s="1">
         <v>46254</v>
       </c>
       <c r="G266" s="1">
-        <v>46255</v>
+        <v>46256</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.2">
@@ -9041,16 +9029,16 @@
         <v>0</v>
       </c>
       <c r="B267" t="s">
+        <v>574</v>
+      </c>
+      <c r="C267" t="s">
+        <v>80</v>
+      </c>
+      <c r="D267" t="s">
+        <v>575</v>
+      </c>
+      <c r="E267" t="s">
         <v>576</v>
-      </c>
-      <c r="C267" t="s">
-        <v>80</v>
-      </c>
-      <c r="D267" t="s">
-        <v>571</v>
-      </c>
-      <c r="E267" t="s">
-        <v>572</v>
       </c>
       <c r="F267" s="1">
         <v>46254</v>
@@ -9067,13 +9055,13 @@
         <v>577</v>
       </c>
       <c r="C268" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D268" t="s">
-        <v>216</v>
+        <v>571</v>
       </c>
       <c r="E268" t="s">
-        <v>217</v>
+        <v>572</v>
       </c>
       <c r="F268" s="1">
         <v>46254</v>
@@ -9090,13 +9078,13 @@
         <v>578</v>
       </c>
       <c r="C269" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D269" t="s">
-        <v>579</v>
+        <v>216</v>
       </c>
       <c r="E269" t="s">
-        <v>580</v>
+        <v>217</v>
       </c>
       <c r="F269" s="1">
         <v>46254</v>
@@ -9110,19 +9098,19 @@
         <v>0</v>
       </c>
       <c r="B270" t="s">
+        <v>579</v>
+      </c>
+      <c r="C270" t="s">
+        <v>80</v>
+      </c>
+      <c r="D270" t="s">
+        <v>580</v>
+      </c>
+      <c r="E270" t="s">
         <v>581</v>
       </c>
-      <c r="C270" t="s">
-        <v>80</v>
-      </c>
-      <c r="D270" t="s">
-        <v>16</v>
-      </c>
-      <c r="E270" t="s">
-        <v>17</v>
-      </c>
       <c r="F270" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G270" s="1">
         <v>46255</v>
@@ -9136,13 +9124,13 @@
         <v>582</v>
       </c>
       <c r="C271" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D271" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="E271" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="F271" s="1">
         <v>46255</v>
@@ -9159,13 +9147,13 @@
         <v>583</v>
       </c>
       <c r="C272" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D272" t="s">
-        <v>584</v>
+        <v>37</v>
       </c>
       <c r="E272" t="s">
-        <v>585</v>
+        <v>38</v>
       </c>
       <c r="F272" s="1">
         <v>46255</v>
@@ -9179,16 +9167,16 @@
         <v>0</v>
       </c>
       <c r="B273" t="s">
+        <v>584</v>
+      </c>
+      <c r="C273" t="s">
+        <v>2</v>
+      </c>
+      <c r="D273" t="s">
+        <v>585</v>
+      </c>
+      <c r="E273" t="s">
         <v>586</v>
-      </c>
-      <c r="C273" t="s">
-        <v>80</v>
-      </c>
-      <c r="D273" t="s">
-        <v>587</v>
-      </c>
-      <c r="E273" t="s">
-        <v>588</v>
       </c>
       <c r="F273" s="1">
         <v>46255</v>
@@ -9202,16 +9190,16 @@
         <v>0</v>
       </c>
       <c r="B274" t="s">
+        <v>587</v>
+      </c>
+      <c r="C274" t="s">
+        <v>80</v>
+      </c>
+      <c r="D274" t="s">
+        <v>588</v>
+      </c>
+      <c r="E274" t="s">
         <v>589</v>
-      </c>
-      <c r="C274" t="s">
-        <v>80</v>
-      </c>
-      <c r="D274" t="s">
-        <v>98</v>
-      </c>
-      <c r="E274" t="s">
-        <v>99</v>
       </c>
       <c r="F274" s="1">
         <v>46255</v>
@@ -9231,10 +9219,10 @@
         <v>80</v>
       </c>
       <c r="D275" t="s">
-        <v>219</v>
+        <v>98</v>
       </c>
       <c r="E275" t="s">
-        <v>220</v>
+        <v>99</v>
       </c>
       <c r="F275" s="1">
         <v>46255</v>
@@ -9277,10 +9265,10 @@
         <v>80</v>
       </c>
       <c r="D277" t="s">
-        <v>593</v>
+        <v>219</v>
       </c>
       <c r="E277" t="s">
-        <v>594</v>
+        <v>220</v>
       </c>
       <c r="F277" s="1">
         <v>46255</v>
@@ -9294,16 +9282,16 @@
         <v>0</v>
       </c>
       <c r="B278" t="s">
+        <v>593</v>
+      </c>
+      <c r="C278" t="s">
+        <v>80</v>
+      </c>
+      <c r="D278" t="s">
+        <v>594</v>
+      </c>
+      <c r="E278" t="s">
         <v>595</v>
-      </c>
-      <c r="C278" t="s">
-        <v>80</v>
-      </c>
-      <c r="D278" t="s">
-        <v>16</v>
-      </c>
-      <c r="E278" t="s">
-        <v>17</v>
       </c>
       <c r="F278" s="1">
         <v>46255</v>
@@ -9323,10 +9311,10 @@
         <v>80</v>
       </c>
       <c r="D279" t="s">
-        <v>337</v>
+        <v>16</v>
       </c>
       <c r="E279" t="s">
-        <v>338</v>
+        <v>17</v>
       </c>
       <c r="F279" s="1">
         <v>46255</v>
@@ -9346,10 +9334,10 @@
         <v>80</v>
       </c>
       <c r="D280" t="s">
-        <v>435</v>
+        <v>337</v>
       </c>
       <c r="E280" t="s">
-        <v>436</v>
+        <v>338</v>
       </c>
       <c r="F280" s="1">
         <v>46255</v>
@@ -9369,10 +9357,10 @@
         <v>80</v>
       </c>
       <c r="D281" t="s">
-        <v>599</v>
+        <v>435</v>
       </c>
       <c r="E281" t="s">
-        <v>600</v>
+        <v>436</v>
       </c>
       <c r="F281" s="1">
         <v>46255</v>
@@ -9386,16 +9374,16 @@
         <v>0</v>
       </c>
       <c r="B282" t="s">
+        <v>599</v>
+      </c>
+      <c r="C282" t="s">
+        <v>80</v>
+      </c>
+      <c r="D282" t="s">
+        <v>600</v>
+      </c>
+      <c r="E282" t="s">
         <v>601</v>
-      </c>
-      <c r="C282" t="s">
-        <v>80</v>
-      </c>
-      <c r="D282" t="s">
-        <v>599</v>
-      </c>
-      <c r="E282" t="s">
-        <v>600</v>
       </c>
       <c r="F282" s="1">
         <v>46255</v>
@@ -9415,10 +9403,10 @@
         <v>80</v>
       </c>
       <c r="D283" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E283" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="F283" s="1">
         <v>46255</v>
@@ -9432,16 +9420,16 @@
         <v>0</v>
       </c>
       <c r="B284" t="s">
+        <v>603</v>
+      </c>
+      <c r="C284" t="s">
+        <v>80</v>
+      </c>
+      <c r="D284" t="s">
+        <v>604</v>
+      </c>
+      <c r="E284" t="s">
         <v>605</v>
-      </c>
-      <c r="C284" t="s">
-        <v>80</v>
-      </c>
-      <c r="D284" t="s">
-        <v>422</v>
-      </c>
-      <c r="E284" t="s">
-        <v>423</v>
       </c>
       <c r="F284" s="1">
         <v>46255</v>
@@ -9484,10 +9472,10 @@
         <v>80</v>
       </c>
       <c r="D286" t="s">
-        <v>367</v>
+        <v>422</v>
       </c>
       <c r="E286" t="s">
-        <v>368</v>
+        <v>423</v>
       </c>
       <c r="F286" s="1">
         <v>46255</v>
@@ -9530,10 +9518,10 @@
         <v>80</v>
       </c>
       <c r="D288" t="s">
-        <v>610</v>
+        <v>367</v>
       </c>
       <c r="E288" t="s">
-        <v>611</v>
+        <v>368</v>
       </c>
       <c r="F288" s="1">
         <v>46255</v>
@@ -9547,16 +9535,16 @@
         <v>0</v>
       </c>
       <c r="B289" t="s">
+        <v>610</v>
+      </c>
+      <c r="C289" t="s">
+        <v>80</v>
+      </c>
+      <c r="D289" t="s">
+        <v>611</v>
+      </c>
+      <c r="E289" t="s">
         <v>612</v>
-      </c>
-      <c r="C289" t="s">
-        <v>80</v>
-      </c>
-      <c r="D289" t="s">
-        <v>429</v>
-      </c>
-      <c r="E289" t="s">
-        <v>430</v>
       </c>
       <c r="F289" s="1">
         <v>46255</v>
@@ -9599,10 +9587,10 @@
         <v>80</v>
       </c>
       <c r="D291" t="s">
-        <v>348</v>
+        <v>429</v>
       </c>
       <c r="E291" t="s">
-        <v>349</v>
+        <v>430</v>
       </c>
       <c r="F291" s="1">
         <v>46255</v>
@@ -9622,10 +9610,10 @@
         <v>80</v>
       </c>
       <c r="D292" t="s">
-        <v>616</v>
+        <v>348</v>
       </c>
       <c r="E292" t="s">
-        <v>617</v>
+        <v>349</v>
       </c>
       <c r="F292" s="1">
         <v>46255</v>
@@ -9639,16 +9627,16 @@
         <v>0</v>
       </c>
       <c r="B293" t="s">
+        <v>616</v>
+      </c>
+      <c r="C293" t="s">
+        <v>80</v>
+      </c>
+      <c r="D293" t="s">
+        <v>617</v>
+      </c>
+      <c r="E293" t="s">
         <v>618</v>
-      </c>
-      <c r="C293" t="s">
-        <v>80</v>
-      </c>
-      <c r="D293" t="s">
-        <v>7</v>
-      </c>
-      <c r="E293" t="s">
-        <v>8</v>
       </c>
       <c r="F293" s="1">
         <v>46255</v>
@@ -9668,10 +9656,10 @@
         <v>80</v>
       </c>
       <c r="D294" t="s">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="E294" t="s">
-        <v>102</v>
+        <v>8</v>
       </c>
       <c r="F294" s="1">
         <v>46255</v>
@@ -9691,10 +9679,10 @@
         <v>80</v>
       </c>
       <c r="D295" t="s">
-        <v>381</v>
+        <v>101</v>
       </c>
       <c r="E295" t="s">
-        <v>382</v>
+        <v>102</v>
       </c>
       <c r="F295" s="1">
         <v>46255</v>
@@ -9714,10 +9702,10 @@
         <v>80</v>
       </c>
       <c r="D296" t="s">
-        <v>599</v>
+        <v>381</v>
       </c>
       <c r="E296" t="s">
-        <v>600</v>
+        <v>382</v>
       </c>
       <c r="F296" s="1">
         <v>46255</v>
@@ -9737,10 +9725,10 @@
         <v>80</v>
       </c>
       <c r="D297" t="s">
-        <v>381</v>
+        <v>600</v>
       </c>
       <c r="E297" t="s">
-        <v>382</v>
+        <v>601</v>
       </c>
       <c r="F297" s="1">
         <v>46255</v>
@@ -9760,10 +9748,10 @@
         <v>80</v>
       </c>
       <c r="D298" t="s">
-        <v>624</v>
+        <v>381</v>
       </c>
       <c r="E298" t="s">
-        <v>625</v>
+        <v>382</v>
       </c>
       <c r="F298" s="1">
         <v>46255</v>
@@ -9777,16 +9765,16 @@
         <v>0</v>
       </c>
       <c r="B299" t="s">
+        <v>624</v>
+      </c>
+      <c r="C299" t="s">
+        <v>80</v>
+      </c>
+      <c r="D299" t="s">
+        <v>625</v>
+      </c>
+      <c r="E299" t="s">
         <v>626</v>
-      </c>
-      <c r="C299" t="s">
-        <v>80</v>
-      </c>
-      <c r="D299" t="s">
-        <v>224</v>
-      </c>
-      <c r="E299" t="s">
-        <v>225</v>
       </c>
       <c r="F299" s="1">
         <v>46255</v>
@@ -9806,10 +9794,10 @@
         <v>80</v>
       </c>
       <c r="D300" t="s">
-        <v>74</v>
+        <v>224</v>
       </c>
       <c r="E300" t="s">
-        <v>75</v>
+        <v>225</v>
       </c>
       <c r="F300" s="1">
         <v>46255</v>
@@ -9829,10 +9817,10 @@
         <v>80</v>
       </c>
       <c r="D301" t="s">
-        <v>629</v>
+        <v>74</v>
       </c>
       <c r="E301" t="s">
-        <v>630</v>
+        <v>75</v>
       </c>
       <c r="F301" s="1">
         <v>46255</v>
@@ -9846,16 +9834,16 @@
         <v>0</v>
       </c>
       <c r="B302" t="s">
+        <v>629</v>
+      </c>
+      <c r="C302" t="s">
+        <v>80</v>
+      </c>
+      <c r="D302" t="s">
+        <v>630</v>
+      </c>
+      <c r="E302" t="s">
         <v>631</v>
-      </c>
-      <c r="C302" t="s">
-        <v>80</v>
-      </c>
-      <c r="D302" t="s">
-        <v>632</v>
-      </c>
-      <c r="E302" t="s">
-        <v>633</v>
       </c>
       <c r="F302" s="1">
         <v>46255</v>
@@ -9869,16 +9857,16 @@
         <v>0</v>
       </c>
       <c r="B303" t="s">
+        <v>632</v>
+      </c>
+      <c r="C303" t="s">
+        <v>80</v>
+      </c>
+      <c r="D303" t="s">
+        <v>633</v>
+      </c>
+      <c r="E303" t="s">
         <v>634</v>
-      </c>
-      <c r="C303" t="s">
-        <v>80</v>
-      </c>
-      <c r="D303" t="s">
-        <v>373</v>
-      </c>
-      <c r="E303" t="s">
-        <v>374</v>
       </c>
       <c r="F303" s="1">
         <v>46255</v>
@@ -9898,10 +9886,10 @@
         <v>80</v>
       </c>
       <c r="D304" t="s">
-        <v>48</v>
+        <v>373</v>
       </c>
       <c r="E304" t="s">
-        <v>49</v>
+        <v>374</v>
       </c>
       <c r="F304" s="1">
         <v>46255</v>
@@ -9921,10 +9909,10 @@
         <v>80</v>
       </c>
       <c r="D305" t="s">
-        <v>373</v>
+        <v>48</v>
       </c>
       <c r="E305" t="s">
-        <v>374</v>
+        <v>49</v>
       </c>
       <c r="F305" s="1">
         <v>46255</v>
@@ -9944,10 +9932,10 @@
         <v>80</v>
       </c>
       <c r="D306" t="s">
-        <v>638</v>
+        <v>373</v>
       </c>
       <c r="E306" t="s">
-        <v>639</v>
+        <v>374</v>
       </c>
       <c r="F306" s="1">
         <v>46255</v>
@@ -9961,16 +9949,16 @@
         <v>0</v>
       </c>
       <c r="B307" t="s">
+        <v>638</v>
+      </c>
+      <c r="C307" t="s">
+        <v>80</v>
+      </c>
+      <c r="D307" t="s">
+        <v>639</v>
+      </c>
+      <c r="E307" t="s">
         <v>640</v>
-      </c>
-      <c r="C307" t="s">
-        <v>80</v>
-      </c>
-      <c r="D307" t="s">
-        <v>638</v>
-      </c>
-      <c r="E307" t="s">
-        <v>639</v>
       </c>
       <c r="F307" s="1">
         <v>46255</v>
@@ -9990,10 +9978,10 @@
         <v>80</v>
       </c>
       <c r="D308" t="s">
-        <v>373</v>
+        <v>639</v>
       </c>
       <c r="E308" t="s">
-        <v>374</v>
+        <v>640</v>
       </c>
       <c r="F308" s="1">
         <v>46255</v>
@@ -10013,10 +10001,10 @@
         <v>80</v>
       </c>
       <c r="D309" t="s">
-        <v>643</v>
+        <v>373</v>
       </c>
       <c r="E309" t="s">
-        <v>644</v>
+        <v>374</v>
       </c>
       <c r="F309" s="1">
         <v>46255</v>
@@ -10030,16 +10018,16 @@
         <v>0</v>
       </c>
       <c r="B310" t="s">
+        <v>643</v>
+      </c>
+      <c r="C310" t="s">
+        <v>80</v>
+      </c>
+      <c r="D310" t="s">
+        <v>644</v>
+      </c>
+      <c r="E310" t="s">
         <v>645</v>
-      </c>
-      <c r="C310" t="s">
-        <v>80</v>
-      </c>
-      <c r="D310" t="s">
-        <v>646</v>
-      </c>
-      <c r="E310" t="s">
-        <v>647</v>
       </c>
       <c r="F310" s="1">
         <v>46255</v>
@@ -10053,16 +10041,16 @@
         <v>0</v>
       </c>
       <c r="B311" t="s">
+        <v>646</v>
+      </c>
+      <c r="C311" t="s">
+        <v>80</v>
+      </c>
+      <c r="D311" t="s">
+        <v>647</v>
+      </c>
+      <c r="E311" t="s">
         <v>648</v>
-      </c>
-      <c r="C311" t="s">
-        <v>80</v>
-      </c>
-      <c r="D311" t="s">
-        <v>101</v>
-      </c>
-      <c r="E311" t="s">
-        <v>102</v>
       </c>
       <c r="F311" s="1">
         <v>46255</v>
@@ -10082,10 +10070,10 @@
         <v>80</v>
       </c>
       <c r="D312" t="s">
-        <v>147</v>
+        <v>101</v>
       </c>
       <c r="E312" t="s">
-        <v>148</v>
+        <v>102</v>
       </c>
       <c r="F312" s="1">
         <v>46255</v>
@@ -10105,10 +10093,10 @@
         <v>80</v>
       </c>
       <c r="D313" t="s">
-        <v>355</v>
+        <v>147</v>
       </c>
       <c r="E313" t="s">
-        <v>356</v>
+        <v>148</v>
       </c>
       <c r="F313" s="1">
         <v>46255</v>
@@ -10128,10 +10116,10 @@
         <v>80</v>
       </c>
       <c r="D314" t="s">
-        <v>652</v>
+        <v>355</v>
       </c>
       <c r="E314" t="s">
-        <v>653</v>
+        <v>356</v>
       </c>
       <c r="F314" s="1">
         <v>46255</v>
@@ -10145,16 +10133,16 @@
         <v>0</v>
       </c>
       <c r="B315" t="s">
+        <v>652</v>
+      </c>
+      <c r="C315" t="s">
+        <v>80</v>
+      </c>
+      <c r="D315" t="s">
+        <v>653</v>
+      </c>
+      <c r="E315" t="s">
         <v>654</v>
-      </c>
-      <c r="C315" t="s">
-        <v>80</v>
-      </c>
-      <c r="D315" t="s">
-        <v>138</v>
-      </c>
-      <c r="E315" t="s">
-        <v>139</v>
       </c>
       <c r="F315" s="1">
         <v>46255</v>
@@ -10174,10 +10162,10 @@
         <v>80</v>
       </c>
       <c r="D316" t="s">
-        <v>652</v>
+        <v>138</v>
       </c>
       <c r="E316" t="s">
-        <v>653</v>
+        <v>139</v>
       </c>
       <c r="F316" s="1">
         <v>46255</v>
@@ -10197,10 +10185,10 @@
         <v>80</v>
       </c>
       <c r="D317" t="s">
-        <v>355</v>
+        <v>653</v>
       </c>
       <c r="E317" t="s">
-        <v>356</v>
+        <v>654</v>
       </c>
       <c r="F317" s="1">
         <v>46255</v>
@@ -10220,10 +10208,10 @@
         <v>80</v>
       </c>
       <c r="D318" t="s">
-        <v>658</v>
+        <v>355</v>
       </c>
       <c r="E318" t="s">
-        <v>659</v>
+        <v>356</v>
       </c>
       <c r="F318" s="1">
         <v>46255</v>
@@ -10237,16 +10225,16 @@
         <v>0</v>
       </c>
       <c r="B319" t="s">
+        <v>658</v>
+      </c>
+      <c r="C319" t="s">
+        <v>80</v>
+      </c>
+      <c r="D319" t="s">
+        <v>659</v>
+      </c>
+      <c r="E319" t="s">
         <v>660</v>
-      </c>
-      <c r="C319" t="s">
-        <v>80</v>
-      </c>
-      <c r="D319" t="s">
-        <v>661</v>
-      </c>
-      <c r="E319" t="s">
-        <v>662</v>
       </c>
       <c r="F319" s="1">
         <v>46255</v>
@@ -10260,16 +10248,16 @@
         <v>0</v>
       </c>
       <c r="B320" t="s">
+        <v>661</v>
+      </c>
+      <c r="C320" t="s">
+        <v>80</v>
+      </c>
+      <c r="D320" t="s">
+        <v>662</v>
+      </c>
+      <c r="E320" t="s">
         <v>663</v>
-      </c>
-      <c r="C320" t="s">
-        <v>80</v>
-      </c>
-      <c r="D320" t="s">
-        <v>181</v>
-      </c>
-      <c r="E320" t="s">
-        <v>182</v>
       </c>
       <c r="F320" s="1">
         <v>46255</v>
@@ -10289,10 +10277,10 @@
         <v>80</v>
       </c>
       <c r="D321" t="s">
-        <v>665</v>
+        <v>181</v>
       </c>
       <c r="E321" t="s">
-        <v>666</v>
+        <v>182</v>
       </c>
       <c r="F321" s="1">
         <v>46255</v>
@@ -10306,22 +10294,22 @@
         <v>0</v>
       </c>
       <c r="B322" t="s">
+        <v>665</v>
+      </c>
+      <c r="C322" t="s">
+        <v>80</v>
+      </c>
+      <c r="D322" t="s">
+        <v>666</v>
+      </c>
+      <c r="E322" t="s">
         <v>667</v>
       </c>
-      <c r="C322" t="s">
-        <v>80</v>
-      </c>
-      <c r="D322" t="s">
-        <v>668</v>
-      </c>
-      <c r="E322" t="s">
-        <v>669</v>
-      </c>
       <c r="F322" s="1">
         <v>46255</v>
       </c>
       <c r="G322" s="1">
-        <v>46255</v>
+        <v>46256</v>
       </c>
     </row>
     <row r="323" spans="1:7" x14ac:dyDescent="0.2">
@@ -10329,16 +10317,16 @@
         <v>0</v>
       </c>
       <c r="B323" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="C323" t="s">
         <v>80</v>
       </c>
       <c r="D323" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
       <c r="E323" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="F323" s="1">
         <v>46255</v>
@@ -10352,16 +10340,16 @@
         <v>0</v>
       </c>
       <c r="B324" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="C324" t="s">
         <v>80</v>
       </c>
       <c r="D324" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="E324" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="F324" s="1">
         <v>46255</v>
@@ -10375,16 +10363,16 @@
         <v>0</v>
       </c>
       <c r="B325" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="C325" t="s">
         <v>80</v>
       </c>
       <c r="D325" t="s">
-        <v>337</v>
+        <v>673</v>
       </c>
       <c r="E325" t="s">
-        <v>338</v>
+        <v>674</v>
       </c>
       <c r="F325" s="1">
         <v>46255</v>
@@ -10398,16 +10386,16 @@
         <v>0</v>
       </c>
       <c r="B326" t="s">
+        <v>675</v>
+      </c>
+      <c r="C326" t="s">
+        <v>80</v>
+      </c>
+      <c r="D326" t="s">
+        <v>676</v>
+      </c>
+      <c r="E326" t="s">
         <v>677</v>
-      </c>
-      <c r="C326" t="s">
-        <v>80</v>
-      </c>
-      <c r="D326" t="s">
-        <v>678</v>
-      </c>
-      <c r="E326" t="s">
-        <v>679</v>
       </c>
       <c r="F326" s="1">
         <v>46255</v>
@@ -10421,16 +10409,16 @@
         <v>0</v>
       </c>
       <c r="B327" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C327" t="s">
         <v>80</v>
       </c>
       <c r="D327" t="s">
-        <v>678</v>
+        <v>337</v>
       </c>
       <c r="E327" t="s">
-        <v>679</v>
+        <v>338</v>
       </c>
       <c r="F327" s="1">
         <v>46255</v>
@@ -10444,16 +10432,16 @@
         <v>0</v>
       </c>
       <c r="B328" t="s">
+        <v>679</v>
+      </c>
+      <c r="C328" t="s">
+        <v>80</v>
+      </c>
+      <c r="D328" t="s">
+        <v>680</v>
+      </c>
+      <c r="E328" t="s">
         <v>681</v>
-      </c>
-      <c r="C328" t="s">
-        <v>80</v>
-      </c>
-      <c r="D328" t="s">
-        <v>682</v>
-      </c>
-      <c r="E328" t="s">
-        <v>683</v>
       </c>
       <c r="F328" s="1">
         <v>46255</v>
@@ -10467,16 +10455,16 @@
         <v>0</v>
       </c>
       <c r="B329" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C329" t="s">
         <v>80</v>
       </c>
       <c r="D329" t="s">
-        <v>685</v>
+        <v>680</v>
       </c>
       <c r="E329" t="s">
-        <v>686</v>
+        <v>681</v>
       </c>
       <c r="F329" s="1">
         <v>46255</v>
@@ -10490,16 +10478,16 @@
         <v>0</v>
       </c>
       <c r="B330" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="C330" t="s">
         <v>80</v>
       </c>
       <c r="D330" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
       <c r="E330" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="F330" s="1">
         <v>46255</v>
@@ -10513,16 +10501,16 @@
         <v>0</v>
       </c>
       <c r="B331" t="s">
-        <v>690</v>
+        <v>686</v>
       </c>
       <c r="C331" t="s">
         <v>80</v>
       </c>
       <c r="D331" t="s">
-        <v>138</v>
+        <v>687</v>
       </c>
       <c r="E331" t="s">
-        <v>139</v>
+        <v>688</v>
       </c>
       <c r="F331" s="1">
         <v>46255</v>
@@ -10536,16 +10524,16 @@
         <v>0</v>
       </c>
       <c r="B332" t="s">
+        <v>689</v>
+      </c>
+      <c r="C332" t="s">
+        <v>80</v>
+      </c>
+      <c r="D332" t="s">
+        <v>690</v>
+      </c>
+      <c r="E332" t="s">
         <v>691</v>
-      </c>
-      <c r="C332" t="s">
-        <v>80</v>
-      </c>
-      <c r="D332" t="s">
-        <v>98</v>
-      </c>
-      <c r="E332" t="s">
-        <v>99</v>
       </c>
       <c r="F332" s="1">
         <v>46255</v>
@@ -10565,10 +10553,10 @@
         <v>80</v>
       </c>
       <c r="D333" t="s">
-        <v>593</v>
+        <v>138</v>
       </c>
       <c r="E333" t="s">
-        <v>594</v>
+        <v>139</v>
       </c>
       <c r="F333" s="1">
         <v>46255</v>
@@ -10588,10 +10576,10 @@
         <v>80</v>
       </c>
       <c r="D334" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="E334" t="s">
-        <v>26</v>
+        <v>99</v>
       </c>
       <c r="F334" s="1">
         <v>46255</v>
@@ -10611,10 +10599,10 @@
         <v>80</v>
       </c>
       <c r="D335" t="s">
-        <v>37</v>
+        <v>594</v>
       </c>
       <c r="E335" t="s">
-        <v>38</v>
+        <v>595</v>
       </c>
       <c r="F335" s="1">
         <v>46255</v>
@@ -10634,10 +10622,10 @@
         <v>80</v>
       </c>
       <c r="D336" t="s">
-        <v>351</v>
+        <v>25</v>
       </c>
       <c r="E336" t="s">
-        <v>352</v>
+        <v>26</v>
       </c>
       <c r="F336" s="1">
         <v>46255</v>
@@ -10657,10 +10645,10 @@
         <v>80</v>
       </c>
       <c r="D337" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="E337" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="F337" s="1">
         <v>46255</v>
@@ -10680,10 +10668,10 @@
         <v>80</v>
       </c>
       <c r="D338" t="s">
-        <v>698</v>
+        <v>351</v>
       </c>
       <c r="E338" t="s">
-        <v>699</v>
+        <v>352</v>
       </c>
       <c r="F338" s="1">
         <v>46255</v>
@@ -10697,16 +10685,16 @@
         <v>0</v>
       </c>
       <c r="B339" t="s">
+        <v>698</v>
+      </c>
+      <c r="C339" t="s">
+        <v>80</v>
+      </c>
+      <c r="D339" t="s">
+        <v>699</v>
+      </c>
+      <c r="E339" t="s">
         <v>700</v>
-      </c>
-      <c r="C339" t="s">
-        <v>80</v>
-      </c>
-      <c r="D339" t="s">
-        <v>701</v>
-      </c>
-      <c r="E339" t="s">
-        <v>702</v>
       </c>
       <c r="F339" s="1">
         <v>46255</v>
@@ -10720,16 +10708,16 @@
         <v>0</v>
       </c>
       <c r="B340" t="s">
+        <v>701</v>
+      </c>
+      <c r="C340" t="s">
+        <v>80</v>
+      </c>
+      <c r="D340" t="s">
+        <v>702</v>
+      </c>
+      <c r="E340" t="s">
         <v>703</v>
-      </c>
-      <c r="C340" t="s">
-        <v>80</v>
-      </c>
-      <c r="D340" t="s">
-        <v>400</v>
-      </c>
-      <c r="E340" t="s">
-        <v>401</v>
       </c>
       <c r="F340" s="1">
         <v>46255</v>
@@ -10749,10 +10737,10 @@
         <v>80</v>
       </c>
       <c r="D341" t="s">
-        <v>705</v>
+        <v>400</v>
       </c>
       <c r="E341" t="s">
-        <v>706</v>
+        <v>401</v>
       </c>
       <c r="F341" s="1">
         <v>46255</v>
@@ -10766,16 +10754,16 @@
         <v>0</v>
       </c>
       <c r="B342" t="s">
+        <v>705</v>
+      </c>
+      <c r="C342" t="s">
+        <v>80</v>
+      </c>
+      <c r="D342" t="s">
+        <v>706</v>
+      </c>
+      <c r="E342" t="s">
         <v>707</v>
-      </c>
-      <c r="C342" t="s">
-        <v>80</v>
-      </c>
-      <c r="D342" t="s">
-        <v>526</v>
-      </c>
-      <c r="E342" t="s">
-        <v>527</v>
       </c>
       <c r="F342" s="1">
         <v>46255</v>
@@ -10795,10 +10783,10 @@
         <v>80</v>
       </c>
       <c r="D343" t="s">
-        <v>709</v>
+        <v>526</v>
       </c>
       <c r="E343" t="s">
-        <v>710</v>
+        <v>527</v>
       </c>
       <c r="F343" s="1">
         <v>46255</v>
@@ -10812,16 +10800,16 @@
         <v>0</v>
       </c>
       <c r="B344" t="s">
+        <v>709</v>
+      </c>
+      <c r="C344" t="s">
+        <v>80</v>
+      </c>
+      <c r="D344" t="s">
+        <v>710</v>
+      </c>
+      <c r="E344" t="s">
         <v>711</v>
-      </c>
-      <c r="C344" t="s">
-        <v>80</v>
-      </c>
-      <c r="D344" t="s">
-        <v>403</v>
-      </c>
-      <c r="E344" t="s">
-        <v>404</v>
       </c>
       <c r="F344" s="1">
         <v>46255</v>
@@ -10841,10 +10829,10 @@
         <v>80</v>
       </c>
       <c r="D345" t="s">
-        <v>713</v>
+        <v>403</v>
       </c>
       <c r="E345" t="s">
-        <v>714</v>
+        <v>404</v>
       </c>
       <c r="F345" s="1">
         <v>46255</v>
@@ -10858,16 +10846,16 @@
         <v>0</v>
       </c>
       <c r="B346" t="s">
+        <v>713</v>
+      </c>
+      <c r="C346" t="s">
+        <v>80</v>
+      </c>
+      <c r="D346" t="s">
+        <v>714</v>
+      </c>
+      <c r="E346" t="s">
         <v>715</v>
-      </c>
-      <c r="C346" t="s">
-        <v>80</v>
-      </c>
-      <c r="D346" t="s">
-        <v>16</v>
-      </c>
-      <c r="E346" t="s">
-        <v>17</v>
       </c>
       <c r="F346" s="1">
         <v>46255</v>
@@ -10878,53 +10866,53 @@
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
+        <v>0</v>
+      </c>
+      <c r="B347" t="s">
         <v>716</v>
       </c>
-      <c r="B347" t="s">
-        <v>717</v>
-      </c>
       <c r="C347" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D347" t="s">
-        <v>348</v>
+        <v>16</v>
       </c>
       <c r="E347" t="s">
-        <v>349</v>
+        <v>17</v>
       </c>
       <c r="F347" s="1">
-        <v>46148</v>
+        <v>46255</v>
       </c>
       <c r="G347" s="1">
-        <v>46149</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="348" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
+        <v>717</v>
+      </c>
+      <c r="B348" t="s">
         <v>718</v>
       </c>
-      <c r="B348" t="s">
-        <v>719</v>
-      </c>
       <c r="C348" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D348" t="s">
-        <v>41</v>
+        <v>348</v>
       </c>
       <c r="E348" t="s">
-        <v>42</v>
+        <v>349</v>
       </c>
       <c r="F348" s="1">
-        <v>46133</v>
+        <v>46148</v>
       </c>
       <c r="G348" s="1">
-        <v>46134</v>
+        <v>46149</v>
       </c>
     </row>
     <row r="349" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B349" t="s">
         <v>720</v>
@@ -10939,7 +10927,7 @@
         <v>42</v>
       </c>
       <c r="F349" s="1">
-        <v>46134</v>
+        <v>46133</v>
       </c>
       <c r="G349" s="1">
         <v>46134</v>
@@ -10947,7 +10935,7 @@
     </row>
     <row r="350" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B350" t="s">
         <v>721</v>
@@ -10956,159 +10944,159 @@
         <v>6</v>
       </c>
       <c r="D350" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E350" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="F350" s="1">
-        <v>46156</v>
+        <v>46134</v>
       </c>
       <c r="G350" s="1">
-        <v>46156</v>
+        <v>46134</v>
       </c>
     </row>
     <row r="351" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B351" t="s">
         <v>722</v>
       </c>
       <c r="C351" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D351" t="s">
-        <v>723</v>
+        <v>19</v>
       </c>
       <c r="E351" t="s">
-        <v>724</v>
+        <v>20</v>
       </c>
       <c r="F351" s="1">
-        <v>46195</v>
+        <v>46156</v>
       </c>
       <c r="G351" s="1">
-        <v>46195</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="352" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B352" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C352" t="s">
         <v>2</v>
       </c>
       <c r="D352" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="E352" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="F352" s="1">
-        <v>46206</v>
+        <v>46195</v>
       </c>
       <c r="G352" s="1">
-        <v>46252</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="353" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B353" t="s">
+        <v>726</v>
+      </c>
+      <c r="C353" t="s">
+        <v>2</v>
+      </c>
+      <c r="D353" t="s">
+        <v>727</v>
+      </c>
+      <c r="E353" t="s">
         <v>728</v>
       </c>
-      <c r="C353" t="s">
-        <v>96</v>
-      </c>
-      <c r="D353" t="s">
-        <v>729</v>
-      </c>
-      <c r="E353" t="s">
-        <v>730</v>
-      </c>
       <c r="F353" s="1">
-        <v>46209</v>
+        <v>46206</v>
       </c>
       <c r="G353" s="1">
-        <v>46218</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="354" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B354" t="s">
+        <v>729</v>
+      </c>
+      <c r="C354" t="s">
+        <v>96</v>
+      </c>
+      <c r="D354" t="s">
+        <v>730</v>
+      </c>
+      <c r="E354" t="s">
         <v>731</v>
       </c>
-      <c r="C354" t="s">
-        <v>6</v>
-      </c>
-      <c r="D354" t="s">
-        <v>732</v>
-      </c>
-      <c r="E354" t="s">
-        <v>733</v>
-      </c>
       <c r="F354" s="1">
-        <v>46213</v>
+        <v>46209</v>
       </c>
       <c r="G354" s="1">
-        <v>46213</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="355" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B355" t="s">
+        <v>732</v>
+      </c>
+      <c r="C355" t="s">
+        <v>6</v>
+      </c>
+      <c r="D355" t="s">
+        <v>733</v>
+      </c>
+      <c r="E355" t="s">
         <v>734</v>
-      </c>
-      <c r="C355" t="s">
-        <v>96</v>
-      </c>
-      <c r="D355" t="s">
-        <v>735</v>
-      </c>
-      <c r="E355" t="s">
-        <v>736</v>
       </c>
       <c r="F355" s="1">
         <v>46213</v>
       </c>
       <c r="G355" s="1">
-        <v>46216</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B356" t="s">
+        <v>735</v>
+      </c>
+      <c r="C356" t="s">
+        <v>96</v>
+      </c>
+      <c r="D356" t="s">
+        <v>736</v>
+      </c>
+      <c r="E356" t="s">
         <v>737</v>
       </c>
-      <c r="C356" t="s">
-        <v>2</v>
-      </c>
-      <c r="D356" t="s">
-        <v>133</v>
-      </c>
-      <c r="E356" t="s">
-        <v>134</v>
-      </c>
       <c r="F356" s="1">
-        <v>46220</v>
+        <v>46213</v>
       </c>
       <c r="G356" s="1">
-        <v>46231</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="357" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B357" t="s">
         <v>738</v>
@@ -11117,67 +11105,67 @@
         <v>2</v>
       </c>
       <c r="D357" t="s">
-        <v>723</v>
+        <v>133</v>
       </c>
       <c r="E357" t="s">
-        <v>724</v>
+        <v>134</v>
       </c>
       <c r="F357" s="1">
-        <v>46223</v>
+        <v>46220</v>
       </c>
       <c r="G357" s="1">
-        <v>46223</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="358" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B358" t="s">
         <v>739</v>
       </c>
       <c r="C358" t="s">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D358" t="s">
-        <v>735</v>
+        <v>724</v>
       </c>
       <c r="E358" t="s">
-        <v>736</v>
+        <v>725</v>
       </c>
       <c r="F358" s="1">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="G358" s="1">
-        <v>46224</v>
+        <v>46223</v>
       </c>
     </row>
     <row r="359" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B359" t="s">
         <v>740</v>
       </c>
       <c r="C359" t="s">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="D359" t="s">
-        <v>723</v>
+        <v>736</v>
       </c>
       <c r="E359" t="s">
-        <v>724</v>
+        <v>737</v>
       </c>
       <c r="F359" s="1">
-        <v>46230</v>
+        <v>46224</v>
       </c>
       <c r="G359" s="1">
-        <v>46231</v>
+        <v>46224</v>
       </c>
     </row>
     <row r="360" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B360" t="s">
         <v>741</v>
@@ -11186,21 +11174,21 @@
         <v>2</v>
       </c>
       <c r="D360" t="s">
-        <v>133</v>
+        <v>724</v>
       </c>
       <c r="E360" t="s">
-        <v>134</v>
+        <v>725</v>
       </c>
       <c r="F360" s="1">
-        <v>46232</v>
+        <v>46230</v>
       </c>
       <c r="G360" s="1">
-        <v>46233</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="361" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B361" t="s">
         <v>742</v>
@@ -11223,7 +11211,7 @@
     </row>
     <row r="362" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B362" t="s">
         <v>743</v>
@@ -11232,21 +11220,21 @@
         <v>2</v>
       </c>
       <c r="D362" t="s">
-        <v>735</v>
+        <v>133</v>
       </c>
       <c r="E362" t="s">
-        <v>736</v>
+        <v>134</v>
       </c>
       <c r="F362" s="1">
-        <v>46238</v>
+        <v>46232</v>
       </c>
       <c r="G362" s="1">
-        <v>46239</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="363" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B363" t="s">
         <v>744</v>
@@ -11255,82 +11243,82 @@
         <v>2</v>
       </c>
       <c r="D363" t="s">
-        <v>41</v>
+        <v>736</v>
       </c>
       <c r="E363" t="s">
-        <v>42</v>
+        <v>737</v>
       </c>
       <c r="F363" s="1">
-        <v>46247</v>
+        <v>46238</v>
       </c>
       <c r="G363" s="1">
-        <v>46252</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="364" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B364" t="s">
         <v>745</v>
       </c>
       <c r="C364" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D364" t="s">
-        <v>746</v>
+        <v>41</v>
       </c>
       <c r="E364" t="s">
-        <v>747</v>
+        <v>42</v>
       </c>
       <c r="F364" s="1">
-        <v>46253</v>
+        <v>46247</v>
       </c>
       <c r="G364" s="1">
-        <v>46253</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="365" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B365" t="s">
+        <v>746</v>
+      </c>
+      <c r="C365" t="s">
+        <v>6</v>
+      </c>
+      <c r="D365" t="s">
+        <v>747</v>
+      </c>
+      <c r="E365" t="s">
         <v>748</v>
-      </c>
-      <c r="C365" t="s">
-        <v>2</v>
-      </c>
-      <c r="D365" t="s">
-        <v>735</v>
-      </c>
-      <c r="E365" t="s">
-        <v>736</v>
       </c>
       <c r="F365" s="1">
         <v>46253</v>
       </c>
       <c r="G365" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="366" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B366" t="s">
         <v>749</v>
       </c>
       <c r="C366" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D366" t="s">
-        <v>472</v>
+        <v>736</v>
       </c>
       <c r="E366" t="s">
-        <v>473</v>
+        <v>737</v>
       </c>
       <c r="F366" s="1">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G366" s="1">
         <v>46254</v>
@@ -11338,7 +11326,7 @@
     </row>
     <row r="367" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B367" t="s">
         <v>750</v>
@@ -11347,21 +11335,21 @@
         <v>80</v>
       </c>
       <c r="D367" t="s">
-        <v>735</v>
+        <v>472</v>
       </c>
       <c r="E367" t="s">
-        <v>736</v>
+        <v>473</v>
       </c>
       <c r="F367" s="1">
         <v>46254</v>
       </c>
       <c r="G367" s="1">
-        <v>46255</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="368" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B368" t="s">
         <v>751</v>
@@ -11370,10 +11358,10 @@
         <v>80</v>
       </c>
       <c r="D368" t="s">
-        <v>138</v>
+        <v>736</v>
       </c>
       <c r="E368" t="s">
-        <v>139</v>
+        <v>737</v>
       </c>
       <c r="F368" s="1">
         <v>46254</v>
@@ -11384,7 +11372,7 @@
     </row>
     <row r="369" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B369" t="s">
         <v>752</v>
@@ -11407,7 +11395,7 @@
     </row>
     <row r="370" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B370" t="s">
         <v>753</v>
@@ -11416,10 +11404,10 @@
         <v>80</v>
       </c>
       <c r="D370" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E370" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F370" s="1">
         <v>46254</v>
@@ -11430,7 +11418,7 @@
     </row>
     <row r="371" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B371" t="s">
         <v>754</v>
@@ -11439,10 +11427,10 @@
         <v>80</v>
       </c>
       <c r="D371" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="E371" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="F371" s="1">
         <v>46254</v>
@@ -11453,7 +11441,7 @@
     </row>
     <row r="372" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B372" t="s">
         <v>755</v>
@@ -11476,7 +11464,7 @@
     </row>
     <row r="373" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B373" t="s">
         <v>756</v>
@@ -11499,7 +11487,7 @@
     </row>
     <row r="374" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B374" t="s">
         <v>757</v>
@@ -11508,10 +11496,10 @@
         <v>80</v>
       </c>
       <c r="D374" t="s">
-        <v>156</v>
+        <v>571</v>
       </c>
       <c r="E374" t="s">
-        <v>157</v>
+        <v>572</v>
       </c>
       <c r="F374" s="1">
         <v>46254</v>
@@ -11522,7 +11510,7 @@
     </row>
     <row r="375" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B375" t="s">
         <v>758</v>
@@ -11545,7 +11533,7 @@
     </row>
     <row r="376" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B376" t="s">
         <v>759</v>
@@ -11554,13 +11542,13 @@
         <v>80</v>
       </c>
       <c r="D376" t="s">
-        <v>571</v>
+        <v>373</v>
       </c>
       <c r="E376" t="s">
-        <v>572</v>
+        <v>374</v>
       </c>
       <c r="F376" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="G376" s="1">
         <v>46255</v>
@@ -11568,7 +11556,7 @@
     </row>
     <row r="377" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B377" t="s">
         <v>760</v>
@@ -11591,7 +11579,7 @@
     </row>
     <row r="378" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A378" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B378" t="s">
         <v>761</v>
@@ -11600,10 +11588,10 @@
         <v>80</v>
       </c>
       <c r="D378" t="s">
-        <v>373</v>
+        <v>762</v>
       </c>
       <c r="E378" t="s">
-        <v>374</v>
+        <v>763</v>
       </c>
       <c r="F378" s="1">
         <v>46255</v>
@@ -11614,82 +11602,82 @@
     </row>
     <row r="379" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
-        <v>718</v>
+        <v>764</v>
       </c>
       <c r="B379" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="C379" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D379" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="E379" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="F379" s="1">
-        <v>46255</v>
+        <v>46063</v>
       </c>
       <c r="G379" s="1">
-        <v>46255</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="380" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
-        <v>718</v>
+        <v>764</v>
       </c>
       <c r="B380" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C380" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D380" t="s">
-        <v>698</v>
+        <v>57</v>
       </c>
       <c r="E380" t="s">
-        <v>699</v>
+        <v>58</v>
       </c>
       <c r="F380" s="1">
-        <v>46255</v>
+        <v>46113</v>
       </c>
       <c r="G380" s="1">
-        <v>46255</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="381" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B381" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="C381" t="s">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D381" t="s">
-        <v>768</v>
+        <v>57</v>
       </c>
       <c r="E381" t="s">
-        <v>769</v>
+        <v>58</v>
       </c>
       <c r="F381" s="1">
-        <v>46063</v>
+        <v>46125</v>
       </c>
       <c r="G381" s="1">
-        <v>46064</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="382" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B382" t="s">
         <v>770</v>
       </c>
       <c r="C382" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D382" t="s">
         <v>57</v>
@@ -11698,15 +11686,15 @@
         <v>58</v>
       </c>
       <c r="F382" s="1">
-        <v>46113</v>
+        <v>46126</v>
       </c>
       <c r="G382" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="383" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B383" t="s">
         <v>771</v>
@@ -11721,15 +11709,15 @@
         <v>58</v>
       </c>
       <c r="F383" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="G383" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="384" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B384" t="s">
         <v>772</v>
@@ -11744,21 +11732,21 @@
         <v>58</v>
       </c>
       <c r="F384" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="G384" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="385" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B385" t="s">
         <v>773</v>
       </c>
       <c r="C385" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D385" t="s">
         <v>57</v>
@@ -11767,15 +11755,15 @@
         <v>58</v>
       </c>
       <c r="F385" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
       <c r="G385" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="386" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A386" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B386" t="s">
         <v>774</v>
@@ -11790,21 +11778,21 @@
         <v>58</v>
       </c>
       <c r="F386" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
       <c r="G386" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="387" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A387" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B387" t="s">
         <v>775</v>
       </c>
       <c r="C387" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D387" t="s">
         <v>57</v>
@@ -11813,15 +11801,15 @@
         <v>58</v>
       </c>
       <c r="F387" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
       <c r="G387" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="388" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A388" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B388" t="s">
         <v>776</v>
@@ -11836,21 +11824,21 @@
         <v>58</v>
       </c>
       <c r="F388" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="G388" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="389" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A389" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B389" t="s">
         <v>777</v>
       </c>
       <c r="C389" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D389" t="s">
         <v>57</v>
@@ -11859,21 +11847,21 @@
         <v>58</v>
       </c>
       <c r="F389" s="1">
-        <v>46174</v>
+        <v>46195</v>
       </c>
       <c r="G389" s="1">
-        <v>46174</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A390" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B390" t="s">
         <v>778</v>
       </c>
       <c r="C390" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D390" t="s">
         <v>57</v>
@@ -11882,21 +11870,21 @@
         <v>58</v>
       </c>
       <c r="F390" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
       <c r="G390" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A391" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B391" t="s">
         <v>779</v>
       </c>
       <c r="C391" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D391" t="s">
         <v>57</v>
@@ -11905,21 +11893,21 @@
         <v>58</v>
       </c>
       <c r="F391" s="1">
-        <v>46195</v>
+        <v>46213</v>
       </c>
       <c r="G391" s="1">
-        <v>46252</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A392" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B392" t="s">
         <v>780</v>
       </c>
       <c r="C392" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D392" t="s">
         <v>57</v>
@@ -11928,38 +11916,38 @@
         <v>58</v>
       </c>
       <c r="F392" s="1">
-        <v>46210</v>
+        <v>46218</v>
       </c>
       <c r="G392" s="1">
-        <v>46210</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A393" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B393" t="s">
         <v>781</v>
       </c>
       <c r="C393" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D393" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E393" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F393" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
       <c r="G393" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A394" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B394" t="s">
         <v>782</v>
@@ -11974,7 +11962,7 @@
         <v>58</v>
       </c>
       <c r="F394" s="1">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="G394" s="1">
         <v>46252</v>
@@ -11982,36 +11970,36 @@
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A395" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B395" t="s">
         <v>783</v>
       </c>
       <c r="C395" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D395" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E395" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F395" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="G395" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A396" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B396" t="s">
         <v>784</v>
       </c>
       <c r="C396" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D396" t="s">
         <v>57</v>
@@ -12023,12 +12011,12 @@
         <v>46227</v>
       </c>
       <c r="G396" s="1">
-        <v>46252</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A397" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B397" t="s">
         <v>785</v>
@@ -12037,13 +12025,13 @@
         <v>80</v>
       </c>
       <c r="D397" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E397" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F397" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="G397" s="1">
         <v>46252</v>
@@ -12051,7 +12039,7 @@
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A398" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B398" t="s">
         <v>786</v>
@@ -12066,44 +12054,44 @@
         <v>58</v>
       </c>
       <c r="F398" s="1">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="G398" s="1">
-        <v>46228</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B399" t="s">
         <v>787</v>
       </c>
       <c r="C399" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D399" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E399" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F399" s="1">
-        <v>46230</v>
+        <v>46254</v>
       </c>
       <c r="G399" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B400" t="s">
         <v>788</v>
       </c>
       <c r="C400" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D400" t="s">
         <v>57</v>
@@ -12112,110 +12100,110 @@
         <v>58</v>
       </c>
       <c r="F400" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
       <c r="G400" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>766</v>
+        <v>789</v>
       </c>
       <c r="B401" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="C401" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D401" t="s">
-        <v>57</v>
+        <v>791</v>
       </c>
       <c r="E401" t="s">
-        <v>58</v>
+        <v>792</v>
       </c>
       <c r="F401" s="1">
-        <v>46254</v>
+        <v>46083</v>
       </c>
       <c r="G401" s="1">
-        <v>46254</v>
+        <v>46084</v>
       </c>
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
-        <v>766</v>
+        <v>789</v>
       </c>
       <c r="B402" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="C402" t="s">
         <v>2</v>
       </c>
       <c r="D402" t="s">
-        <v>57</v>
+        <v>791</v>
       </c>
       <c r="E402" t="s">
-        <v>58</v>
+        <v>792</v>
       </c>
       <c r="F402" s="1">
-        <v>46255</v>
+        <v>46132</v>
       </c>
       <c r="G402" s="1">
-        <v>46255</v>
+        <v>46133</v>
       </c>
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
-        <v>766</v>
+        <v>789</v>
       </c>
       <c r="B403" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="C403" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D403" t="s">
-        <v>57</v>
+        <v>795</v>
       </c>
       <c r="E403" t="s">
-        <v>58</v>
+        <v>796</v>
       </c>
       <c r="F403" s="1">
-        <v>46255</v>
+        <v>46157</v>
       </c>
       <c r="G403" s="1">
-        <v>46255</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
-        <v>766</v>
+        <v>789</v>
       </c>
       <c r="B404" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
       <c r="C404" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D404" t="s">
-        <v>57</v>
+        <v>798</v>
       </c>
       <c r="E404" t="s">
-        <v>58</v>
+        <v>799</v>
       </c>
       <c r="F404" s="1">
-        <v>46255</v>
+        <v>46168</v>
       </c>
       <c r="G404" s="1">
-        <v>46255</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="B405" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="C405" t="s">
         <v>2</v>
@@ -12227,18 +12215,18 @@
         <v>796</v>
       </c>
       <c r="F405" s="1">
-        <v>46083</v>
+        <v>46244</v>
       </c>
       <c r="G405" s="1">
-        <v>46084</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="B406" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="C406" t="s">
         <v>2</v>
@@ -12250,147 +12238,55 @@
         <v>796</v>
       </c>
       <c r="F406" s="1">
-        <v>46132</v>
+        <v>46247</v>
       </c>
       <c r="G406" s="1">
-        <v>46133</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="B407" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="C407" t="s">
         <v>2</v>
       </c>
       <c r="D407" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="E407" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
       <c r="F407" s="1">
-        <v>46157</v>
+        <v>46247</v>
       </c>
       <c r="G407" s="1">
-        <v>46157</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="B408" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="C408" t="s">
         <v>2</v>
       </c>
       <c r="D408" t="s">
-        <v>802</v>
+        <v>795</v>
       </c>
       <c r="E408" t="s">
-        <v>803</v>
+        <v>796</v>
       </c>
       <c r="F408" s="1">
-        <v>46168</v>
+        <v>46255</v>
       </c>
       <c r="G408" s="1">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="409" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A409" t="s">
-        <v>793</v>
-      </c>
-      <c r="B409" t="s">
-        <v>804</v>
-      </c>
-      <c r="C409" t="s">
-        <v>2</v>
-      </c>
-      <c r="D409" t="s">
-        <v>799</v>
-      </c>
-      <c r="E409" t="s">
-        <v>800</v>
-      </c>
-      <c r="F409" s="1">
-        <v>46244</v>
-      </c>
-      <c r="G409" s="1">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="410" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A410" t="s">
-        <v>793</v>
-      </c>
-      <c r="B410" t="s">
-        <v>805</v>
-      </c>
-      <c r="C410" t="s">
-        <v>2</v>
-      </c>
-      <c r="D410" t="s">
-        <v>799</v>
-      </c>
-      <c r="E410" t="s">
-        <v>800</v>
-      </c>
-      <c r="F410" s="1">
-        <v>46247</v>
-      </c>
-      <c r="G410" s="1">
-        <v>46247</v>
-      </c>
-    </row>
-    <row r="411" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A411" t="s">
-        <v>793</v>
-      </c>
-      <c r="B411" t="s">
-        <v>806</v>
-      </c>
-      <c r="C411" t="s">
-        <v>2</v>
-      </c>
-      <c r="D411" t="s">
-        <v>795</v>
-      </c>
-      <c r="E411" t="s">
-        <v>796</v>
-      </c>
-      <c r="F411" s="1">
-        <v>46247</v>
-      </c>
-      <c r="G411" s="1">
-        <v>46247</v>
-      </c>
-    </row>
-    <row r="412" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A412" t="s">
-        <v>793</v>
-      </c>
-      <c r="B412" t="s">
-        <v>807</v>
-      </c>
-      <c r="C412" t="s">
-        <v>80</v>
-      </c>
-      <c r="D412" t="s">
-        <v>799</v>
-      </c>
-      <c r="E412" t="s">
-        <v>800</v>
-      </c>
-      <c r="F412" s="1">
-        <v>46255</v>
-      </c>
-      <c r="G412" s="1">
         <v>46255</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Transmicion - 31/08/2026 05:59:57
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Transmicion.xlsx
+++ b/Data_ERP/Pedidos Transmicion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFCF6CEA-E211-44D0-9B14-95D9B4A65337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3389E81-2B0A-4D8B-B054-ABD39129DDCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25230" yWindow="4080" windowWidth="15375" windowHeight="8325" xr2:uid="{0387AA51-D7FF-49B4-9616-210EF5E8A02F}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{AC707633-82CA-4A69-8930-E54342FE1B21}"/>
   </bookViews>
   <sheets>
     <sheet name="transmicion" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2152" uniqueCount="795">
   <si>
     <t>0001</t>
   </si>
@@ -2257,21 +2257,9 @@
     <t xml:space="preserve">    2846</t>
   </si>
   <si>
-    <t xml:space="preserve">    2849</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2851</t>
   </si>
   <si>
-    <t xml:space="preserve">    2860</t>
-  </si>
-  <si>
-    <t>MB13</t>
-  </si>
-  <si>
-    <t>MATERIALES BASUALDO S.A.</t>
-  </si>
-  <si>
     <t xml:space="preserve">    2862</t>
   </si>
   <si>
@@ -2354,24 +2342,6 @@
   </si>
   <si>
     <t xml:space="preserve">    2301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2334</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2335</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2336</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2339</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    2340</t>
   </si>
   <si>
     <t>9999</t>
@@ -2884,31 +2854,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{961C53E3-9F57-4010-80CB-BC209C238E0C}">
-  <dimension ref="A1:G438"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2526AF24-EA90-4723-B15F-F71EC0F581FF}">
+  <dimension ref="A1:G430"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>798</v>
+        <v>788</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>799</v>
+        <v>789</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>800</v>
+        <v>790</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>801</v>
+        <v>791</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>802</v>
+        <v>792</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>803</v>
+        <v>793</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>804</v>
+        <v>794</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -7013,7 +6983,7 @@
         <v>381</v>
       </c>
       <c r="C180" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D180" t="s">
         <v>16</v>
@@ -7059,7 +7029,7 @@
         <v>385</v>
       </c>
       <c r="C182" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D182" t="s">
         <v>16</v>
@@ -7151,7 +7121,7 @@
         <v>395</v>
       </c>
       <c r="C186" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D186" t="s">
         <v>16</v>
@@ -7220,7 +7190,7 @@
         <v>398</v>
       </c>
       <c r="C189" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D189" t="s">
         <v>16</v>
@@ -7381,7 +7351,7 @@
         <v>409</v>
       </c>
       <c r="C196" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D196" t="s">
         <v>16</v>
@@ -7473,7 +7443,7 @@
         <v>417</v>
       </c>
       <c r="C200" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D200" t="s">
         <v>16</v>
@@ -7496,7 +7466,7 @@
         <v>418</v>
       </c>
       <c r="C201" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D201" t="s">
         <v>419</v>
@@ -7519,7 +7489,7 @@
         <v>421</v>
       </c>
       <c r="C202" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D202" t="s">
         <v>377</v>
@@ -7588,7 +7558,7 @@
         <v>428</v>
       </c>
       <c r="C205" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D205" t="s">
         <v>171</v>
@@ -7680,7 +7650,7 @@
         <v>436</v>
       </c>
       <c r="C209" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D209" t="s">
         <v>437</v>
@@ -7841,7 +7811,7 @@
         <v>449</v>
       </c>
       <c r="C216" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D216" t="s">
         <v>450</v>
@@ -7910,7 +7880,7 @@
         <v>456</v>
       </c>
       <c r="C219" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D219" t="s">
         <v>450</v>
@@ -7979,7 +7949,7 @@
         <v>463</v>
       </c>
       <c r="C222" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D222" t="s">
         <v>454</v>
@@ -8002,7 +7972,7 @@
         <v>464</v>
       </c>
       <c r="C223" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D223" t="s">
         <v>299</v>
@@ -8048,7 +8018,7 @@
         <v>466</v>
       </c>
       <c r="C225" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D225" t="s">
         <v>467</v>
@@ -8071,7 +8041,7 @@
         <v>469</v>
       </c>
       <c r="C226" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D226" t="s">
         <v>470</v>
@@ -8393,7 +8363,7 @@
         <v>489</v>
       </c>
       <c r="C240" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D240" t="s">
         <v>490</v>
@@ -8485,7 +8455,7 @@
         <v>499</v>
       </c>
       <c r="C244" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D244" t="s">
         <v>419</v>
@@ -8508,7 +8478,7 @@
         <v>500</v>
       </c>
       <c r="C245" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D245" t="s">
         <v>437</v>
@@ -8830,7 +8800,7 @@
         <v>522</v>
       </c>
       <c r="C259" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D259" t="s">
         <v>467</v>
@@ -9014,7 +8984,7 @@
         <v>538</v>
       </c>
       <c r="C267" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D267" t="s">
         <v>536</v>
@@ -9037,7 +9007,7 @@
         <v>539</v>
       </c>
       <c r="C268" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D268" t="s">
         <v>426</v>
@@ -9060,7 +9030,7 @@
         <v>540</v>
       </c>
       <c r="C269" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D269" t="s">
         <v>467</v>
@@ -9083,7 +9053,7 @@
         <v>541</v>
       </c>
       <c r="C270" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D270" t="s">
         <v>16</v>
@@ -9129,7 +9099,7 @@
         <v>543</v>
       </c>
       <c r="C272" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D272" t="s">
         <v>544</v>
@@ -9175,7 +9145,7 @@
         <v>547</v>
       </c>
       <c r="C274" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D274" t="s">
         <v>548</v>
@@ -9198,7 +9168,7 @@
         <v>550</v>
       </c>
       <c r="C275" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D275" t="s">
         <v>551</v>
@@ -9290,7 +9260,7 @@
         <v>556</v>
       </c>
       <c r="C279" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D279" t="s">
         <v>557</v>
@@ -9336,7 +9306,7 @@
         <v>562</v>
       </c>
       <c r="C281" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D281" t="s">
         <v>563</v>
@@ -9842,7 +9812,7 @@
         <v>596</v>
       </c>
       <c r="C303" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D303" t="s">
         <v>597</v>
@@ -9865,7 +9835,7 @@
         <v>599</v>
       </c>
       <c r="C304" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D304" t="s">
         <v>600</v>
@@ -9980,7 +9950,7 @@
         <v>610</v>
       </c>
       <c r="C309" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D309" t="s">
         <v>450</v>
@@ -10003,7 +9973,7 @@
         <v>611</v>
       </c>
       <c r="C310" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D310" t="s">
         <v>93</v>
@@ -10026,7 +9996,7 @@
         <v>612</v>
       </c>
       <c r="C311" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D311" t="s">
         <v>93</v>
@@ -10095,7 +10065,7 @@
         <v>619</v>
       </c>
       <c r="C314" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D314" t="s">
         <v>620</v>
@@ -10118,7 +10088,7 @@
         <v>622</v>
       </c>
       <c r="C315" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D315" t="s">
         <v>430</v>
@@ -10187,7 +10157,7 @@
         <v>625</v>
       </c>
       <c r="C318" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D318" t="s">
         <v>101</v>
@@ -10417,7 +10387,7 @@
         <v>643</v>
       </c>
       <c r="C328" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D328" t="s">
         <v>450</v>
@@ -10440,7 +10410,7 @@
         <v>644</v>
       </c>
       <c r="C329" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D329" t="s">
         <v>450</v>
@@ -10486,7 +10456,7 @@
         <v>646</v>
       </c>
       <c r="C331" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D331" t="s">
         <v>450</v>
@@ -10578,7 +10548,7 @@
         <v>654</v>
       </c>
       <c r="C335" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D335" t="s">
         <v>200</v>
@@ -10808,7 +10778,7 @@
         <v>672</v>
       </c>
       <c r="C345" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D345" t="s">
         <v>673</v>
@@ -11383,7 +11353,7 @@
         <v>703</v>
       </c>
       <c r="C370" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D370" t="s">
         <v>470</v>
@@ -11981,19 +11951,19 @@
         <v>745</v>
       </c>
       <c r="C396" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D396" t="s">
-        <v>450</v>
+        <v>127</v>
       </c>
       <c r="E396" t="s">
-        <v>451</v>
+        <v>128</v>
       </c>
       <c r="F396" s="1">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="G396" s="1">
-        <v>46258</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.2">
@@ -12004,19 +11974,19 @@
         <v>746</v>
       </c>
       <c r="C397" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D397" t="s">
-        <v>127</v>
+        <v>433</v>
       </c>
       <c r="E397" t="s">
-        <v>128</v>
+        <v>434</v>
       </c>
       <c r="F397" s="1">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="G397" s="1">
-        <v>46259</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.2">
@@ -12030,96 +12000,96 @@
         <v>80</v>
       </c>
       <c r="D398" t="s">
-        <v>748</v>
+        <v>726</v>
       </c>
       <c r="E398" t="s">
-        <v>749</v>
+        <v>727</v>
       </c>
       <c r="F398" s="1">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="G398" s="1">
-        <v>46261</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A399" t="s">
-        <v>715</v>
+        <v>748</v>
       </c>
       <c r="B399" t="s">
+        <v>749</v>
+      </c>
+      <c r="C399" t="s">
+        <v>96</v>
+      </c>
+      <c r="D399" t="s">
         <v>750</v>
       </c>
-      <c r="C399" t="s">
-        <v>80</v>
-      </c>
-      <c r="D399" t="s">
-        <v>433</v>
-      </c>
       <c r="E399" t="s">
-        <v>434</v>
+        <v>751</v>
       </c>
       <c r="F399" s="1">
-        <v>46262</v>
+        <v>46063</v>
       </c>
       <c r="G399" s="1">
-        <v>46262</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>715</v>
+        <v>748</v>
       </c>
       <c r="B400" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C400" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D400" t="s">
-        <v>726</v>
+        <v>57</v>
       </c>
       <c r="E400" t="s">
-        <v>727</v>
+        <v>58</v>
       </c>
       <c r="F400" s="1">
-        <v>46262</v>
+        <v>46113</v>
       </c>
       <c r="G400" s="1">
-        <v>46262</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B401" t="s">
         <v>753</v>
       </c>
       <c r="C401" t="s">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D401" t="s">
-        <v>754</v>
+        <v>57</v>
       </c>
       <c r="E401" t="s">
-        <v>755</v>
+        <v>58</v>
       </c>
       <c r="F401" s="1">
-        <v>46063</v>
+        <v>46125</v>
       </c>
       <c r="G401" s="1">
-        <v>46064</v>
+        <v>46125</v>
       </c>
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A402" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B402" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="C402" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D402" t="s">
         <v>57</v>
@@ -12128,18 +12098,18 @@
         <v>58</v>
       </c>
       <c r="F402" s="1">
-        <v>46113</v>
+        <v>46126</v>
       </c>
       <c r="G402" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A403" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B403" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="C403" t="s">
         <v>2</v>
@@ -12151,18 +12121,18 @@
         <v>58</v>
       </c>
       <c r="F403" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="G403" s="1">
-        <v>46125</v>
+        <v>46126</v>
       </c>
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A404" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B404" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="C404" t="s">
         <v>2</v>
@@ -12174,21 +12144,21 @@
         <v>58</v>
       </c>
       <c r="F404" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
       <c r="G404" s="1">
-        <v>46126</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B405" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C405" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D405" t="s">
         <v>57</v>
@@ -12197,18 +12167,18 @@
         <v>58</v>
       </c>
       <c r="F405" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
       <c r="G405" s="1">
-        <v>46126</v>
+        <v>46132</v>
       </c>
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B406" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="C406" t="s">
         <v>2</v>
@@ -12220,21 +12190,21 @@
         <v>58</v>
       </c>
       <c r="F406" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
       <c r="G406" s="1">
-        <v>46128</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B407" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C407" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D407" t="s">
         <v>57</v>
@@ -12243,18 +12213,18 @@
         <v>58</v>
       </c>
       <c r="F407" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
       <c r="G407" s="1">
-        <v>46132</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B408" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="C408" t="s">
         <v>2</v>
@@ -12266,21 +12236,21 @@
         <v>58</v>
       </c>
       <c r="F408" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
       <c r="G408" s="1">
-        <v>46161</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="409" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A409" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B409" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="C409" t="s">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D409" t="s">
         <v>57</v>
@@ -12289,21 +12259,21 @@
         <v>58</v>
       </c>
       <c r="F409" s="1">
-        <v>46174</v>
+        <v>46195</v>
       </c>
       <c r="G409" s="1">
-        <v>46174</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B410" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="C410" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D410" t="s">
         <v>57</v>
@@ -12312,21 +12282,21 @@
         <v>58</v>
       </c>
       <c r="F410" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
       <c r="G410" s="1">
-        <v>46174</v>
+        <v>46210</v>
       </c>
     </row>
     <row r="411" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A411" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B411" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="C411" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D411" t="s">
         <v>57</v>
@@ -12335,21 +12305,21 @@
         <v>58</v>
       </c>
       <c r="F411" s="1">
-        <v>46195</v>
+        <v>46213</v>
       </c>
       <c r="G411" s="1">
-        <v>46252</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="412" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B412" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="C412" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D412" t="s">
         <v>57</v>
@@ -12358,41 +12328,41 @@
         <v>58</v>
       </c>
       <c r="F412" s="1">
-        <v>46210</v>
+        <v>46218</v>
       </c>
       <c r="G412" s="1">
-        <v>46210</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="413" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B413" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="C413" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D413" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E413" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F413" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
       <c r="G413" s="1">
-        <v>46213</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="414" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B414" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="C414" t="s">
         <v>80</v>
@@ -12404,7 +12374,7 @@
         <v>58</v>
       </c>
       <c r="F414" s="1">
-        <v>46218</v>
+        <v>46227</v>
       </c>
       <c r="G414" s="1">
         <v>46252</v>
@@ -12412,36 +12382,36 @@
     </row>
     <row r="415" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B415" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="C415" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="D415" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E415" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F415" s="1">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="G415" s="1">
-        <v>46226</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="416" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B416" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C416" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D416" t="s">
         <v>57</v>
@@ -12453,27 +12423,27 @@
         <v>46227</v>
       </c>
       <c r="G416" s="1">
-        <v>46252</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A417" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B417" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C417" t="s">
         <v>80</v>
       </c>
       <c r="D417" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E417" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="F417" s="1">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="G417" s="1">
         <v>46252</v>
@@ -12481,10 +12451,10 @@
     </row>
     <row r="418" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A418" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B418" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="C418" t="s">
         <v>6</v>
@@ -12496,44 +12466,44 @@
         <v>58</v>
       </c>
       <c r="F418" s="1">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="G418" s="1">
-        <v>46228</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="419" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A419" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B419" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="C419" t="s">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="D419" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E419" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F419" s="1">
-        <v>46230</v>
+        <v>46254</v>
       </c>
       <c r="G419" s="1">
-        <v>46252</v>
+        <v>46254</v>
       </c>
     </row>
     <row r="420" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A420" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B420" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="C420" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D420" t="s">
         <v>57</v>
@@ -12542,18 +12512,18 @@
         <v>58</v>
       </c>
       <c r="F420" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
       <c r="G420" s="1">
-        <v>46231</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="421" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A421" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B421" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C421" t="s">
         <v>6</v>
@@ -12565,400 +12535,216 @@
         <v>58</v>
       </c>
       <c r="F421" s="1">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="G421" s="1">
-        <v>46254</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="422" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A422" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B422" t="s">
+        <v>775</v>
+      </c>
+      <c r="C422" t="s">
+        <v>2</v>
+      </c>
+      <c r="D422" t="s">
         <v>776</v>
       </c>
-      <c r="C422" t="s">
-        <v>2</v>
-      </c>
-      <c r="D422" t="s">
-        <v>57</v>
-      </c>
       <c r="E422" t="s">
-        <v>58</v>
+        <v>777</v>
       </c>
       <c r="F422" s="1">
-        <v>46255</v>
+        <v>46083</v>
       </c>
       <c r="G422" s="1">
-        <v>46255</v>
+        <v>46084</v>
       </c>
     </row>
     <row r="423" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A423" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B423" t="s">
+        <v>778</v>
+      </c>
+      <c r="C423" t="s">
+        <v>2</v>
+      </c>
+      <c r="D423" t="s">
+        <v>776</v>
+      </c>
+      <c r="E423" t="s">
         <v>777</v>
       </c>
-      <c r="C423" t="s">
-        <v>6</v>
-      </c>
-      <c r="D423" t="s">
-        <v>57</v>
-      </c>
-      <c r="E423" t="s">
-        <v>58</v>
-      </c>
       <c r="F423" s="1">
-        <v>46260</v>
+        <v>46132</v>
       </c>
       <c r="G423" s="1">
-        <v>46260</v>
+        <v>46133</v>
       </c>
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A424" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B424" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="C424" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D424" t="s">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="E424" t="s">
-        <v>58</v>
+        <v>706</v>
       </c>
       <c r="F424" s="1">
-        <v>46262</v>
+        <v>46157</v>
       </c>
       <c r="G424" s="1">
-        <v>46262</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="425" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A425" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B425" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="C425" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D425" t="s">
-        <v>57</v>
+        <v>781</v>
       </c>
       <c r="E425" t="s">
-        <v>58</v>
+        <v>782</v>
       </c>
       <c r="F425" s="1">
-        <v>46262</v>
+        <v>46168</v>
       </c>
       <c r="G425" s="1">
-        <v>46262</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="426" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A426" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B426" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="C426" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D426" t="s">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="E426" t="s">
-        <v>58</v>
+        <v>706</v>
       </c>
       <c r="F426" s="1">
-        <v>46262</v>
+        <v>46244</v>
       </c>
       <c r="G426" s="1">
-        <v>46262</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="427" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A427" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B427" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="C427" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D427" t="s">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="E427" t="s">
-        <v>58</v>
+        <v>706</v>
       </c>
       <c r="F427" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
       <c r="G427" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="428" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A428" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B428" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="C428" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D428" t="s">
-        <v>57</v>
+        <v>776</v>
       </c>
       <c r="E428" t="s">
-        <v>58</v>
+        <v>777</v>
       </c>
       <c r="F428" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
       <c r="G428" s="1">
-        <v>46262</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A429" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="B429" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="C429" t="s">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="D429" t="s">
-        <v>57</v>
+        <v>705</v>
       </c>
       <c r="E429" t="s">
-        <v>58</v>
+        <v>706</v>
       </c>
       <c r="F429" s="1">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="G429" s="1">
-        <v>46262</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A430" t="s">
-        <v>784</v>
+        <v>774</v>
       </c>
       <c r="B430" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="C430" t="s">
         <v>2</v>
       </c>
       <c r="D430" t="s">
-        <v>786</v>
+        <v>705</v>
       </c>
       <c r="E430" t="s">
-        <v>787</v>
+        <v>706</v>
       </c>
       <c r="F430" s="1">
-        <v>46083</v>
+        <v>46258</v>
       </c>
       <c r="G430" s="1">
-        <v>46084</v>
-      </c>
-    </row>
-    <row r="431" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A431" t="s">
-        <v>784</v>
-      </c>
-      <c r="B431" t="s">
-        <v>788</v>
-      </c>
-      <c r="C431" t="s">
-        <v>2</v>
-      </c>
-      <c r="D431" t="s">
-        <v>786</v>
-      </c>
-      <c r="E431" t="s">
-        <v>787</v>
-      </c>
-      <c r="F431" s="1">
-        <v>46132</v>
-      </c>
-      <c r="G431" s="1">
-        <v>46133</v>
-      </c>
-    </row>
-    <row r="432" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A432" t="s">
-        <v>784</v>
-      </c>
-      <c r="B432" t="s">
-        <v>789</v>
-      </c>
-      <c r="C432" t="s">
-        <v>2</v>
-      </c>
-      <c r="D432" t="s">
-        <v>705</v>
-      </c>
-      <c r="E432" t="s">
-        <v>706</v>
-      </c>
-      <c r="F432" s="1">
-        <v>46157</v>
-      </c>
-      <c r="G432" s="1">
-        <v>46157</v>
-      </c>
-    </row>
-    <row r="433" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A433" t="s">
-        <v>784</v>
-      </c>
-      <c r="B433" t="s">
-        <v>790</v>
-      </c>
-      <c r="C433" t="s">
-        <v>2</v>
-      </c>
-      <c r="D433" t="s">
-        <v>791</v>
-      </c>
-      <c r="E433" t="s">
-        <v>792</v>
-      </c>
-      <c r="F433" s="1">
-        <v>46168</v>
-      </c>
-      <c r="G433" s="1">
-        <v>46170</v>
-      </c>
-    </row>
-    <row r="434" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A434" t="s">
-        <v>784</v>
-      </c>
-      <c r="B434" t="s">
-        <v>793</v>
-      </c>
-      <c r="C434" t="s">
-        <v>2</v>
-      </c>
-      <c r="D434" t="s">
-        <v>705</v>
-      </c>
-      <c r="E434" t="s">
-        <v>706</v>
-      </c>
-      <c r="F434" s="1">
-        <v>46244</v>
-      </c>
-      <c r="G434" s="1">
-        <v>46244</v>
-      </c>
-    </row>
-    <row r="435" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A435" t="s">
-        <v>784</v>
-      </c>
-      <c r="B435" t="s">
-        <v>794</v>
-      </c>
-      <c r="C435" t="s">
-        <v>2</v>
-      </c>
-      <c r="D435" t="s">
-        <v>705</v>
-      </c>
-      <c r="E435" t="s">
-        <v>706</v>
-      </c>
-      <c r="F435" s="1">
-        <v>46247</v>
-      </c>
-      <c r="G435" s="1">
-        <v>46247</v>
-      </c>
-    </row>
-    <row r="436" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A436" t="s">
-        <v>784</v>
-      </c>
-      <c r="B436" t="s">
-        <v>795</v>
-      </c>
-      <c r="C436" t="s">
-        <v>2</v>
-      </c>
-      <c r="D436" t="s">
-        <v>786</v>
-      </c>
-      <c r="E436" t="s">
-        <v>787</v>
-      </c>
-      <c r="F436" s="1">
-        <v>46247</v>
-      </c>
-      <c r="G436" s="1">
-        <v>46247</v>
-      </c>
-    </row>
-    <row r="437" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A437" t="s">
-        <v>784</v>
-      </c>
-      <c r="B437" t="s">
-        <v>796</v>
-      </c>
-      <c r="C437" t="s">
-        <v>2</v>
-      </c>
-      <c r="D437" t="s">
-        <v>705</v>
-      </c>
-      <c r="E437" t="s">
-        <v>706</v>
-      </c>
-      <c r="F437" s="1">
-        <v>46255</v>
-      </c>
-      <c r="G437" s="1">
-        <v>46255</v>
-      </c>
-    </row>
-    <row r="438" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A438" t="s">
-        <v>784</v>
-      </c>
-      <c r="B438" t="s">
-        <v>797</v>
-      </c>
-      <c r="C438" t="s">
-        <v>2</v>
-      </c>
-      <c r="D438" t="s">
-        <v>705</v>
-      </c>
-      <c r="E438" t="s">
-        <v>706</v>
-      </c>
-      <c r="F438" s="1">
-        <v>46258</v>
-      </c>
-      <c r="G438" s="1">
         <v>46258</v>
       </c>
     </row>

</xml_diff>